<commit_message>
Changes to memory map layout
</commit_message>
<xml_diff>
--- a/wh40k_NTAG215_memoryMapping.xlsx
+++ b/wh40k_NTAG215_memoryMapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fuzzy\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fuzzy\wh40k_nfc_project\wh40k_nfc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF9B248-7B90-4B14-BD62-CFD15ACBEAEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23062AE8-122C-4DEC-BC0B-3DF28DBF9347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -537,28 +537,13 @@
   <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -568,167 +553,179 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -741,7 +738,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -755,6 +752,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -765,30 +789,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1199,112 +1199,112 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="83"/>
+      <c r="D2" s="84" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6"/>
-      <c r="I2" s="11" t="s">
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="86"/>
+      <c r="I2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="6">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="7">
         <v>0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="7">
         <v>1</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="7">
         <v>2</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="7">
         <v>3</v>
       </c>
-      <c r="I3" s="29" t="s">
+      <c r="I3" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="29">
+      <c r="J3" s="11">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B4" s="7">
+      <c r="B4" s="3">
         <v>0</v>
       </c>
-      <c r="C4" s="14" t="str">
+      <c r="C4" s="8" t="str">
         <f>DEC2HEX(B4)&amp;"h"</f>
         <v>0h</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="I4" s="84" t="s">
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="87"/>
+      <c r="I4" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="84">
+      <c r="J4" s="18">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B5" s="8">
+      <c r="B5" s="4">
         <v>1</v>
       </c>
-      <c r="C5" s="8" t="str">
+      <c r="C5" s="4" t="str">
         <f t="shared" ref="C5:C68" si="0">DEC2HEX(B5)&amp;"h"</f>
         <v>1h</v>
       </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="I5" s="30" t="s">
+      <c r="D5" s="88"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+      <c r="G5" s="87"/>
+      <c r="I5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="30">
-        <v>50</v>
+      <c r="J5" s="12">
+        <v>52</v>
       </c>
       <c r="K5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B6" s="8">
+      <c r="B6" s="4">
         <v>2</v>
       </c>
-      <c r="C6" s="8" t="str">
+      <c r="C6" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2h</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="17" t="s">
+      <c r="D6" s="9"/>
+      <c r="E6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="89" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="19"/>
-      <c r="I6" s="31" t="s">
+      <c r="G6" s="90"/>
+      <c r="I6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="J6" s="31">
+      <c r="J6" s="13">
         <v>20</v>
       </c>
       <c r="K6" t="s">
@@ -1312,23 +1312,23 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B7" s="8">
+      <c r="B7" s="4">
         <v>3</v>
       </c>
-      <c r="C7" s="8" t="str">
+      <c r="C7" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3h</v>
       </c>
-      <c r="D7" s="81" t="s">
+      <c r="D7" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="82"/>
-      <c r="F7" s="82"/>
-      <c r="G7" s="83"/>
-      <c r="I7" s="31" t="s">
+      <c r="E7" s="92"/>
+      <c r="F7" s="92"/>
+      <c r="G7" s="93"/>
+      <c r="I7" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="31">
+      <c r="J7" s="13">
         <v>20</v>
       </c>
       <c r="K7" t="s">
@@ -1336,23 +1336,23 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B8" s="8">
+      <c r="B8" s="4">
         <v>4</v>
       </c>
-      <c r="C8" s="8" t="str">
+      <c r="C8" s="4" t="str">
         <f t="shared" si="0"/>
         <v>4h</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="22"/>
-      <c r="I8" s="41" t="s">
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="30"/>
+      <c r="I8" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="J8" s="41">
+      <c r="J8" s="14">
         <v>20</v>
       </c>
       <c r="K8" t="s">
@@ -1360,21 +1360,21 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B9" s="8">
+      <c r="B9" s="4">
         <v>5</v>
       </c>
-      <c r="C9" s="8" t="str">
+      <c r="C9" s="4" t="str">
         <f t="shared" si="0"/>
         <v>5h</v>
       </c>
-      <c r="D9" s="23"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="25"/>
-      <c r="I9" s="42" t="s">
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="33"/>
+      <c r="I9" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="42">
+      <c r="J9" s="15">
         <v>20</v>
       </c>
       <c r="K9" t="s">
@@ -1382,984 +1382,984 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B10" s="8">
+      <c r="B10" s="4">
         <v>6</v>
       </c>
-      <c r="C10" s="8" t="str">
+      <c r="C10" s="4" t="str">
         <f t="shared" si="0"/>
         <v>6h</v>
       </c>
-      <c r="D10" s="23"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="25"/>
-      <c r="I10" s="71" t="s">
+      <c r="D10" s="31"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="33"/>
+      <c r="I10" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="J10" s="71">
+      <c r="J10" s="17">
         <v>200</v>
       </c>
-      <c r="K10" s="70" t="s">
+      <c r="K10" s="16" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B11" s="8">
+      <c r="B11" s="4">
         <v>7</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="4" t="str">
         <f t="shared" si="0"/>
         <v>7h</v>
       </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="25"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="33"/>
       <c r="K11" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B12" s="8">
+      <c r="B12" s="4">
         <v>8</v>
       </c>
-      <c r="C12" s="8" t="str">
+      <c r="C12" s="4" t="str">
         <f t="shared" si="0"/>
         <v>8h</v>
       </c>
-      <c r="D12" s="23"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="25"/>
+      <c r="D12" s="31"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="33"/>
       <c r="K12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B13" s="8">
+      <c r="B13" s="4">
         <v>9</v>
       </c>
-      <c r="C13" s="8" t="str">
+      <c r="C13" s="4" t="str">
         <f t="shared" si="0"/>
         <v>9h</v>
       </c>
-      <c r="D13" s="23"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="25"/>
-      <c r="I13" s="85" t="s">
+      <c r="D13" s="31"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="33"/>
+      <c r="I13" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="J13" s="85">
+      <c r="J13" s="19">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B14" s="8">
+      <c r="B14" s="4">
         <v>10</v>
       </c>
-      <c r="C14" s="8" t="str">
+      <c r="C14" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Ah</v>
       </c>
-      <c r="D14" s="23"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="25"/>
-      <c r="I14" s="93" t="s">
+      <c r="D14" s="31"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="33"/>
+      <c r="I14" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="J14" s="93">
+      <c r="J14" s="21">
         <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B15" s="8">
+      <c r="B15" s="4">
         <v>11</v>
       </c>
-      <c r="C15" s="8" t="str">
+      <c r="C15" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Bh</v>
       </c>
-      <c r="D15" s="23"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="25"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="33"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B16" s="8">
+      <c r="B16" s="4">
         <v>12</v>
       </c>
-      <c r="C16" s="8" t="str">
+      <c r="C16" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Ch</v>
       </c>
-      <c r="D16" s="23"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="25"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="33"/>
       <c r="I16" t="s">
         <v>38</v>
       </c>
       <c r="J16">
         <f>SUM(J2:J14)</f>
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B17" s="8">
+      <c r="B17" s="4">
         <v>13</v>
       </c>
-      <c r="C17" s="8" t="str">
+      <c r="C17" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Dh</v>
       </c>
-      <c r="D17" s="23"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="25"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="33"/>
       <c r="I17" t="s">
         <v>39</v>
       </c>
       <c r="J17">
         <f>540-J16</f>
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B18" s="8">
+      <c r="B18" s="4">
         <v>14</v>
       </c>
-      <c r="C18" s="8" t="str">
+      <c r="C18" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Eh</v>
       </c>
-      <c r="D18" s="23"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="25"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B19" s="8">
+      <c r="B19" s="4">
         <v>15</v>
       </c>
-      <c r="C19" s="8" t="str">
+      <c r="C19" s="4" t="str">
         <f t="shared" si="0"/>
         <v>Fh</v>
       </c>
-      <c r="D19" s="23"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="25"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="33"/>
     </row>
     <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" s="8">
+      <c r="B20" s="4">
         <v>16</v>
       </c>
-      <c r="C20" s="8" t="str">
+      <c r="C20" s="4" t="str">
         <f t="shared" si="0"/>
         <v>10h</v>
       </c>
-      <c r="D20" s="26"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="28"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="36"/>
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B21" s="8">
+      <c r="B21" s="4">
         <v>17</v>
       </c>
-      <c r="C21" s="8" t="str">
+      <c r="C21" s="4" t="str">
         <f t="shared" si="0"/>
         <v>11h</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="34"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
+      <c r="G21" s="48"/>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B22" s="8">
+      <c r="B22" s="4">
         <v>18</v>
       </c>
-      <c r="C22" s="8" t="str">
+      <c r="C22" s="4" t="str">
         <f t="shared" si="0"/>
         <v>12h</v>
       </c>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="37"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
+      <c r="G22" s="51"/>
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B23" s="8">
+      <c r="B23" s="4">
         <v>19</v>
       </c>
-      <c r="C23" s="8" t="str">
+      <c r="C23" s="4" t="str">
         <f t="shared" si="0"/>
         <v>13h</v>
       </c>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="37"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="50"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="51"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B24" s="8">
+      <c r="B24" s="4">
         <v>20</v>
       </c>
-      <c r="C24" s="8" t="str">
+      <c r="C24" s="4" t="str">
         <f t="shared" si="0"/>
         <v>14h</v>
       </c>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="37"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="51"/>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B25" s="8">
+      <c r="B25" s="4">
         <v>21</v>
       </c>
-      <c r="C25" s="8" t="str">
+      <c r="C25" s="4" t="str">
         <f t="shared" si="0"/>
         <v>15h</v>
       </c>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="40"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53"/>
+      <c r="G25" s="54"/>
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B26" s="8">
+      <c r="B26" s="4">
         <v>22</v>
       </c>
-      <c r="C26" s="8" t="str">
+      <c r="C26" s="4" t="str">
         <f t="shared" si="0"/>
         <v>16h</v>
       </c>
-      <c r="D26" s="62" t="s">
+      <c r="D26" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="63"/>
-      <c r="F26" s="63"/>
-      <c r="G26" s="64"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="56"/>
+      <c r="G26" s="57"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B27" s="8">
+      <c r="B27" s="4">
         <v>23</v>
       </c>
-      <c r="C27" s="8" t="str">
+      <c r="C27" s="4" t="str">
         <f t="shared" si="0"/>
         <v>17h</v>
       </c>
-      <c r="D27" s="65"/>
-      <c r="E27" s="66"/>
-      <c r="F27" s="66"/>
-      <c r="G27" s="67"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="59"/>
+      <c r="F27" s="59"/>
+      <c r="G27" s="60"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B28" s="8">
+      <c r="B28" s="4">
         <v>24</v>
       </c>
-      <c r="C28" s="8" t="str">
+      <c r="C28" s="4" t="str">
         <f t="shared" si="0"/>
         <v>18h</v>
       </c>
-      <c r="D28" s="65"/>
-      <c r="E28" s="66"/>
-      <c r="F28" s="66"/>
-      <c r="G28" s="67"/>
+      <c r="D28" s="58"/>
+      <c r="E28" s="59"/>
+      <c r="F28" s="59"/>
+      <c r="G28" s="60"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B29" s="8">
+      <c r="B29" s="4">
         <v>25</v>
       </c>
-      <c r="C29" s="8" t="str">
+      <c r="C29" s="4" t="str">
         <f t="shared" si="0"/>
         <v>19h</v>
       </c>
-      <c r="D29" s="65"/>
-      <c r="E29" s="66"/>
-      <c r="F29" s="66"/>
-      <c r="G29" s="67"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="59"/>
+      <c r="G29" s="60"/>
     </row>
     <row r="30" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B30" s="8">
+      <c r="B30" s="4">
         <v>26</v>
       </c>
-      <c r="C30" s="8" t="str">
+      <c r="C30" s="4" t="str">
         <f t="shared" si="0"/>
         <v>1Ah</v>
       </c>
-      <c r="D30" s="68"/>
-      <c r="E30" s="69"/>
-      <c r="F30" s="69"/>
-      <c r="G30" s="61"/>
+      <c r="D30" s="61"/>
+      <c r="E30" s="62"/>
+      <c r="F30" s="62"/>
+      <c r="G30" s="63"/>
     </row>
     <row r="31" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B31" s="8">
+      <c r="B31" s="4">
         <v>27</v>
       </c>
-      <c r="C31" s="8" t="str">
+      <c r="C31" s="4" t="str">
         <f t="shared" si="0"/>
         <v>1Bh</v>
       </c>
-      <c r="D31" s="43" t="s">
+      <c r="D31" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="E31" s="44"/>
-      <c r="F31" s="44"/>
-      <c r="G31" s="45"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="39"/>
     </row>
     <row r="32" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B32" s="8">
+      <c r="B32" s="4">
         <v>28</v>
       </c>
-      <c r="C32" s="8" t="str">
+      <c r="C32" s="4" t="str">
         <f t="shared" si="0"/>
         <v>1Ch</v>
       </c>
-      <c r="D32" s="46"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="48"/>
+      <c r="D32" s="40"/>
+      <c r="E32" s="41"/>
+      <c r="F32" s="41"/>
+      <c r="G32" s="42"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B33" s="8">
+      <c r="B33" s="4">
         <v>29</v>
       </c>
-      <c r="C33" s="8" t="str">
+      <c r="C33" s="4" t="str">
         <f t="shared" si="0"/>
         <v>1Dh</v>
       </c>
-      <c r="D33" s="46"/>
-      <c r="E33" s="47"/>
-      <c r="F33" s="47"/>
-      <c r="G33" s="48"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B34" s="8">
+      <c r="B34" s="4">
         <v>30</v>
       </c>
-      <c r="C34" s="8" t="str">
+      <c r="C34" s="4" t="str">
         <f t="shared" si="0"/>
         <v>1Eh</v>
       </c>
-      <c r="D34" s="46"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="48"/>
+      <c r="D34" s="40"/>
+      <c r="E34" s="41"/>
+      <c r="F34" s="41"/>
+      <c r="G34" s="42"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B35" s="8">
+      <c r="B35" s="4">
         <v>31</v>
       </c>
-      <c r="C35" s="8" t="str">
+      <c r="C35" s="4" t="str">
         <f t="shared" si="0"/>
         <v>1Fh</v>
       </c>
-      <c r="D35" s="49"/>
-      <c r="E35" s="50"/>
-      <c r="F35" s="50"/>
-      <c r="G35" s="51"/>
+      <c r="D35" s="43"/>
+      <c r="E35" s="44"/>
+      <c r="F35" s="44"/>
+      <c r="G35" s="45"/>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B36" s="8">
+      <c r="B36" s="4">
         <v>32</v>
       </c>
-      <c r="C36" s="8" t="str">
+      <c r="C36" s="4" t="str">
         <f t="shared" si="0"/>
         <v>20h</v>
       </c>
-      <c r="D36" s="52" t="s">
+      <c r="D36" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="E36" s="53"/>
-      <c r="F36" s="53"/>
-      <c r="G36" s="54"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="66"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B37" s="8">
+      <c r="B37" s="4">
         <v>33</v>
       </c>
-      <c r="C37" s="8" t="str">
+      <c r="C37" s="4" t="str">
         <f t="shared" si="0"/>
         <v>21h</v>
       </c>
-      <c r="D37" s="55"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="57"/>
+      <c r="D37" s="67"/>
+      <c r="E37" s="68"/>
+      <c r="F37" s="68"/>
+      <c r="G37" s="69"/>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B38" s="8">
+      <c r="B38" s="4">
         <v>34</v>
       </c>
-      <c r="C38" s="8" t="str">
+      <c r="C38" s="4" t="str">
         <f t="shared" si="0"/>
         <v>22h</v>
       </c>
-      <c r="D38" s="55"/>
-      <c r="E38" s="56"/>
-      <c r="F38" s="56"/>
-      <c r="G38" s="57"/>
+      <c r="D38" s="67"/>
+      <c r="E38" s="68"/>
+      <c r="F38" s="68"/>
+      <c r="G38" s="69"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B39" s="8">
+      <c r="B39" s="4">
         <v>35</v>
       </c>
-      <c r="C39" s="8" t="str">
+      <c r="C39" s="4" t="str">
         <f t="shared" si="0"/>
         <v>23h</v>
       </c>
-      <c r="D39" s="55"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
+      <c r="D39" s="67"/>
+      <c r="E39" s="68"/>
+      <c r="F39" s="68"/>
+      <c r="G39" s="69"/>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B40" s="8">
+      <c r="B40" s="4">
         <v>36</v>
       </c>
-      <c r="C40" s="8" t="str">
+      <c r="C40" s="4" t="str">
         <f t="shared" si="0"/>
         <v>24h</v>
       </c>
-      <c r="D40" s="58"/>
-      <c r="E40" s="59"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="60"/>
+      <c r="D40" s="70"/>
+      <c r="E40" s="71"/>
+      <c r="F40" s="71"/>
+      <c r="G40" s="72"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B41" s="8">
+      <c r="B41" s="4">
         <v>37</v>
       </c>
-      <c r="C41" s="8" t="str">
+      <c r="C41" s="4" t="str">
         <f t="shared" si="0"/>
         <v>25h</v>
       </c>
-      <c r="D41" s="72" t="s">
+      <c r="D41" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="E41" s="73"/>
-      <c r="F41" s="73"/>
-      <c r="G41" s="74"/>
+      <c r="E41" s="74"/>
+      <c r="F41" s="74"/>
+      <c r="G41" s="75"/>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B42" s="8">
+      <c r="B42" s="4">
         <v>38</v>
       </c>
-      <c r="C42" s="8" t="str">
+      <c r="C42" s="4" t="str">
         <f t="shared" si="0"/>
         <v>26h</v>
       </c>
-      <c r="D42" s="75"/>
-      <c r="E42" s="76"/>
-      <c r="F42" s="76"/>
-      <c r="G42" s="77"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="77"/>
+      <c r="F42" s="77"/>
+      <c r="G42" s="78"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B43" s="8">
+      <c r="B43" s="4">
         <v>39</v>
       </c>
-      <c r="C43" s="8" t="str">
+      <c r="C43" s="4" t="str">
         <f t="shared" si="0"/>
         <v>27h</v>
       </c>
-      <c r="D43" s="75"/>
-      <c r="E43" s="76"/>
-      <c r="F43" s="76"/>
-      <c r="G43" s="77"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="77"/>
+      <c r="F43" s="77"/>
+      <c r="G43" s="78"/>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B44" s="8">
+      <c r="B44" s="4">
         <v>40</v>
       </c>
-      <c r="C44" s="8" t="str">
+      <c r="C44" s="4" t="str">
         <f t="shared" si="0"/>
         <v>28h</v>
       </c>
-      <c r="D44" s="75"/>
-      <c r="E44" s="76"/>
-      <c r="F44" s="76"/>
-      <c r="G44" s="77"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="77"/>
+      <c r="F44" s="77"/>
+      <c r="G44" s="78"/>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B45" s="8">
+      <c r="B45" s="4">
         <v>41</v>
       </c>
-      <c r="C45" s="8" t="str">
+      <c r="C45" s="4" t="str">
         <f t="shared" si="0"/>
         <v>29h</v>
       </c>
-      <c r="D45" s="75"/>
-      <c r="E45" s="76"/>
-      <c r="F45" s="76"/>
-      <c r="G45" s="77"/>
+      <c r="D45" s="76"/>
+      <c r="E45" s="77"/>
+      <c r="F45" s="77"/>
+      <c r="G45" s="78"/>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B46" s="8">
+      <c r="B46" s="4">
         <v>42</v>
       </c>
-      <c r="C46" s="8" t="str">
+      <c r="C46" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2Ah</v>
       </c>
-      <c r="D46" s="75"/>
-      <c r="E46" s="76"/>
-      <c r="F46" s="76"/>
-      <c r="G46" s="77"/>
+      <c r="D46" s="76"/>
+      <c r="E46" s="77"/>
+      <c r="F46" s="77"/>
+      <c r="G46" s="78"/>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B47" s="8">
+      <c r="B47" s="4">
         <v>43</v>
       </c>
-      <c r="C47" s="8" t="str">
+      <c r="C47" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2Bh</v>
       </c>
-      <c r="D47" s="75"/>
-      <c r="E47" s="76"/>
-      <c r="F47" s="76"/>
-      <c r="G47" s="77"/>
+      <c r="D47" s="76"/>
+      <c r="E47" s="77"/>
+      <c r="F47" s="77"/>
+      <c r="G47" s="78"/>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B48" s="8">
+      <c r="B48" s="4">
         <v>44</v>
       </c>
-      <c r="C48" s="8" t="str">
+      <c r="C48" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2Ch</v>
       </c>
-      <c r="D48" s="75"/>
-      <c r="E48" s="76"/>
-      <c r="F48" s="76"/>
-      <c r="G48" s="77"/>
+      <c r="D48" s="76"/>
+      <c r="E48" s="77"/>
+      <c r="F48" s="77"/>
+      <c r="G48" s="78"/>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B49" s="8">
+      <c r="B49" s="4">
         <v>45</v>
       </c>
-      <c r="C49" s="8" t="str">
+      <c r="C49" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2Dh</v>
       </c>
-      <c r="D49" s="75"/>
-      <c r="E49" s="76"/>
-      <c r="F49" s="76"/>
-      <c r="G49" s="77"/>
+      <c r="D49" s="76"/>
+      <c r="E49" s="77"/>
+      <c r="F49" s="77"/>
+      <c r="G49" s="78"/>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B50" s="8">
+      <c r="B50" s="4">
         <v>46</v>
       </c>
-      <c r="C50" s="8" t="str">
+      <c r="C50" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2Eh</v>
       </c>
-      <c r="D50" s="75"/>
-      <c r="E50" s="76"/>
-      <c r="F50" s="76"/>
-      <c r="G50" s="77"/>
+      <c r="D50" s="76"/>
+      <c r="E50" s="77"/>
+      <c r="F50" s="77"/>
+      <c r="G50" s="78"/>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B51" s="8">
+      <c r="B51" s="4">
         <v>47</v>
       </c>
-      <c r="C51" s="8" t="str">
+      <c r="C51" s="4" t="str">
         <f t="shared" si="0"/>
         <v>2Fh</v>
       </c>
-      <c r="D51" s="75"/>
-      <c r="E51" s="76"/>
-      <c r="F51" s="76"/>
-      <c r="G51" s="77"/>
+      <c r="D51" s="76"/>
+      <c r="E51" s="77"/>
+      <c r="F51" s="77"/>
+      <c r="G51" s="78"/>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B52" s="8">
+      <c r="B52" s="4">
         <v>48</v>
       </c>
-      <c r="C52" s="8" t="str">
+      <c r="C52" s="4" t="str">
         <f t="shared" si="0"/>
         <v>30h</v>
       </c>
-      <c r="D52" s="75"/>
-      <c r="E52" s="76"/>
-      <c r="F52" s="76"/>
-      <c r="G52" s="77"/>
+      <c r="D52" s="76"/>
+      <c r="E52" s="77"/>
+      <c r="F52" s="77"/>
+      <c r="G52" s="78"/>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B53" s="8">
+      <c r="B53" s="4">
         <v>49</v>
       </c>
-      <c r="C53" s="8" t="str">
+      <c r="C53" s="4" t="str">
         <f t="shared" si="0"/>
         <v>31h</v>
       </c>
-      <c r="D53" s="75"/>
-      <c r="E53" s="76"/>
-      <c r="F53" s="76"/>
-      <c r="G53" s="77"/>
+      <c r="D53" s="76"/>
+      <c r="E53" s="77"/>
+      <c r="F53" s="77"/>
+      <c r="G53" s="78"/>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B54" s="8">
+      <c r="B54" s="4">
         <v>50</v>
       </c>
-      <c r="C54" s="8" t="str">
+      <c r="C54" s="4" t="str">
         <f t="shared" si="0"/>
         <v>32h</v>
       </c>
-      <c r="D54" s="75"/>
-      <c r="E54" s="76"/>
-      <c r="F54" s="76"/>
-      <c r="G54" s="77"/>
+      <c r="D54" s="76"/>
+      <c r="E54" s="77"/>
+      <c r="F54" s="77"/>
+      <c r="G54" s="78"/>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B55" s="8">
+      <c r="B55" s="4">
         <v>51</v>
       </c>
-      <c r="C55" s="8" t="str">
+      <c r="C55" s="4" t="str">
         <f t="shared" si="0"/>
         <v>33h</v>
       </c>
-      <c r="D55" s="75"/>
-      <c r="E55" s="76"/>
-      <c r="F55" s="76"/>
-      <c r="G55" s="77"/>
+      <c r="D55" s="76"/>
+      <c r="E55" s="77"/>
+      <c r="F55" s="77"/>
+      <c r="G55" s="78"/>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B56" s="8">
+      <c r="B56" s="4">
         <v>52</v>
       </c>
-      <c r="C56" s="8" t="str">
+      <c r="C56" s="4" t="str">
         <f t="shared" si="0"/>
         <v>34h</v>
       </c>
-      <c r="D56" s="75"/>
-      <c r="E56" s="76"/>
-      <c r="F56" s="76"/>
-      <c r="G56" s="77"/>
+      <c r="D56" s="76"/>
+      <c r="E56" s="77"/>
+      <c r="F56" s="77"/>
+      <c r="G56" s="78"/>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B57" s="8">
+      <c r="B57" s="4">
         <v>53</v>
       </c>
-      <c r="C57" s="8" t="str">
+      <c r="C57" s="4" t="str">
         <f t="shared" si="0"/>
         <v>35h</v>
       </c>
-      <c r="D57" s="75"/>
-      <c r="E57" s="76"/>
-      <c r="F57" s="76"/>
-      <c r="G57" s="77"/>
+      <c r="D57" s="76"/>
+      <c r="E57" s="77"/>
+      <c r="F57" s="77"/>
+      <c r="G57" s="78"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B58" s="8">
+      <c r="B58" s="4">
         <v>54</v>
       </c>
-      <c r="C58" s="8" t="str">
+      <c r="C58" s="4" t="str">
         <f t="shared" si="0"/>
         <v>36h</v>
       </c>
-      <c r="D58" s="75"/>
-      <c r="E58" s="76"/>
-      <c r="F58" s="76"/>
-      <c r="G58" s="77"/>
+      <c r="D58" s="76"/>
+      <c r="E58" s="77"/>
+      <c r="F58" s="77"/>
+      <c r="G58" s="78"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B59" s="8">
+      <c r="B59" s="4">
         <v>55</v>
       </c>
-      <c r="C59" s="8" t="str">
+      <c r="C59" s="4" t="str">
         <f t="shared" si="0"/>
         <v>37h</v>
       </c>
-      <c r="D59" s="75"/>
-      <c r="E59" s="76"/>
-      <c r="F59" s="76"/>
-      <c r="G59" s="77"/>
+      <c r="D59" s="76"/>
+      <c r="E59" s="77"/>
+      <c r="F59" s="77"/>
+      <c r="G59" s="78"/>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B60" s="8">
+      <c r="B60" s="4">
         <v>56</v>
       </c>
-      <c r="C60" s="8" t="str">
+      <c r="C60" s="4" t="str">
         <f t="shared" si="0"/>
         <v>38h</v>
       </c>
-      <c r="D60" s="75"/>
-      <c r="E60" s="76"/>
-      <c r="F60" s="76"/>
-      <c r="G60" s="77"/>
+      <c r="D60" s="76"/>
+      <c r="E60" s="77"/>
+      <c r="F60" s="77"/>
+      <c r="G60" s="78"/>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B61" s="8">
+      <c r="B61" s="4">
         <v>57</v>
       </c>
-      <c r="C61" s="8" t="str">
+      <c r="C61" s="4" t="str">
         <f t="shared" si="0"/>
         <v>39h</v>
       </c>
-      <c r="D61" s="75"/>
-      <c r="E61" s="76"/>
-      <c r="F61" s="76"/>
-      <c r="G61" s="77"/>
+      <c r="D61" s="76"/>
+      <c r="E61" s="77"/>
+      <c r="F61" s="77"/>
+      <c r="G61" s="78"/>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B62" s="8">
+      <c r="B62" s="4">
         <v>58</v>
       </c>
-      <c r="C62" s="8" t="str">
+      <c r="C62" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3Ah</v>
       </c>
-      <c r="D62" s="75"/>
-      <c r="E62" s="76"/>
-      <c r="F62" s="76"/>
-      <c r="G62" s="77"/>
+      <c r="D62" s="76"/>
+      <c r="E62" s="77"/>
+      <c r="F62" s="77"/>
+      <c r="G62" s="78"/>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B63" s="8">
+      <c r="B63" s="4">
         <v>59</v>
       </c>
-      <c r="C63" s="8" t="str">
+      <c r="C63" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3Bh</v>
       </c>
-      <c r="D63" s="75"/>
-      <c r="E63" s="76"/>
-      <c r="F63" s="76"/>
-      <c r="G63" s="77"/>
+      <c r="D63" s="76"/>
+      <c r="E63" s="77"/>
+      <c r="F63" s="77"/>
+      <c r="G63" s="78"/>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B64" s="8">
+      <c r="B64" s="4">
         <v>60</v>
       </c>
-      <c r="C64" s="8" t="str">
+      <c r="C64" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3Ch</v>
       </c>
-      <c r="D64" s="75"/>
-      <c r="E64" s="76"/>
-      <c r="F64" s="76"/>
-      <c r="G64" s="77"/>
+      <c r="D64" s="76"/>
+      <c r="E64" s="77"/>
+      <c r="F64" s="77"/>
+      <c r="G64" s="78"/>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B65" s="8">
+      <c r="B65" s="4">
         <v>61</v>
       </c>
-      <c r="C65" s="8" t="str">
+      <c r="C65" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3Dh</v>
       </c>
-      <c r="D65" s="75"/>
-      <c r="E65" s="76"/>
-      <c r="F65" s="76"/>
-      <c r="G65" s="77"/>
+      <c r="D65" s="76"/>
+      <c r="E65" s="77"/>
+      <c r="F65" s="77"/>
+      <c r="G65" s="78"/>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B66" s="8">
+      <c r="B66" s="4">
         <v>62</v>
       </c>
-      <c r="C66" s="8" t="str">
+      <c r="C66" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3Eh</v>
       </c>
-      <c r="D66" s="75"/>
-      <c r="E66" s="76"/>
-      <c r="F66" s="76"/>
-      <c r="G66" s="77"/>
+      <c r="D66" s="76"/>
+      <c r="E66" s="77"/>
+      <c r="F66" s="77"/>
+      <c r="G66" s="78"/>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B67" s="8">
+      <c r="B67" s="4">
         <v>63</v>
       </c>
-      <c r="C67" s="8" t="str">
+      <c r="C67" s="4" t="str">
         <f t="shared" si="0"/>
         <v>3Fh</v>
       </c>
-      <c r="D67" s="75"/>
-      <c r="E67" s="76"/>
-      <c r="F67" s="76"/>
-      <c r="G67" s="77"/>
+      <c r="D67" s="76"/>
+      <c r="E67" s="77"/>
+      <c r="F67" s="77"/>
+      <c r="G67" s="78"/>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B68" s="8">
+      <c r="B68" s="4">
         <v>64</v>
       </c>
-      <c r="C68" s="8" t="str">
+      <c r="C68" s="4" t="str">
         <f t="shared" si="0"/>
         <v>40h</v>
       </c>
-      <c r="D68" s="75"/>
-      <c r="E68" s="76"/>
-      <c r="F68" s="76"/>
-      <c r="G68" s="77"/>
+      <c r="D68" s="76"/>
+      <c r="E68" s="77"/>
+      <c r="F68" s="77"/>
+      <c r="G68" s="78"/>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B69" s="8">
+      <c r="B69" s="4">
         <v>65</v>
       </c>
-      <c r="C69" s="8" t="str">
+      <c r="C69" s="4" t="str">
         <f t="shared" ref="C69:C132" si="1">DEC2HEX(B69)&amp;"h"</f>
         <v>41h</v>
       </c>
-      <c r="D69" s="75"/>
-      <c r="E69" s="76"/>
-      <c r="F69" s="76"/>
-      <c r="G69" s="77"/>
+      <c r="D69" s="76"/>
+      <c r="E69" s="77"/>
+      <c r="F69" s="77"/>
+      <c r="G69" s="78"/>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B70" s="8">
+      <c r="B70" s="4">
         <v>66</v>
       </c>
-      <c r="C70" s="8" t="str">
+      <c r="C70" s="4" t="str">
         <f t="shared" si="1"/>
         <v>42h</v>
       </c>
-      <c r="D70" s="75"/>
-      <c r="E70" s="76"/>
-      <c r="F70" s="76"/>
-      <c r="G70" s="77"/>
+      <c r="D70" s="76"/>
+      <c r="E70" s="77"/>
+      <c r="F70" s="77"/>
+      <c r="G70" s="78"/>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B71" s="8">
+      <c r="B71" s="4">
         <v>67</v>
       </c>
-      <c r="C71" s="8" t="str">
+      <c r="C71" s="4" t="str">
         <f t="shared" si="1"/>
         <v>43h</v>
       </c>
-      <c r="D71" s="75"/>
-      <c r="E71" s="76"/>
-      <c r="F71" s="76"/>
-      <c r="G71" s="77"/>
+      <c r="D71" s="76"/>
+      <c r="E71" s="77"/>
+      <c r="F71" s="77"/>
+      <c r="G71" s="78"/>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B72" s="8">
+      <c r="B72" s="4">
         <v>68</v>
       </c>
-      <c r="C72" s="8" t="str">
+      <c r="C72" s="4" t="str">
         <f t="shared" si="1"/>
         <v>44h</v>
       </c>
-      <c r="D72" s="75"/>
-      <c r="E72" s="76"/>
-      <c r="F72" s="76"/>
-      <c r="G72" s="77"/>
+      <c r="D72" s="76"/>
+      <c r="E72" s="77"/>
+      <c r="F72" s="77"/>
+      <c r="G72" s="78"/>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B73" s="8">
+      <c r="B73" s="4">
         <v>69</v>
       </c>
-      <c r="C73" s="8" t="str">
+      <c r="C73" s="4" t="str">
         <f t="shared" si="1"/>
         <v>45h</v>
       </c>
-      <c r="D73" s="75"/>
-      <c r="E73" s="76"/>
-      <c r="F73" s="76"/>
-      <c r="G73" s="77"/>
+      <c r="D73" s="76"/>
+      <c r="E73" s="77"/>
+      <c r="F73" s="77"/>
+      <c r="G73" s="78"/>
     </row>
     <row r="74" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B74" s="8">
+      <c r="B74" s="4">
         <v>70</v>
       </c>
-      <c r="C74" s="8" t="str">
+      <c r="C74" s="4" t="str">
         <f t="shared" si="1"/>
         <v>46h</v>
       </c>
-      <c r="D74" s="75"/>
-      <c r="E74" s="76"/>
-      <c r="F74" s="76"/>
-      <c r="G74" s="77"/>
+      <c r="D74" s="76"/>
+      <c r="E74" s="77"/>
+      <c r="F74" s="77"/>
+      <c r="G74" s="78"/>
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B75" s="8">
+      <c r="B75" s="4">
         <v>71</v>
       </c>
-      <c r="C75" s="8" t="str">
+      <c r="C75" s="4" t="str">
         <f t="shared" si="1"/>
         <v>47h</v>
       </c>
-      <c r="D75" s="75"/>
-      <c r="E75" s="76"/>
-      <c r="F75" s="76"/>
-      <c r="G75" s="77"/>
+      <c r="D75" s="76"/>
+      <c r="E75" s="77"/>
+      <c r="F75" s="77"/>
+      <c r="G75" s="78"/>
     </row>
     <row r="76" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B76" s="8">
+      <c r="B76" s="4">
         <v>72</v>
       </c>
-      <c r="C76" s="8" t="str">
+      <c r="C76" s="4" t="str">
         <f t="shared" si="1"/>
         <v>48h</v>
       </c>
-      <c r="D76" s="75"/>
-      <c r="E76" s="76"/>
-      <c r="F76" s="76"/>
-      <c r="G76" s="77"/>
+      <c r="D76" s="76"/>
+      <c r="E76" s="77"/>
+      <c r="F76" s="77"/>
+      <c r="G76" s="78"/>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B77" s="8">
+      <c r="B77" s="4">
         <v>73</v>
       </c>
-      <c r="C77" s="8" t="str">
+      <c r="C77" s="4" t="str">
         <f t="shared" si="1"/>
         <v>49h</v>
       </c>
-      <c r="D77" s="75"/>
-      <c r="E77" s="76"/>
-      <c r="F77" s="76"/>
-      <c r="G77" s="77"/>
+      <c r="D77" s="76"/>
+      <c r="E77" s="77"/>
+      <c r="F77" s="77"/>
+      <c r="G77" s="78"/>
     </row>
     <row r="78" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B78" s="8">
+      <c r="B78" s="4">
         <v>74</v>
       </c>
-      <c r="C78" s="8" t="str">
+      <c r="C78" s="4" t="str">
         <f t="shared" si="1"/>
         <v>4Ah</v>
       </c>
-      <c r="D78" s="75"/>
-      <c r="E78" s="76"/>
-      <c r="F78" s="76"/>
-      <c r="G78" s="77"/>
+      <c r="D78" s="76"/>
+      <c r="E78" s="77"/>
+      <c r="F78" s="77"/>
+      <c r="G78" s="78"/>
     </row>
     <row r="79" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B79" s="8">
+      <c r="B79" s="4">
         <v>75</v>
       </c>
-      <c r="C79" s="8" t="str">
+      <c r="C79" s="4" t="str">
         <f t="shared" si="1"/>
         <v>4Bh</v>
       </c>
-      <c r="D79" s="75"/>
-      <c r="E79" s="76"/>
-      <c r="F79" s="76"/>
-      <c r="G79" s="77"/>
+      <c r="D79" s="76"/>
+      <c r="E79" s="77"/>
+      <c r="F79" s="77"/>
+      <c r="G79" s="78"/>
     </row>
     <row r="80" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B80" s="8">
+      <c r="B80" s="4">
         <v>76</v>
       </c>
-      <c r="C80" s="8" t="str">
+      <c r="C80" s="4" t="str">
         <f t="shared" si="1"/>
         <v>4Ch</v>
       </c>
-      <c r="D80" s="78"/>
-      <c r="E80" s="79"/>
-      <c r="F80" s="79"/>
-      <c r="G80" s="80"/>
+      <c r="D80" s="79"/>
+      <c r="E80" s="80"/>
+      <c r="F80" s="80"/>
+      <c r="G80" s="81"/>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B81" s="8">
+      <c r="B81" s="4">
         <v>77</v>
       </c>
-      <c r="C81" s="8" t="str">
+      <c r="C81" s="4" t="str">
         <f t="shared" si="1"/>
         <v>4Dh</v>
       </c>
@@ -2369,10 +2369,10 @@
       <c r="G81" s="1"/>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B82" s="8">
+      <c r="B82" s="4">
         <v>78</v>
       </c>
-      <c r="C82" s="8" t="str">
+      <c r="C82" s="4" t="str">
         <f t="shared" si="1"/>
         <v>4Eh</v>
       </c>
@@ -2382,10 +2382,10 @@
       <c r="G82" s="1"/>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B83" s="8">
+      <c r="B83" s="4">
         <v>79</v>
       </c>
-      <c r="C83" s="8" t="str">
+      <c r="C83" s="4" t="str">
         <f t="shared" si="1"/>
         <v>4Fh</v>
       </c>
@@ -2395,10 +2395,10 @@
       <c r="G83" s="1"/>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B84" s="8">
+      <c r="B84" s="4">
         <v>80</v>
       </c>
-      <c r="C84" s="8" t="str">
+      <c r="C84" s="4" t="str">
         <f t="shared" si="1"/>
         <v>50h</v>
       </c>
@@ -2408,10 +2408,10 @@
       <c r="G84" s="1"/>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B85" s="8">
+      <c r="B85" s="4">
         <v>81</v>
       </c>
-      <c r="C85" s="8" t="str">
+      <c r="C85" s="4" t="str">
         <f t="shared" si="1"/>
         <v>51h</v>
       </c>
@@ -2421,10 +2421,10 @@
       <c r="G85" s="1"/>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B86" s="8">
+      <c r="B86" s="4">
         <v>82</v>
       </c>
-      <c r="C86" s="8" t="str">
+      <c r="C86" s="4" t="str">
         <f t="shared" si="1"/>
         <v>52h</v>
       </c>
@@ -2434,10 +2434,10 @@
       <c r="G86" s="1"/>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B87" s="8">
+      <c r="B87" s="4">
         <v>83</v>
       </c>
-      <c r="C87" s="8" t="str">
+      <c r="C87" s="4" t="str">
         <f t="shared" si="1"/>
         <v>53h</v>
       </c>
@@ -2447,10 +2447,10 @@
       <c r="G87" s="1"/>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B88" s="8">
+      <c r="B88" s="4">
         <v>84</v>
       </c>
-      <c r="C88" s="8" t="str">
+      <c r="C88" s="4" t="str">
         <f t="shared" si="1"/>
         <v>54h</v>
       </c>
@@ -2460,10 +2460,10 @@
       <c r="G88" s="1"/>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B89" s="8">
+      <c r="B89" s="4">
         <v>85</v>
       </c>
-      <c r="C89" s="8" t="str">
+      <c r="C89" s="4" t="str">
         <f t="shared" si="1"/>
         <v>55h</v>
       </c>
@@ -2473,10 +2473,10 @@
       <c r="G89" s="1"/>
     </row>
     <row r="90" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B90" s="8">
+      <c r="B90" s="4">
         <v>86</v>
       </c>
-      <c r="C90" s="8" t="str">
+      <c r="C90" s="4" t="str">
         <f t="shared" si="1"/>
         <v>56h</v>
       </c>
@@ -2486,10 +2486,10 @@
       <c r="G90" s="1"/>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B91" s="8">
+      <c r="B91" s="4">
         <v>87</v>
       </c>
-      <c r="C91" s="8" t="str">
+      <c r="C91" s="4" t="str">
         <f t="shared" si="1"/>
         <v>57h</v>
       </c>
@@ -2499,10 +2499,10 @@
       <c r="G91" s="1"/>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B92" s="8">
+      <c r="B92" s="4">
         <v>88</v>
       </c>
-      <c r="C92" s="8" t="str">
+      <c r="C92" s="4" t="str">
         <f t="shared" si="1"/>
         <v>58h</v>
       </c>
@@ -2512,10 +2512,10 @@
       <c r="G92" s="1"/>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B93" s="8">
+      <c r="B93" s="4">
         <v>89</v>
       </c>
-      <c r="C93" s="8" t="str">
+      <c r="C93" s="4" t="str">
         <f t="shared" si="1"/>
         <v>59h</v>
       </c>
@@ -2525,10 +2525,10 @@
       <c r="G93" s="1"/>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B94" s="8">
+      <c r="B94" s="4">
         <v>90</v>
       </c>
-      <c r="C94" s="8" t="str">
+      <c r="C94" s="4" t="str">
         <f t="shared" si="1"/>
         <v>5Ah</v>
       </c>
@@ -2538,10 +2538,10 @@
       <c r="G94" s="1"/>
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B95" s="8">
+      <c r="B95" s="4">
         <v>91</v>
       </c>
-      <c r="C95" s="8" t="str">
+      <c r="C95" s="4" t="str">
         <f t="shared" si="1"/>
         <v>5Bh</v>
       </c>
@@ -2551,10 +2551,10 @@
       <c r="G95" s="1"/>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B96" s="8">
+      <c r="B96" s="4">
         <v>92</v>
       </c>
-      <c r="C96" s="8" t="str">
+      <c r="C96" s="4" t="str">
         <f t="shared" si="1"/>
         <v>5Ch</v>
       </c>
@@ -2564,10 +2564,10 @@
       <c r="G96" s="1"/>
     </row>
     <row r="97" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B97" s="8">
+      <c r="B97" s="4">
         <v>93</v>
       </c>
-      <c r="C97" s="8" t="str">
+      <c r="C97" s="4" t="str">
         <f t="shared" si="1"/>
         <v>5Dh</v>
       </c>
@@ -2577,10 +2577,10 @@
       <c r="G97" s="1"/>
     </row>
     <row r="98" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B98" s="8">
+      <c r="B98" s="4">
         <v>94</v>
       </c>
-      <c r="C98" s="8" t="str">
+      <c r="C98" s="4" t="str">
         <f t="shared" si="1"/>
         <v>5Eh</v>
       </c>
@@ -2590,10 +2590,10 @@
       <c r="G98" s="1"/>
     </row>
     <row r="99" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B99" s="8">
+      <c r="B99" s="4">
         <v>95</v>
       </c>
-      <c r="C99" s="8" t="str">
+      <c r="C99" s="4" t="str">
         <f t="shared" si="1"/>
         <v>5Fh</v>
       </c>
@@ -2603,10 +2603,10 @@
       <c r="G99" s="1"/>
     </row>
     <row r="100" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B100" s="8">
+      <c r="B100" s="4">
         <v>96</v>
       </c>
-      <c r="C100" s="8" t="str">
+      <c r="C100" s="4" t="str">
         <f t="shared" si="1"/>
         <v>60h</v>
       </c>
@@ -2616,10 +2616,10 @@
       <c r="G100" s="1"/>
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B101" s="8">
+      <c r="B101" s="4">
         <v>97</v>
       </c>
-      <c r="C101" s="8" t="str">
+      <c r="C101" s="4" t="str">
         <f t="shared" si="1"/>
         <v>61h</v>
       </c>
@@ -2629,10 +2629,10 @@
       <c r="G101" s="1"/>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B102" s="8">
+      <c r="B102" s="4">
         <v>98</v>
       </c>
-      <c r="C102" s="8" t="str">
+      <c r="C102" s="4" t="str">
         <f t="shared" si="1"/>
         <v>62h</v>
       </c>
@@ -2642,10 +2642,10 @@
       <c r="G102" s="1"/>
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B103" s="8">
+      <c r="B103" s="4">
         <v>99</v>
       </c>
-      <c r="C103" s="8" t="str">
+      <c r="C103" s="4" t="str">
         <f t="shared" si="1"/>
         <v>63h</v>
       </c>
@@ -2655,10 +2655,10 @@
       <c r="G103" s="1"/>
     </row>
     <row r="104" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B104" s="8">
+      <c r="B104" s="4">
         <v>100</v>
       </c>
-      <c r="C104" s="8" t="str">
+      <c r="C104" s="4" t="str">
         <f t="shared" si="1"/>
         <v>64h</v>
       </c>
@@ -2668,10 +2668,10 @@
       <c r="G104" s="1"/>
     </row>
     <row r="105" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B105" s="8">
+      <c r="B105" s="4">
         <v>101</v>
       </c>
-      <c r="C105" s="8" t="str">
+      <c r="C105" s="4" t="str">
         <f t="shared" si="1"/>
         <v>65h</v>
       </c>
@@ -2681,10 +2681,10 @@
       <c r="G105" s="1"/>
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B106" s="8">
+      <c r="B106" s="4">
         <v>102</v>
       </c>
-      <c r="C106" s="8" t="str">
+      <c r="C106" s="4" t="str">
         <f t="shared" si="1"/>
         <v>66h</v>
       </c>
@@ -2694,10 +2694,10 @@
       <c r="G106" s="1"/>
     </row>
     <row r="107" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B107" s="8">
+      <c r="B107" s="4">
         <v>103</v>
       </c>
-      <c r="C107" s="8" t="str">
+      <c r="C107" s="4" t="str">
         <f t="shared" si="1"/>
         <v>67h</v>
       </c>
@@ -2707,10 +2707,10 @@
       <c r="G107" s="1"/>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B108" s="8">
+      <c r="B108" s="4">
         <v>104</v>
       </c>
-      <c r="C108" s="8" t="str">
+      <c r="C108" s="4" t="str">
         <f t="shared" si="1"/>
         <v>68h</v>
       </c>
@@ -2720,10 +2720,10 @@
       <c r="G108" s="1"/>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B109" s="8">
+      <c r="B109" s="4">
         <v>105</v>
       </c>
-      <c r="C109" s="8" t="str">
+      <c r="C109" s="4" t="str">
         <f t="shared" si="1"/>
         <v>69h</v>
       </c>
@@ -2733,10 +2733,10 @@
       <c r="G109" s="1"/>
     </row>
     <row r="110" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B110" s="8">
+      <c r="B110" s="4">
         <v>106</v>
       </c>
-      <c r="C110" s="8" t="str">
+      <c r="C110" s="4" t="str">
         <f t="shared" si="1"/>
         <v>6Ah</v>
       </c>
@@ -2746,10 +2746,10 @@
       <c r="G110" s="1"/>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B111" s="8">
+      <c r="B111" s="4">
         <v>107</v>
       </c>
-      <c r="C111" s="8" t="str">
+      <c r="C111" s="4" t="str">
         <f t="shared" si="1"/>
         <v>6Bh</v>
       </c>
@@ -2759,10 +2759,10 @@
       <c r="G111" s="1"/>
     </row>
     <row r="112" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B112" s="8">
+      <c r="B112" s="4">
         <v>108</v>
       </c>
-      <c r="C112" s="8" t="str">
+      <c r="C112" s="4" t="str">
         <f t="shared" si="1"/>
         <v>6Ch</v>
       </c>
@@ -2772,10 +2772,10 @@
       <c r="G112" s="1"/>
     </row>
     <row r="113" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B113" s="8">
+      <c r="B113" s="4">
         <v>109</v>
       </c>
-      <c r="C113" s="8" t="str">
+      <c r="C113" s="4" t="str">
         <f t="shared" si="1"/>
         <v>6Dh</v>
       </c>
@@ -2785,10 +2785,10 @@
       <c r="G113" s="1"/>
     </row>
     <row r="114" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B114" s="8">
+      <c r="B114" s="4">
         <v>110</v>
       </c>
-      <c r="C114" s="8" t="str">
+      <c r="C114" s="4" t="str">
         <f t="shared" si="1"/>
         <v>6Eh</v>
       </c>
@@ -2798,10 +2798,10 @@
       <c r="G114" s="1"/>
     </row>
     <row r="115" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B115" s="8">
+      <c r="B115" s="4">
         <v>111</v>
       </c>
-      <c r="C115" s="8" t="str">
+      <c r="C115" s="4" t="str">
         <f t="shared" si="1"/>
         <v>6Fh</v>
       </c>
@@ -2811,10 +2811,10 @@
       <c r="G115" s="1"/>
     </row>
     <row r="116" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B116" s="8">
+      <c r="B116" s="4">
         <v>112</v>
       </c>
-      <c r="C116" s="8" t="str">
+      <c r="C116" s="4" t="str">
         <f t="shared" si="1"/>
         <v>70h</v>
       </c>
@@ -2824,10 +2824,10 @@
       <c r="G116" s="1"/>
     </row>
     <row r="117" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B117" s="8">
+      <c r="B117" s="4">
         <v>113</v>
       </c>
-      <c r="C117" s="8" t="str">
+      <c r="C117" s="4" t="str">
         <f t="shared" si="1"/>
         <v>71h</v>
       </c>
@@ -2837,10 +2837,10 @@
       <c r="G117" s="1"/>
     </row>
     <row r="118" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B118" s="8">
+      <c r="B118" s="4">
         <v>114</v>
       </c>
-      <c r="C118" s="8" t="str">
+      <c r="C118" s="4" t="str">
         <f t="shared" si="1"/>
         <v>72h</v>
       </c>
@@ -2850,10 +2850,10 @@
       <c r="G118" s="1"/>
     </row>
     <row r="119" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B119" s="8">
+      <c r="B119" s="4">
         <v>115</v>
       </c>
-      <c r="C119" s="8" t="str">
+      <c r="C119" s="4" t="str">
         <f t="shared" si="1"/>
         <v>73h</v>
       </c>
@@ -2863,10 +2863,10 @@
       <c r="G119" s="1"/>
     </row>
     <row r="120" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B120" s="8">
+      <c r="B120" s="4">
         <v>116</v>
       </c>
-      <c r="C120" s="8" t="str">
+      <c r="C120" s="4" t="str">
         <f t="shared" si="1"/>
         <v>74h</v>
       </c>
@@ -2876,10 +2876,10 @@
       <c r="G120" s="1"/>
     </row>
     <row r="121" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B121" s="8">
+      <c r="B121" s="4">
         <v>117</v>
       </c>
-      <c r="C121" s="8" t="str">
+      <c r="C121" s="4" t="str">
         <f t="shared" si="1"/>
         <v>75h</v>
       </c>
@@ -2889,10 +2889,10 @@
       <c r="G121" s="1"/>
     </row>
     <row r="122" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B122" s="8">
+      <c r="B122" s="4">
         <v>118</v>
       </c>
-      <c r="C122" s="8" t="str">
+      <c r="C122" s="4" t="str">
         <f t="shared" si="1"/>
         <v>76h</v>
       </c>
@@ -2902,10 +2902,10 @@
       <c r="G122" s="1"/>
     </row>
     <row r="123" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B123" s="8">
+      <c r="B123" s="4">
         <v>119</v>
       </c>
-      <c r="C123" s="8" t="str">
+      <c r="C123" s="4" t="str">
         <f t="shared" si="1"/>
         <v>77h</v>
       </c>
@@ -2915,10 +2915,10 @@
       <c r="G123" s="1"/>
     </row>
     <row r="124" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B124" s="8">
+      <c r="B124" s="4">
         <v>120</v>
       </c>
-      <c r="C124" s="8" t="str">
+      <c r="C124" s="4" t="str">
         <f t="shared" si="1"/>
         <v>78h</v>
       </c>
@@ -2928,10 +2928,10 @@
       <c r="G124" s="1"/>
     </row>
     <row r="125" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B125" s="8">
+      <c r="B125" s="4">
         <v>121</v>
       </c>
-      <c r="C125" s="8" t="str">
+      <c r="C125" s="4" t="str">
         <f t="shared" si="1"/>
         <v>79h</v>
       </c>
@@ -2941,10 +2941,10 @@
       <c r="G125" s="1"/>
     </row>
     <row r="126" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B126" s="8">
+      <c r="B126" s="4">
         <v>122</v>
       </c>
-      <c r="C126" s="8" t="str">
+      <c r="C126" s="4" t="str">
         <f t="shared" si="1"/>
         <v>7Ah</v>
       </c>
@@ -2954,10 +2954,10 @@
       <c r="G126" s="1"/>
     </row>
     <row r="127" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B127" s="8">
+      <c r="B127" s="4">
         <v>123</v>
       </c>
-      <c r="C127" s="8" t="str">
+      <c r="C127" s="4" t="str">
         <f t="shared" si="1"/>
         <v>7Bh</v>
       </c>
@@ -2967,10 +2967,10 @@
       <c r="G127" s="1"/>
     </row>
     <row r="128" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B128" s="8">
+      <c r="B128" s="4">
         <v>124</v>
       </c>
-      <c r="C128" s="8" t="str">
+      <c r="C128" s="4" t="str">
         <f t="shared" si="1"/>
         <v>7Ch</v>
       </c>
@@ -2980,10 +2980,10 @@
       <c r="G128" s="1"/>
     </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B129" s="8">
+      <c r="B129" s="4">
         <v>125</v>
       </c>
-      <c r="C129" s="8" t="str">
+      <c r="C129" s="4" t="str">
         <f t="shared" si="1"/>
         <v>7Dh</v>
       </c>
@@ -2993,10 +2993,10 @@
       <c r="G129" s="1"/>
     </row>
     <row r="130" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B130" s="8">
+      <c r="B130" s="4">
         <v>126</v>
       </c>
-      <c r="C130" s="8" t="str">
+      <c r="C130" s="4" t="str">
         <f t="shared" si="1"/>
         <v>7Eh</v>
       </c>
@@ -3006,10 +3006,10 @@
       <c r="G130" s="1"/>
     </row>
     <row r="131" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B131" s="8">
+      <c r="B131" s="4">
         <v>127</v>
       </c>
-      <c r="C131" s="8" t="str">
+      <c r="C131" s="4" t="str">
         <f t="shared" si="1"/>
         <v>7Fh</v>
       </c>
@@ -3019,10 +3019,10 @@
       <c r="G131" s="1"/>
     </row>
     <row r="132" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B132" s="8">
+      <c r="B132" s="4">
         <v>128</v>
       </c>
-      <c r="C132" s="8" t="str">
+      <c r="C132" s="4" t="str">
         <f t="shared" si="1"/>
         <v>80h</v>
       </c>
@@ -3032,10 +3032,10 @@
       <c r="G132" s="1"/>
     </row>
     <row r="133" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B133" s="8">
+      <c r="B133" s="4">
         <v>129</v>
       </c>
-      <c r="C133" s="8" t="str">
+      <c r="C133" s="4" t="str">
         <f t="shared" ref="C133:C138" si="2">DEC2HEX(B133)&amp;"h"</f>
         <v>81h</v>
       </c>
@@ -3045,103 +3045,103 @@
       <c r="G133" s="1"/>
     </row>
     <row r="134" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B134" s="8">
+      <c r="B134" s="4">
         <v>130</v>
       </c>
-      <c r="C134" s="8" t="str">
+      <c r="C134" s="4" t="str">
         <f t="shared" si="2"/>
         <v>82h</v>
       </c>
-      <c r="D134" s="86" t="s">
+      <c r="D134" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="E134" s="87"/>
-      <c r="F134" s="88"/>
-      <c r="G134" s="92" t="s">
+      <c r="E134" s="23"/>
+      <c r="F134" s="24"/>
+      <c r="G134" s="20" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="135" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B135" s="8">
+      <c r="B135" s="4">
         <v>131</v>
       </c>
-      <c r="C135" s="8" t="str">
+      <c r="C135" s="4" t="str">
         <f t="shared" si="2"/>
         <v>83h</v>
       </c>
-      <c r="D135" s="89" t="s">
+      <c r="D135" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="E135" s="90"/>
-      <c r="F135" s="90"/>
-      <c r="G135" s="91"/>
+      <c r="E135" s="27"/>
+      <c r="F135" s="27"/>
+      <c r="G135" s="26"/>
     </row>
     <row r="136" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B136" s="8">
+      <c r="B136" s="4">
         <v>132</v>
       </c>
-      <c r="C136" s="8" t="str">
+      <c r="C136" s="4" t="str">
         <f t="shared" si="2"/>
         <v>84h</v>
       </c>
-      <c r="D136" s="89" t="s">
+      <c r="D136" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="E136" s="90"/>
-      <c r="F136" s="90"/>
-      <c r="G136" s="91"/>
+      <c r="E136" s="27"/>
+      <c r="F136" s="27"/>
+      <c r="G136" s="26"/>
     </row>
     <row r="137" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B137" s="8">
+      <c r="B137" s="4">
         <v>133</v>
       </c>
-      <c r="C137" s="8" t="str">
+      <c r="C137" s="4" t="str">
         <f t="shared" si="2"/>
         <v>85h</v>
       </c>
-      <c r="D137" s="89" t="s">
+      <c r="D137" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="E137" s="90"/>
-      <c r="F137" s="90"/>
-      <c r="G137" s="91"/>
+      <c r="E137" s="27"/>
+      <c r="F137" s="27"/>
+      <c r="G137" s="26"/>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B138" s="8">
+      <c r="B138" s="4">
         <v>134</v>
       </c>
-      <c r="C138" s="8" t="str">
+      <c r="C138" s="4" t="str">
         <f t="shared" si="2"/>
         <v>86h</v>
       </c>
-      <c r="D138" s="89" t="s">
+      <c r="D138" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="E138" s="91"/>
-      <c r="F138" s="89" t="s">
+      <c r="E138" s="26"/>
+      <c r="F138" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="G138" s="91"/>
+      <c r="G138" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="D41:G80"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D4:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="D8:G20"/>
+    <mergeCell ref="D31:G35"/>
+    <mergeCell ref="D21:G25"/>
+    <mergeCell ref="D26:G30"/>
+    <mergeCell ref="D36:G40"/>
     <mergeCell ref="D134:F134"/>
     <mergeCell ref="D138:E138"/>
     <mergeCell ref="F138:G138"/>
     <mergeCell ref="D135:G135"/>
     <mergeCell ref="D136:G136"/>
     <mergeCell ref="D137:G137"/>
-    <mergeCell ref="D8:G20"/>
-    <mergeCell ref="D31:G35"/>
-    <mergeCell ref="D21:G25"/>
-    <mergeCell ref="D26:G30"/>
-    <mergeCell ref="D36:G40"/>
-    <mergeCell ref="D41:G80"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="D4:G5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="D7:G7"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="K10" r:id="rId1" xr:uid="{4CDEDA9D-6A17-4E55-8BF2-30A318687126}"/>
@@ -3152,6 +3152,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100428D6099D6E2B6448E8A88B2B567960C" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d06e3c45a3f093fe91a85c3d3a514f99">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="602d6013-12bf-42a7-bc7f-2fade0e82371" xmlns:ns4="98306238-8ebe-44ab-acf1-12aa768c5e84" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="892bbdd5d735959505dc654187d2f43d" ns3:_="" ns4:_="">
     <xsd:import namespace="602d6013-12bf-42a7-bc7f-2fade0e82371"/>
@@ -3346,15 +3355,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3364,6 +3364,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AF9C2AB-D531-4B8D-9A76-F0FAB1D11F28}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3378,14 +3386,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Got the readPages function to print card data (still in progress)
</commit_message>
<xml_diff>
--- a/wh40k_NTAG215_memoryMapping.xlsx
+++ b/wh40k_NTAG215_memoryMapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fuzzy\wh40k_nfc_project\wh40k_nfc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23062AE8-122C-4DEC-BC0B-3DF28DBF9347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03717F51-B96D-431E-AA05-9B9B2C78FE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="19420" windowHeight="10300" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
+    <workbookView xWindow="0" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>NTAG215</t>
   </si>
@@ -122,24 +122,6 @@
     <t>"Total Deaths: 9"</t>
   </si>
   <si>
-    <t>Dynamic Lock Bytes</t>
-  </si>
-  <si>
-    <t>RFUI</t>
-  </si>
-  <si>
-    <t>CFG 0</t>
-  </si>
-  <si>
-    <t>CFG 1</t>
-  </si>
-  <si>
-    <t>PWD</t>
-  </si>
-  <si>
-    <t>PACK</t>
-  </si>
-  <si>
     <t>Lock/internal</t>
   </si>
   <si>
@@ -156,6 +138,36 @@
   </si>
   <si>
     <t>Remaining Bytes</t>
+  </si>
+  <si>
+    <t>current health</t>
+  </si>
+  <si>
+    <t>total kills</t>
+  </si>
+  <si>
+    <t>total deaths</t>
+  </si>
+  <si>
+    <t>max health</t>
+  </si>
+  <si>
+    <t>OTHER DATA</t>
+  </si>
+  <si>
+    <t>dgi</t>
+  </si>
+  <si>
+    <t>dynamic game id (dgi)</t>
+  </si>
+  <si>
+    <t>model type</t>
+  </si>
+  <si>
+    <t># of models in group</t>
+  </si>
+  <si>
+    <t>EXTRA SPACE</t>
   </si>
 </sst>
 </file>
@@ -179,7 +191,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -252,8 +264,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -372,15 +414,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -453,77 +486,6 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -534,7 +496,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -550,10 +512,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -569,190 +531,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -771,24 +550,50 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -826,7 +631,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>127050</xdr:colOff>
+      <xdr:colOff>127051</xdr:colOff>
       <xdr:row>39</xdr:row>
       <xdr:rowOff>124951</xdr:rowOff>
     </xdr:to>
@@ -1181,40 +986,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E22B5351-43EC-4BE6-A109-53A8CF40F7FA}">
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K155"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18.90625" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" customWidth="1"/>
+    <col min="6" max="6" width="19.36328125" customWidth="1"/>
+    <col min="7" max="7" width="17.08984375" customWidth="1"/>
+    <col min="9" max="9" width="20.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="J1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K1" t="s">
-        <v>11</v>
-      </c>
     </row>
     <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="82" t="s">
+      <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="83"/>
-      <c r="D2" s="84" t="s">
+      <c r="C2" s="22"/>
+      <c r="D2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="86"/>
-      <c r="I2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="J2" s="6">
-        <v>9</v>
-      </c>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25"/>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="2" t="s">
@@ -1235,12 +1032,6 @@
       <c r="G3" s="7">
         <v>3</v>
       </c>
-      <c r="I3" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="11">
-        <v>3</v>
-      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B4" s="3">
@@ -1250,17 +1041,14 @@
         <f>DEC2HEX(B4)&amp;"h"</f>
         <v>0h</v>
       </c>
-      <c r="D4" s="87" t="s">
+      <c r="D4" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="I4" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="18">
-        <v>4</v>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="26"/>
+      <c r="J4" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -1271,18 +1059,15 @@
         <f t="shared" ref="C5:C68" si="0">DEC2HEX(B5)&amp;"h"</f>
         <v>1h</v>
       </c>
-      <c r="D5" s="88"/>
-      <c r="E5" s="87"/>
-      <c r="F5" s="87"/>
-      <c r="G5" s="87"/>
-      <c r="I5" s="12" t="s">
+      <c r="D5" s="27"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="26"/>
+      <c r="I5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="J5" s="6">
         <v>9</v>
-      </c>
-      <c r="J5" s="12">
-        <v>52</v>
-      </c>
-      <c r="K5" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1297,18 +1082,18 @@
       <c r="E6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="89" t="s">
+      <c r="F6" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="90"/>
-      <c r="I6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="J6" s="13">
-        <v>20</v>
+      <c r="G6" s="29"/>
+      <c r="I6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="J6" s="11">
+        <v>3</v>
       </c>
       <c r="K6" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
@@ -1319,20 +1104,17 @@
         <f t="shared" si="0"/>
         <v>3h</v>
       </c>
-      <c r="D7" s="91" t="s">
+      <c r="D7" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="92"/>
-      <c r="F7" s="92"/>
-      <c r="G7" s="93"/>
-      <c r="I7" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" s="13">
-        <v>20</v>
-      </c>
-      <c r="K7" t="s">
-        <v>24</v>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="32"/>
+      <c r="I7" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="J7" s="18">
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -1343,20 +1125,21 @@
         <f t="shared" si="0"/>
         <v>4h</v>
       </c>
-      <c r="D8" s="28" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="30"/>
-      <c r="I8" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="J8" s="14">
-        <v>20</v>
-      </c>
-      <c r="K8" t="s">
-        <v>26</v>
+      <c r="D8" s="40" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="43"/>
+      <c r="I8" s="39" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" s="39">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -1367,18 +1150,23 @@
         <f t="shared" si="0"/>
         <v>5h</v>
       </c>
-      <c r="D9" s="31"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="33"/>
-      <c r="I9" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="15">
-        <v>20</v>
-      </c>
-      <c r="K9" t="s">
-        <v>27</v>
+      <c r="D9" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="42" t="s">
+        <v>36</v>
+      </c>
+      <c r="I9" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -1389,18 +1177,17 @@
         <f t="shared" si="0"/>
         <v>6h</v>
       </c>
-      <c r="D10" s="31"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="33"/>
-      <c r="I10" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" s="17">
-        <v>200</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>19</v>
+      <c r="D10" s="46" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="46"/>
+      <c r="F10" s="46"/>
+      <c r="G10" s="46"/>
+      <c r="I10" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -1411,12 +1198,17 @@
         <f t="shared" si="0"/>
         <v>7h</v>
       </c>
-      <c r="D11" s="31"/>
-      <c r="E11" s="32"/>
-      <c r="F11" s="32"/>
-      <c r="G11" s="33"/>
-      <c r="K11" t="s">
-        <v>21</v>
+      <c r="D11" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="I11" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" s="43">
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -1427,13 +1219,10 @@
         <f t="shared" si="0"/>
         <v>8h</v>
       </c>
-      <c r="D12" s="31"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="33"/>
-      <c r="K12" t="s">
-        <v>22</v>
-      </c>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B13" s="4">
@@ -1443,16 +1232,10 @@
         <f t="shared" si="0"/>
         <v>9h</v>
       </c>
-      <c r="D13" s="31"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="33"/>
-      <c r="I13" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="J13" s="19">
-        <v>3</v>
-      </c>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B14" s="4">
@@ -1462,16 +1245,10 @@
         <f t="shared" si="0"/>
         <v>Ah</v>
       </c>
-      <c r="D14" s="31"/>
-      <c r="E14" s="32"/>
-      <c r="F14" s="32"/>
-      <c r="G14" s="33"/>
-      <c r="I14" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="J14" s="21">
-        <v>17</v>
-      </c>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B15" s="4">
@@ -1481,10 +1258,19 @@
         <f t="shared" si="0"/>
         <v>Bh</v>
       </c>
-      <c r="D15" s="31"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="I15" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="J15" s="12">
+        <v>52</v>
+      </c>
+      <c r="K15" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B16" s="4">
@@ -1494,19 +1280,21 @@
         <f t="shared" si="0"/>
         <v>Ch</v>
       </c>
-      <c r="D16" s="31"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="33"/>
-      <c r="I16" t="s">
-        <v>38</v>
-      </c>
-      <c r="J16">
-        <f>SUM(J2:J14)</f>
-        <v>368</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="I16" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="J16" s="41">
+        <v>1</v>
+      </c>
+      <c r="K16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B17" s="4">
         <v>13</v>
       </c>
@@ -1514,19 +1302,21 @@
         <f t="shared" si="0"/>
         <v>Dh</v>
       </c>
-      <c r="D17" s="31"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33"/>
-      <c r="I17" t="s">
-        <v>39</v>
-      </c>
-      <c r="J17">
-        <f>540-J16</f>
-        <v>172</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="I17" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="13">
+        <v>1</v>
+      </c>
+      <c r="K17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B18" s="4">
         <v>14</v>
       </c>
@@ -1534,12 +1324,21 @@
         <f t="shared" si="0"/>
         <v>Eh</v>
       </c>
-      <c r="D18" s="31"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33"/>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="I18" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="14">
+        <v>1</v>
+      </c>
+      <c r="K18" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B19" s="4">
         <v>15</v>
       </c>
@@ -1547,12 +1346,21 @@
         <f t="shared" si="0"/>
         <v>Fh</v>
       </c>
-      <c r="D19" s="31"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="33"/>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="I19" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J19" s="15">
+        <v>1</v>
+      </c>
+      <c r="K19" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B20" s="4">
         <v>16</v>
       </c>
@@ -1561,11 +1369,17 @@
         <v>10h</v>
       </c>
       <c r="D20" s="34"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="36"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="I20" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="J20" s="43">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B21" s="4">
         <v>17</v>
       </c>
@@ -1573,14 +1387,21 @@
         <f t="shared" si="0"/>
         <v>11h</v>
       </c>
-      <c r="D21" s="46" t="s">
-        <v>17</v>
-      </c>
-      <c r="E21" s="47"/>
-      <c r="F21" s="47"/>
-      <c r="G21" s="48"/>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="I21" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" s="17">
+        <v>200</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B22" s="4">
         <v>18</v>
       </c>
@@ -1588,12 +1409,15 @@
         <f t="shared" si="0"/>
         <v>12h</v>
       </c>
-      <c r="D22" s="49"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
-      <c r="G22" s="51"/>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="K22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B23" s="4">
         <v>19</v>
       </c>
@@ -1601,12 +1425,15 @@
         <f t="shared" si="0"/>
         <v>13h</v>
       </c>
-      <c r="D23" s="49"/>
-      <c r="E23" s="50"/>
-      <c r="F23" s="50"/>
-      <c r="G23" s="51"/>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
+      <c r="K23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B24" s="4">
         <v>20</v>
       </c>
@@ -1614,12 +1441,14 @@
         <f t="shared" si="0"/>
         <v>14h</v>
       </c>
-      <c r="D24" s="49"/>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="51"/>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="I24" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="J24" s="19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B25" s="4">
         <v>21</v>
       </c>
@@ -1627,12 +1456,20 @@
         <f t="shared" si="0"/>
         <v>15h</v>
       </c>
-      <c r="D25" s="52"/>
-      <c r="E25" s="53"/>
-      <c r="F25" s="53"/>
-      <c r="G25" s="54"/>
-    </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D25" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="43"/>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+      <c r="I25" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="J25" s="20">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B26" s="4">
         <v>22</v>
       </c>
@@ -1640,14 +1477,8 @@
         <f t="shared" si="0"/>
         <v>16h</v>
       </c>
-      <c r="D26" s="55" t="s">
-        <v>18</v>
-      </c>
-      <c r="E26" s="56"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="57"/>
-    </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B27" s="4">
         <v>23</v>
       </c>
@@ -1655,12 +1486,15 @@
         <f t="shared" si="0"/>
         <v>17h</v>
       </c>
-      <c r="D27" s="58"/>
-      <c r="E27" s="59"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="60"/>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="I27" t="s">
+        <v>32</v>
+      </c>
+      <c r="J27">
+        <f>SUM(J5:J25)</f>
+        <v>304</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B28" s="4">
         <v>24</v>
       </c>
@@ -1668,12 +1502,15 @@
         <f t="shared" si="0"/>
         <v>18h</v>
       </c>
-      <c r="D28" s="58"/>
-      <c r="E28" s="59"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="60"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="I28" t="s">
+        <v>33</v>
+      </c>
+      <c r="J28">
+        <f>540-J27</f>
+        <v>236</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B29" s="4">
         <v>25</v>
       </c>
@@ -1681,12 +1518,8 @@
         <f t="shared" si="0"/>
         <v>19h</v>
       </c>
-      <c r="D29" s="58"/>
-      <c r="E29" s="59"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="60"/>
-    </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B30" s="4">
         <v>26</v>
       </c>
@@ -1694,12 +1527,8 @@
         <f t="shared" si="0"/>
         <v>1Ah</v>
       </c>
-      <c r="D30" s="61"/>
-      <c r="E30" s="62"/>
-      <c r="F30" s="62"/>
-      <c r="G30" s="63"/>
-    </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B31" s="4">
         <v>27</v>
       </c>
@@ -1707,14 +1536,8 @@
         <f t="shared" si="0"/>
         <v>1Bh</v>
       </c>
-      <c r="D31" s="37" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" s="38"/>
-      <c r="F31" s="38"/>
-      <c r="G31" s="39"/>
-    </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B32" s="4">
         <v>28</v>
       </c>
@@ -1722,12 +1545,8 @@
         <f t="shared" si="0"/>
         <v>1Ch</v>
       </c>
-      <c r="D32" s="40"/>
-      <c r="E32" s="41"/>
-      <c r="F32" s="41"/>
-      <c r="G32" s="42"/>
-    </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B33" s="4">
         <v>29</v>
       </c>
@@ -1735,12 +1554,8 @@
         <f t="shared" si="0"/>
         <v>1Dh</v>
       </c>
-      <c r="D33" s="40"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
-    </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B34" s="4">
         <v>30</v>
       </c>
@@ -1748,12 +1563,8 @@
         <f t="shared" si="0"/>
         <v>1Eh</v>
       </c>
-      <c r="D34" s="40"/>
-      <c r="E34" s="41"/>
-      <c r="F34" s="41"/>
-      <c r="G34" s="42"/>
-    </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B35" s="4">
         <v>31</v>
       </c>
@@ -1761,12 +1572,8 @@
         <f t="shared" si="0"/>
         <v>1Fh</v>
       </c>
-      <c r="D35" s="43"/>
-      <c r="E35" s="44"/>
-      <c r="F35" s="44"/>
-      <c r="G35" s="45"/>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B36" s="4">
         <v>32</v>
       </c>
@@ -1774,14 +1581,8 @@
         <f t="shared" si="0"/>
         <v>20h</v>
       </c>
-      <c r="D36" s="64" t="s">
-        <v>14</v>
-      </c>
-      <c r="E36" s="65"/>
-      <c r="F36" s="65"/>
-      <c r="G36" s="66"/>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B37" s="4">
         <v>33</v>
       </c>
@@ -1789,12 +1590,8 @@
         <f t="shared" si="0"/>
         <v>21h</v>
       </c>
-      <c r="D37" s="67"/>
-      <c r="E37" s="68"/>
-      <c r="F37" s="68"/>
-      <c r="G37" s="69"/>
-    </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B38" s="4">
         <v>34</v>
       </c>
@@ -1802,12 +1599,8 @@
         <f t="shared" si="0"/>
         <v>22h</v>
       </c>
-      <c r="D38" s="67"/>
-      <c r="E38" s="68"/>
-      <c r="F38" s="68"/>
-      <c r="G38" s="69"/>
-    </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B39" s="4">
         <v>35</v>
       </c>
@@ -1815,12 +1608,8 @@
         <f t="shared" si="0"/>
         <v>23h</v>
       </c>
-      <c r="D39" s="67"/>
-      <c r="E39" s="68"/>
-      <c r="F39" s="68"/>
-      <c r="G39" s="69"/>
-    </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B40" s="4">
         <v>36</v>
       </c>
@@ -1828,12 +1617,8 @@
         <f t="shared" si="0"/>
         <v>24h</v>
       </c>
-      <c r="D40" s="70"/>
-      <c r="E40" s="71"/>
-      <c r="F40" s="71"/>
-      <c r="G40" s="72"/>
-    </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B41" s="4">
         <v>37</v>
       </c>
@@ -1841,14 +1626,8 @@
         <f t="shared" si="0"/>
         <v>25h</v>
       </c>
-      <c r="D41" s="73" t="s">
-        <v>23</v>
-      </c>
-      <c r="E41" s="74"/>
-      <c r="F41" s="74"/>
-      <c r="G41" s="75"/>
-    </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B42" s="4">
         <v>38</v>
       </c>
@@ -1856,12 +1635,8 @@
         <f t="shared" si="0"/>
         <v>26h</v>
       </c>
-      <c r="D42" s="76"/>
-      <c r="E42" s="77"/>
-      <c r="F42" s="77"/>
-      <c r="G42" s="78"/>
-    </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B43" s="4">
         <v>39</v>
       </c>
@@ -1869,12 +1644,8 @@
         <f t="shared" si="0"/>
         <v>27h</v>
       </c>
-      <c r="D43" s="76"/>
-      <c r="E43" s="77"/>
-      <c r="F43" s="77"/>
-      <c r="G43" s="78"/>
-    </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B44" s="4">
         <v>40</v>
       </c>
@@ -1882,12 +1653,8 @@
         <f t="shared" si="0"/>
         <v>28h</v>
       </c>
-      <c r="D44" s="76"/>
-      <c r="E44" s="77"/>
-      <c r="F44" s="77"/>
-      <c r="G44" s="78"/>
-    </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B45" s="4">
         <v>41</v>
       </c>
@@ -1895,12 +1662,8 @@
         <f t="shared" si="0"/>
         <v>29h</v>
       </c>
-      <c r="D45" s="76"/>
-      <c r="E45" s="77"/>
-      <c r="F45" s="77"/>
-      <c r="G45" s="78"/>
-    </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B46" s="4">
         <v>42</v>
       </c>
@@ -1908,12 +1671,8 @@
         <f t="shared" si="0"/>
         <v>2Ah</v>
       </c>
-      <c r="D46" s="76"/>
-      <c r="E46" s="77"/>
-      <c r="F46" s="77"/>
-      <c r="G46" s="78"/>
-    </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B47" s="4">
         <v>43</v>
       </c>
@@ -1921,12 +1680,8 @@
         <f t="shared" si="0"/>
         <v>2Bh</v>
       </c>
-      <c r="D47" s="76"/>
-      <c r="E47" s="77"/>
-      <c r="F47" s="77"/>
-      <c r="G47" s="78"/>
-    </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B48" s="4">
         <v>44</v>
       </c>
@@ -1934,12 +1689,8 @@
         <f t="shared" si="0"/>
         <v>2Ch</v>
       </c>
-      <c r="D48" s="76"/>
-      <c r="E48" s="77"/>
-      <c r="F48" s="77"/>
-      <c r="G48" s="78"/>
-    </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B49" s="4">
         <v>45</v>
       </c>
@@ -1947,12 +1698,8 @@
         <f t="shared" si="0"/>
         <v>2Dh</v>
       </c>
-      <c r="D49" s="76"/>
-      <c r="E49" s="77"/>
-      <c r="F49" s="77"/>
-      <c r="G49" s="78"/>
-    </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B50" s="4">
         <v>46</v>
       </c>
@@ -1960,12 +1707,8 @@
         <f t="shared" si="0"/>
         <v>2Eh</v>
       </c>
-      <c r="D50" s="76"/>
-      <c r="E50" s="77"/>
-      <c r="F50" s="77"/>
-      <c r="G50" s="78"/>
-    </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B51" s="4">
         <v>47</v>
       </c>
@@ -1973,12 +1716,8 @@
         <f t="shared" si="0"/>
         <v>2Fh</v>
       </c>
-      <c r="D51" s="76"/>
-      <c r="E51" s="77"/>
-      <c r="F51" s="77"/>
-      <c r="G51" s="78"/>
-    </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B52" s="4">
         <v>48</v>
       </c>
@@ -1986,12 +1725,8 @@
         <f t="shared" si="0"/>
         <v>30h</v>
       </c>
-      <c r="D52" s="76"/>
-      <c r="E52" s="77"/>
-      <c r="F52" s="77"/>
-      <c r="G52" s="78"/>
-    </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B53" s="4">
         <v>49</v>
       </c>
@@ -1999,12 +1734,8 @@
         <f t="shared" si="0"/>
         <v>31h</v>
       </c>
-      <c r="D53" s="76"/>
-      <c r="E53" s="77"/>
-      <c r="F53" s="77"/>
-      <c r="G53" s="78"/>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B54" s="4">
         <v>50</v>
       </c>
@@ -2012,12 +1743,8 @@
         <f t="shared" si="0"/>
         <v>32h</v>
       </c>
-      <c r="D54" s="76"/>
-      <c r="E54" s="77"/>
-      <c r="F54" s="77"/>
-      <c r="G54" s="78"/>
-    </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B55" s="4">
         <v>51</v>
       </c>
@@ -2025,12 +1752,8 @@
         <f t="shared" si="0"/>
         <v>33h</v>
       </c>
-      <c r="D55" s="76"/>
-      <c r="E55" s="77"/>
-      <c r="F55" s="77"/>
-      <c r="G55" s="78"/>
-    </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B56" s="4">
         <v>52</v>
       </c>
@@ -2038,12 +1761,8 @@
         <f t="shared" si="0"/>
         <v>34h</v>
       </c>
-      <c r="D56" s="76"/>
-      <c r="E56" s="77"/>
-      <c r="F56" s="77"/>
-      <c r="G56" s="78"/>
-    </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B57" s="4">
         <v>53</v>
       </c>
@@ -2051,12 +1770,8 @@
         <f t="shared" si="0"/>
         <v>35h</v>
       </c>
-      <c r="D57" s="76"/>
-      <c r="E57" s="77"/>
-      <c r="F57" s="77"/>
-      <c r="G57" s="78"/>
-    </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B58" s="4">
         <v>54</v>
       </c>
@@ -2064,12 +1779,8 @@
         <f t="shared" si="0"/>
         <v>36h</v>
       </c>
-      <c r="D58" s="76"/>
-      <c r="E58" s="77"/>
-      <c r="F58" s="77"/>
-      <c r="G58" s="78"/>
-    </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B59" s="4">
         <v>55</v>
       </c>
@@ -2077,12 +1788,8 @@
         <f t="shared" si="0"/>
         <v>37h</v>
       </c>
-      <c r="D59" s="76"/>
-      <c r="E59" s="77"/>
-      <c r="F59" s="77"/>
-      <c r="G59" s="78"/>
-    </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B60" s="4">
         <v>56</v>
       </c>
@@ -2090,12 +1797,8 @@
         <f t="shared" si="0"/>
         <v>38h</v>
       </c>
-      <c r="D60" s="76"/>
-      <c r="E60" s="77"/>
-      <c r="F60" s="77"/>
-      <c r="G60" s="78"/>
-    </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B61" s="4">
         <v>57</v>
       </c>
@@ -2103,12 +1806,8 @@
         <f t="shared" si="0"/>
         <v>39h</v>
       </c>
-      <c r="D61" s="76"/>
-      <c r="E61" s="77"/>
-      <c r="F61" s="77"/>
-      <c r="G61" s="78"/>
-    </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B62" s="4">
         <v>58</v>
       </c>
@@ -2116,12 +1815,8 @@
         <f t="shared" si="0"/>
         <v>3Ah</v>
       </c>
-      <c r="D62" s="76"/>
-      <c r="E62" s="77"/>
-      <c r="F62" s="77"/>
-      <c r="G62" s="78"/>
-    </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B63" s="4">
         <v>59</v>
       </c>
@@ -2129,12 +1824,8 @@
         <f t="shared" si="0"/>
         <v>3Bh</v>
       </c>
-      <c r="D63" s="76"/>
-      <c r="E63" s="77"/>
-      <c r="F63" s="77"/>
-      <c r="G63" s="78"/>
-    </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B64" s="4">
         <v>60</v>
       </c>
@@ -2142,12 +1833,8 @@
         <f t="shared" si="0"/>
         <v>3Ch</v>
       </c>
-      <c r="D64" s="76"/>
-      <c r="E64" s="77"/>
-      <c r="F64" s="77"/>
-      <c r="G64" s="78"/>
-    </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B65" s="4">
         <v>61</v>
       </c>
@@ -2155,12 +1842,8 @@
         <f t="shared" si="0"/>
         <v>3Dh</v>
       </c>
-      <c r="D65" s="76"/>
-      <c r="E65" s="77"/>
-      <c r="F65" s="77"/>
-      <c r="G65" s="78"/>
-    </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B66" s="4">
         <v>62</v>
       </c>
@@ -2168,12 +1851,8 @@
         <f t="shared" si="0"/>
         <v>3Eh</v>
       </c>
-      <c r="D66" s="76"/>
-      <c r="E66" s="77"/>
-      <c r="F66" s="77"/>
-      <c r="G66" s="78"/>
-    </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B67" s="4">
         <v>63</v>
       </c>
@@ -2181,12 +1860,8 @@
         <f t="shared" si="0"/>
         <v>3Fh</v>
       </c>
-      <c r="D67" s="76"/>
-      <c r="E67" s="77"/>
-      <c r="F67" s="77"/>
-      <c r="G67" s="78"/>
-    </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B68" s="4">
         <v>64</v>
       </c>
@@ -2194,12 +1869,8 @@
         <f t="shared" si="0"/>
         <v>40h</v>
       </c>
-      <c r="D68" s="76"/>
-      <c r="E68" s="77"/>
-      <c r="F68" s="77"/>
-      <c r="G68" s="78"/>
-    </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B69" s="4">
         <v>65</v>
       </c>
@@ -2207,12 +1878,8 @@
         <f t="shared" ref="C69:C132" si="1">DEC2HEX(B69)&amp;"h"</f>
         <v>41h</v>
       </c>
-      <c r="D69" s="76"/>
-      <c r="E69" s="77"/>
-      <c r="F69" s="77"/>
-      <c r="G69" s="78"/>
-    </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B70" s="4">
         <v>66</v>
       </c>
@@ -2220,12 +1887,8 @@
         <f t="shared" si="1"/>
         <v>42h</v>
       </c>
-      <c r="D70" s="76"/>
-      <c r="E70" s="77"/>
-      <c r="F70" s="77"/>
-      <c r="G70" s="78"/>
-    </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B71" s="4">
         <v>67</v>
       </c>
@@ -2233,12 +1896,8 @@
         <f t="shared" si="1"/>
         <v>43h</v>
       </c>
-      <c r="D71" s="76"/>
-      <c r="E71" s="77"/>
-      <c r="F71" s="77"/>
-      <c r="G71" s="78"/>
-    </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B72" s="4">
         <v>68</v>
       </c>
@@ -2246,12 +1905,8 @@
         <f t="shared" si="1"/>
         <v>44h</v>
       </c>
-      <c r="D72" s="76"/>
-      <c r="E72" s="77"/>
-      <c r="F72" s="77"/>
-      <c r="G72" s="78"/>
-    </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B73" s="4">
         <v>69</v>
       </c>
@@ -2259,12 +1914,8 @@
         <f t="shared" si="1"/>
         <v>45h</v>
       </c>
-      <c r="D73" s="76"/>
-      <c r="E73" s="77"/>
-      <c r="F73" s="77"/>
-      <c r="G73" s="78"/>
-    </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B74" s="4">
         <v>70</v>
       </c>
@@ -2272,12 +1923,8 @@
         <f t="shared" si="1"/>
         <v>46h</v>
       </c>
-      <c r="D74" s="76"/>
-      <c r="E74" s="77"/>
-      <c r="F74" s="77"/>
-      <c r="G74" s="78"/>
-    </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B75" s="4">
         <v>71</v>
       </c>
@@ -2285,12 +1932,8 @@
         <f t="shared" si="1"/>
         <v>47h</v>
       </c>
-      <c r="D75" s="76"/>
-      <c r="E75" s="77"/>
-      <c r="F75" s="77"/>
-      <c r="G75" s="78"/>
-    </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B76" s="4">
         <v>72</v>
       </c>
@@ -2298,12 +1941,8 @@
         <f t="shared" si="1"/>
         <v>48h</v>
       </c>
-      <c r="D76" s="76"/>
-      <c r="E76" s="77"/>
-      <c r="F76" s="77"/>
-      <c r="G76" s="78"/>
-    </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B77" s="4">
         <v>73</v>
       </c>
@@ -2311,12 +1950,8 @@
         <f t="shared" si="1"/>
         <v>49h</v>
       </c>
-      <c r="D77" s="76"/>
-      <c r="E77" s="77"/>
-      <c r="F77" s="77"/>
-      <c r="G77" s="78"/>
-    </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B78" s="4">
         <v>74</v>
       </c>
@@ -2324,12 +1959,8 @@
         <f t="shared" si="1"/>
         <v>4Ah</v>
       </c>
-      <c r="D78" s="76"/>
-      <c r="E78" s="77"/>
-      <c r="F78" s="77"/>
-      <c r="G78" s="78"/>
-    </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B79" s="4">
         <v>75</v>
       </c>
@@ -2337,12 +1968,8 @@
         <f t="shared" si="1"/>
         <v>4Bh</v>
       </c>
-      <c r="D79" s="76"/>
-      <c r="E79" s="77"/>
-      <c r="F79" s="77"/>
-      <c r="G79" s="78"/>
-    </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B80" s="4">
         <v>76</v>
       </c>
@@ -2350,10 +1977,6 @@
         <f t="shared" si="1"/>
         <v>4Ch</v>
       </c>
-      <c r="D80" s="79"/>
-      <c r="E80" s="80"/>
-      <c r="F80" s="80"/>
-      <c r="G80" s="81"/>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B81" s="4">
@@ -2558,10 +2181,12 @@
         <f t="shared" si="1"/>
         <v>5Ch</v>
       </c>
-      <c r="D96" s="1"/>
-      <c r="E96" s="1"/>
-      <c r="F96" s="1"/>
-      <c r="G96" s="1"/>
+      <c r="D96" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="E96" s="33"/>
+      <c r="F96" s="33"/>
+      <c r="G96" s="33"/>
     </row>
     <row r="97" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B97" s="4">
@@ -2571,10 +2196,10 @@
         <f t="shared" si="1"/>
         <v>5Dh</v>
       </c>
-      <c r="D97" s="1"/>
-      <c r="E97" s="1"/>
-      <c r="F97" s="1"/>
-      <c r="G97" s="1"/>
+      <c r="D97" s="33"/>
+      <c r="E97" s="33"/>
+      <c r="F97" s="33"/>
+      <c r="G97" s="33"/>
     </row>
     <row r="98" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B98" s="4">
@@ -2584,10 +2209,10 @@
         <f t="shared" si="1"/>
         <v>5Eh</v>
       </c>
-      <c r="D98" s="1"/>
-      <c r="E98" s="1"/>
-      <c r="F98" s="1"/>
-      <c r="G98" s="1"/>
+      <c r="D98" s="33"/>
+      <c r="E98" s="33"/>
+      <c r="F98" s="33"/>
+      <c r="G98" s="33"/>
     </row>
     <row r="99" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B99" s="4">
@@ -2597,10 +2222,10 @@
         <f t="shared" si="1"/>
         <v>5Fh</v>
       </c>
-      <c r="D99" s="1"/>
-      <c r="E99" s="1"/>
-      <c r="F99" s="1"/>
-      <c r="G99" s="1"/>
+      <c r="D99" s="33"/>
+      <c r="E99" s="33"/>
+      <c r="F99" s="33"/>
+      <c r="G99" s="33"/>
     </row>
     <row r="100" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B100" s="4">
@@ -2610,10 +2235,10 @@
         <f t="shared" si="1"/>
         <v>60h</v>
       </c>
-      <c r="D100" s="1"/>
-      <c r="E100" s="1"/>
-      <c r="F100" s="1"/>
-      <c r="G100" s="1"/>
+      <c r="D100" s="33"/>
+      <c r="E100" s="33"/>
+      <c r="F100" s="33"/>
+      <c r="G100" s="33"/>
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B101" s="4">
@@ -2623,10 +2248,12 @@
         <f t="shared" si="1"/>
         <v>61h</v>
       </c>
-      <c r="D101" s="1"/>
-      <c r="E101" s="1"/>
-      <c r="F101" s="1"/>
-      <c r="G101" s="1"/>
+      <c r="D101" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="E101" s="35"/>
+      <c r="F101" s="35"/>
+      <c r="G101" s="35"/>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B102" s="4">
@@ -2636,10 +2263,10 @@
         <f t="shared" si="1"/>
         <v>62h</v>
       </c>
-      <c r="D102" s="1"/>
-      <c r="E102" s="1"/>
-      <c r="F102" s="1"/>
-      <c r="G102" s="1"/>
+      <c r="D102" s="35"/>
+      <c r="E102" s="35"/>
+      <c r="F102" s="35"/>
+      <c r="G102" s="35"/>
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B103" s="4">
@@ -2649,10 +2276,10 @@
         <f t="shared" si="1"/>
         <v>63h</v>
       </c>
-      <c r="D103" s="1"/>
-      <c r="E103" s="1"/>
-      <c r="F103" s="1"/>
-      <c r="G103" s="1"/>
+      <c r="D103" s="35"/>
+      <c r="E103" s="35"/>
+      <c r="F103" s="35"/>
+      <c r="G103" s="35"/>
     </row>
     <row r="104" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B104" s="4">
@@ -2662,10 +2289,10 @@
         <f t="shared" si="1"/>
         <v>64h</v>
       </c>
-      <c r="D104" s="1"/>
-      <c r="E104" s="1"/>
-      <c r="F104" s="1"/>
-      <c r="G104" s="1"/>
+      <c r="D104" s="35"/>
+      <c r="E104" s="35"/>
+      <c r="F104" s="35"/>
+      <c r="G104" s="35"/>
     </row>
     <row r="105" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B105" s="4">
@@ -2675,10 +2302,10 @@
         <f t="shared" si="1"/>
         <v>65h</v>
       </c>
-      <c r="D105" s="1"/>
-      <c r="E105" s="1"/>
-      <c r="F105" s="1"/>
-      <c r="G105" s="1"/>
+      <c r="D105" s="35"/>
+      <c r="E105" s="35"/>
+      <c r="F105" s="35"/>
+      <c r="G105" s="35"/>
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B106" s="4">
@@ -2688,10 +2315,12 @@
         <f t="shared" si="1"/>
         <v>66h</v>
       </c>
-      <c r="D106" s="1"/>
-      <c r="E106" s="1"/>
-      <c r="F106" s="1"/>
-      <c r="G106" s="1"/>
+      <c r="D106" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E106" s="36"/>
+      <c r="F106" s="36"/>
+      <c r="G106" s="36"/>
     </row>
     <row r="107" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B107" s="4">
@@ -2701,10 +2330,10 @@
         <f t="shared" si="1"/>
         <v>67h</v>
       </c>
-      <c r="D107" s="1"/>
-      <c r="E107" s="1"/>
-      <c r="F107" s="1"/>
-      <c r="G107" s="1"/>
+      <c r="D107" s="36"/>
+      <c r="E107" s="36"/>
+      <c r="F107" s="36"/>
+      <c r="G107" s="36"/>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B108" s="4">
@@ -2714,10 +2343,10 @@
         <f t="shared" si="1"/>
         <v>68h</v>
       </c>
-      <c r="D108" s="1"/>
-      <c r="E108" s="1"/>
-      <c r="F108" s="1"/>
-      <c r="G108" s="1"/>
+      <c r="D108" s="36"/>
+      <c r="E108" s="36"/>
+      <c r="F108" s="36"/>
+      <c r="G108" s="36"/>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B109" s="4">
@@ -2727,10 +2356,10 @@
         <f t="shared" si="1"/>
         <v>69h</v>
       </c>
-      <c r="D109" s="1"/>
-      <c r="E109" s="1"/>
-      <c r="F109" s="1"/>
-      <c r="G109" s="1"/>
+      <c r="D109" s="36"/>
+      <c r="E109" s="36"/>
+      <c r="F109" s="36"/>
+      <c r="G109" s="36"/>
     </row>
     <row r="110" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B110" s="4">
@@ -2740,10 +2369,10 @@
         <f t="shared" si="1"/>
         <v>6Ah</v>
       </c>
-      <c r="D110" s="1"/>
-      <c r="E110" s="1"/>
-      <c r="F110" s="1"/>
-      <c r="G110" s="1"/>
+      <c r="D110" s="36"/>
+      <c r="E110" s="36"/>
+      <c r="F110" s="36"/>
+      <c r="G110" s="36"/>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B111" s="4">
@@ -2753,10 +2382,12 @@
         <f t="shared" si="1"/>
         <v>6Bh</v>
       </c>
-      <c r="D111" s="1"/>
-      <c r="E111" s="1"/>
-      <c r="F111" s="1"/>
-      <c r="G111" s="1"/>
+      <c r="D111" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="E111" s="37"/>
+      <c r="F111" s="37"/>
+      <c r="G111" s="37"/>
     </row>
     <row r="112" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B112" s="4">
@@ -2766,10 +2397,10 @@
         <f t="shared" si="1"/>
         <v>6Ch</v>
       </c>
-      <c r="D112" s="1"/>
-      <c r="E112" s="1"/>
-      <c r="F112" s="1"/>
-      <c r="G112" s="1"/>
+      <c r="D112" s="37"/>
+      <c r="E112" s="37"/>
+      <c r="F112" s="37"/>
+      <c r="G112" s="37"/>
     </row>
     <row r="113" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B113" s="4">
@@ -2779,10 +2410,10 @@
         <f t="shared" si="1"/>
         <v>6Dh</v>
       </c>
-      <c r="D113" s="1"/>
-      <c r="E113" s="1"/>
-      <c r="F113" s="1"/>
-      <c r="G113" s="1"/>
+      <c r="D113" s="37"/>
+      <c r="E113" s="37"/>
+      <c r="F113" s="37"/>
+      <c r="G113" s="37"/>
     </row>
     <row r="114" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B114" s="4">
@@ -2792,10 +2423,10 @@
         <f t="shared" si="1"/>
         <v>6Eh</v>
       </c>
-      <c r="D114" s="1"/>
-      <c r="E114" s="1"/>
-      <c r="F114" s="1"/>
-      <c r="G114" s="1"/>
+      <c r="D114" s="37"/>
+      <c r="E114" s="37"/>
+      <c r="F114" s="37"/>
+      <c r="G114" s="37"/>
     </row>
     <row r="115" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B115" s="4">
@@ -2805,10 +2436,10 @@
         <f t="shared" si="1"/>
         <v>6Fh</v>
       </c>
-      <c r="D115" s="1"/>
-      <c r="E115" s="1"/>
-      <c r="F115" s="1"/>
-      <c r="G115" s="1"/>
+      <c r="D115" s="37"/>
+      <c r="E115" s="37"/>
+      <c r="F115" s="37"/>
+      <c r="G115" s="37"/>
     </row>
     <row r="116" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B116" s="4">
@@ -2818,10 +2449,12 @@
         <f t="shared" si="1"/>
         <v>70h</v>
       </c>
-      <c r="D116" s="1"/>
-      <c r="E116" s="1"/>
-      <c r="F116" s="1"/>
-      <c r="G116" s="1"/>
+      <c r="D116" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="E116" s="38"/>
+      <c r="F116" s="38"/>
+      <c r="G116" s="38"/>
     </row>
     <row r="117" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B117" s="4">
@@ -2831,10 +2464,10 @@
         <f t="shared" si="1"/>
         <v>71h</v>
       </c>
-      <c r="D117" s="1"/>
-      <c r="E117" s="1"/>
-      <c r="F117" s="1"/>
-      <c r="G117" s="1"/>
+      <c r="D117" s="38"/>
+      <c r="E117" s="38"/>
+      <c r="F117" s="38"/>
+      <c r="G117" s="38"/>
     </row>
     <row r="118" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B118" s="4">
@@ -2844,10 +2477,10 @@
         <f t="shared" si="1"/>
         <v>72h</v>
       </c>
-      <c r="D118" s="1"/>
-      <c r="E118" s="1"/>
-      <c r="F118" s="1"/>
-      <c r="G118" s="1"/>
+      <c r="D118" s="38"/>
+      <c r="E118" s="38"/>
+      <c r="F118" s="38"/>
+      <c r="G118" s="38"/>
     </row>
     <row r="119" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B119" s="4">
@@ -2857,10 +2490,10 @@
         <f t="shared" si="1"/>
         <v>73h</v>
       </c>
-      <c r="D119" s="1"/>
-      <c r="E119" s="1"/>
-      <c r="F119" s="1"/>
-      <c r="G119" s="1"/>
+      <c r="D119" s="38"/>
+      <c r="E119" s="38"/>
+      <c r="F119" s="38"/>
+      <c r="G119" s="38"/>
     </row>
     <row r="120" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B120" s="4">
@@ -2870,10 +2503,10 @@
         <f t="shared" si="1"/>
         <v>74h</v>
       </c>
-      <c r="D120" s="1"/>
-      <c r="E120" s="1"/>
-      <c r="F120" s="1"/>
-      <c r="G120" s="1"/>
+      <c r="D120" s="38"/>
+      <c r="E120" s="38"/>
+      <c r="F120" s="38"/>
+      <c r="G120" s="38"/>
     </row>
     <row r="121" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B121" s="4">
@@ -2883,10 +2516,10 @@
         <f t="shared" si="1"/>
         <v>75h</v>
       </c>
-      <c r="D121" s="1"/>
-      <c r="E121" s="1"/>
-      <c r="F121" s="1"/>
-      <c r="G121" s="1"/>
+      <c r="D121" s="38"/>
+      <c r="E121" s="38"/>
+      <c r="F121" s="38"/>
+      <c r="G121" s="38"/>
     </row>
     <row r="122" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B122" s="4">
@@ -2896,10 +2529,10 @@
         <f t="shared" si="1"/>
         <v>76h</v>
       </c>
-      <c r="D122" s="1"/>
-      <c r="E122" s="1"/>
-      <c r="F122" s="1"/>
-      <c r="G122" s="1"/>
+      <c r="D122" s="38"/>
+      <c r="E122" s="38"/>
+      <c r="F122" s="38"/>
+      <c r="G122" s="38"/>
     </row>
     <row r="123" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B123" s="4">
@@ -2909,10 +2542,10 @@
         <f t="shared" si="1"/>
         <v>77h</v>
       </c>
-      <c r="D123" s="1"/>
-      <c r="E123" s="1"/>
-      <c r="F123" s="1"/>
-      <c r="G123" s="1"/>
+      <c r="D123" s="38"/>
+      <c r="E123" s="38"/>
+      <c r="F123" s="38"/>
+      <c r="G123" s="38"/>
     </row>
     <row r="124" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B124" s="4">
@@ -2922,10 +2555,10 @@
         <f t="shared" si="1"/>
         <v>78h</v>
       </c>
-      <c r="D124" s="1"/>
-      <c r="E124" s="1"/>
-      <c r="F124" s="1"/>
-      <c r="G124" s="1"/>
+      <c r="D124" s="38"/>
+      <c r="E124" s="38"/>
+      <c r="F124" s="38"/>
+      <c r="G124" s="38"/>
     </row>
     <row r="125" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B125" s="4">
@@ -2935,10 +2568,10 @@
         <f t="shared" si="1"/>
         <v>79h</v>
       </c>
-      <c r="D125" s="1"/>
-      <c r="E125" s="1"/>
-      <c r="F125" s="1"/>
-      <c r="G125" s="1"/>
+      <c r="D125" s="38"/>
+      <c r="E125" s="38"/>
+      <c r="F125" s="38"/>
+      <c r="G125" s="38"/>
     </row>
     <row r="126" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B126" s="4">
@@ -2948,10 +2581,10 @@
         <f t="shared" si="1"/>
         <v>7Ah</v>
       </c>
-      <c r="D126" s="1"/>
-      <c r="E126" s="1"/>
-      <c r="F126" s="1"/>
-      <c r="G126" s="1"/>
+      <c r="D126" s="38"/>
+      <c r="E126" s="38"/>
+      <c r="F126" s="38"/>
+      <c r="G126" s="38"/>
     </row>
     <row r="127" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B127" s="4">
@@ -2961,10 +2594,10 @@
         <f t="shared" si="1"/>
         <v>7Bh</v>
       </c>
-      <c r="D127" s="1"/>
-      <c r="E127" s="1"/>
-      <c r="F127" s="1"/>
-      <c r="G127" s="1"/>
+      <c r="D127" s="38"/>
+      <c r="E127" s="38"/>
+      <c r="F127" s="38"/>
+      <c r="G127" s="38"/>
     </row>
     <row r="128" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B128" s="4">
@@ -2974,10 +2607,10 @@
         <f t="shared" si="1"/>
         <v>7Ch</v>
       </c>
-      <c r="D128" s="1"/>
-      <c r="E128" s="1"/>
-      <c r="F128" s="1"/>
-      <c r="G128" s="1"/>
+      <c r="D128" s="38"/>
+      <c r="E128" s="38"/>
+      <c r="F128" s="38"/>
+      <c r="G128" s="38"/>
     </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B129" s="4">
@@ -2987,10 +2620,10 @@
         <f t="shared" si="1"/>
         <v>7Dh</v>
       </c>
-      <c r="D129" s="1"/>
-      <c r="E129" s="1"/>
-      <c r="F129" s="1"/>
-      <c r="G129" s="1"/>
+      <c r="D129" s="38"/>
+      <c r="E129" s="38"/>
+      <c r="F129" s="38"/>
+      <c r="G129" s="38"/>
     </row>
     <row r="130" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B130" s="4">
@@ -3000,10 +2633,10 @@
         <f t="shared" si="1"/>
         <v>7Eh</v>
       </c>
-      <c r="D130" s="1"/>
-      <c r="E130" s="1"/>
-      <c r="F130" s="1"/>
-      <c r="G130" s="1"/>
+      <c r="D130" s="38"/>
+      <c r="E130" s="38"/>
+      <c r="F130" s="38"/>
+      <c r="G130" s="38"/>
     </row>
     <row r="131" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B131" s="4">
@@ -3013,10 +2646,10 @@
         <f t="shared" si="1"/>
         <v>7Fh</v>
       </c>
-      <c r="D131" s="1"/>
-      <c r="E131" s="1"/>
-      <c r="F131" s="1"/>
-      <c r="G131" s="1"/>
+      <c r="D131" s="38"/>
+      <c r="E131" s="38"/>
+      <c r="F131" s="38"/>
+      <c r="G131" s="38"/>
     </row>
     <row r="132" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B132" s="4">
@@ -3026,10 +2659,10 @@
         <f t="shared" si="1"/>
         <v>80h</v>
       </c>
-      <c r="D132" s="1"/>
-      <c r="E132" s="1"/>
-      <c r="F132" s="1"/>
-      <c r="G132" s="1"/>
+      <c r="D132" s="38"/>
+      <c r="E132" s="38"/>
+      <c r="F132" s="38"/>
+      <c r="G132" s="38"/>
     </row>
     <row r="133" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B133" s="4">
@@ -3039,10 +2672,10 @@
         <f t="shared" ref="C133:C138" si="2">DEC2HEX(B133)&amp;"h"</f>
         <v>81h</v>
       </c>
-      <c r="D133" s="1"/>
-      <c r="E133" s="1"/>
-      <c r="F133" s="1"/>
-      <c r="G133" s="1"/>
+      <c r="D133" s="38"/>
+      <c r="E133" s="38"/>
+      <c r="F133" s="38"/>
+      <c r="G133" s="38"/>
     </row>
     <row r="134" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B134" s="4">
@@ -3052,14 +2685,10 @@
         <f t="shared" si="2"/>
         <v>82h</v>
       </c>
-      <c r="D134" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="E134" s="23"/>
-      <c r="F134" s="24"/>
-      <c r="G134" s="20" t="s">
-        <v>29</v>
-      </c>
+      <c r="D134" s="38"/>
+      <c r="E134" s="38"/>
+      <c r="F134" s="38"/>
+      <c r="G134" s="38"/>
     </row>
     <row r="135" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B135" s="4">
@@ -3069,12 +2698,10 @@
         <f t="shared" si="2"/>
         <v>83h</v>
       </c>
-      <c r="D135" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="E135" s="27"/>
-      <c r="F135" s="27"/>
-      <c r="G135" s="26"/>
+      <c r="D135" s="38"/>
+      <c r="E135" s="38"/>
+      <c r="F135" s="38"/>
+      <c r="G135" s="38"/>
     </row>
     <row r="136" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B136" s="4">
@@ -3084,12 +2711,10 @@
         <f t="shared" si="2"/>
         <v>84h</v>
       </c>
-      <c r="D136" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="E136" s="27"/>
-      <c r="F136" s="27"/>
-      <c r="G136" s="26"/>
+      <c r="D136" s="38"/>
+      <c r="E136" s="38"/>
+      <c r="F136" s="38"/>
+      <c r="G136" s="38"/>
     </row>
     <row r="137" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B137" s="4">
@@ -3099,12 +2724,10 @@
         <f t="shared" si="2"/>
         <v>85h</v>
       </c>
-      <c r="D137" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="E137" s="27"/>
-      <c r="F137" s="27"/>
-      <c r="G137" s="26"/>
+      <c r="D137" s="38"/>
+      <c r="E137" s="38"/>
+      <c r="F137" s="38"/>
+      <c r="G137" s="38"/>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B138" s="4">
@@ -3114,37 +2737,123 @@
         <f t="shared" si="2"/>
         <v>86h</v>
       </c>
-      <c r="D138" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="E138" s="26"/>
-      <c r="F138" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="G138" s="26"/>
+      <c r="D138" s="38"/>
+      <c r="E138" s="38"/>
+      <c r="F138" s="38"/>
+      <c r="G138" s="38"/>
+    </row>
+    <row r="139" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D139" s="38"/>
+      <c r="E139" s="38"/>
+      <c r="F139" s="38"/>
+      <c r="G139" s="38"/>
+    </row>
+    <row r="140" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D140" s="38"/>
+      <c r="E140" s="38"/>
+      <c r="F140" s="38"/>
+      <c r="G140" s="38"/>
+    </row>
+    <row r="141" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D141" s="38"/>
+      <c r="E141" s="38"/>
+      <c r="F141" s="38"/>
+      <c r="G141" s="38"/>
+    </row>
+    <row r="142" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D142" s="38"/>
+      <c r="E142" s="38"/>
+      <c r="F142" s="38"/>
+      <c r="G142" s="38"/>
+    </row>
+    <row r="143" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D143" s="38"/>
+      <c r="E143" s="38"/>
+      <c r="F143" s="38"/>
+      <c r="G143" s="38"/>
+    </row>
+    <row r="144" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D144" s="38"/>
+      <c r="E144" s="38"/>
+      <c r="F144" s="38"/>
+      <c r="G144" s="38"/>
+    </row>
+    <row r="145" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D145" s="38"/>
+      <c r="E145" s="38"/>
+      <c r="F145" s="38"/>
+      <c r="G145" s="38"/>
+    </row>
+    <row r="146" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D146" s="38"/>
+      <c r="E146" s="38"/>
+      <c r="F146" s="38"/>
+      <c r="G146" s="38"/>
+    </row>
+    <row r="147" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D147" s="38"/>
+      <c r="E147" s="38"/>
+      <c r="F147" s="38"/>
+      <c r="G147" s="38"/>
+    </row>
+    <row r="148" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D148" s="38"/>
+      <c r="E148" s="38"/>
+      <c r="F148" s="38"/>
+      <c r="G148" s="38"/>
+    </row>
+    <row r="149" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D149" s="38"/>
+      <c r="E149" s="38"/>
+      <c r="F149" s="38"/>
+      <c r="G149" s="38"/>
+    </row>
+    <row r="150" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D150" s="38"/>
+      <c r="E150" s="38"/>
+      <c r="F150" s="38"/>
+      <c r="G150" s="38"/>
+    </row>
+    <row r="151" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D151" s="38"/>
+      <c r="E151" s="38"/>
+      <c r="F151" s="38"/>
+      <c r="G151" s="38"/>
+    </row>
+    <row r="152" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D152" s="38"/>
+      <c r="E152" s="38"/>
+      <c r="F152" s="38"/>
+      <c r="G152" s="38"/>
+    </row>
+    <row r="153" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D153" s="38"/>
+      <c r="E153" s="38"/>
+      <c r="F153" s="38"/>
+      <c r="G153" s="38"/>
+    </row>
+    <row r="154" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D154" s="38"/>
+      <c r="E154" s="38"/>
+      <c r="F154" s="38"/>
+      <c r="G154" s="38"/>
+    </row>
+    <row r="155" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D155" s="38"/>
+      <c r="E155" s="38"/>
+      <c r="F155" s="38"/>
+      <c r="G155" s="38"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="D41:G80"/>
+  <mergeCells count="5">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="D4:G5"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="D7:G7"/>
-    <mergeCell ref="D8:G20"/>
-    <mergeCell ref="D31:G35"/>
-    <mergeCell ref="D21:G25"/>
-    <mergeCell ref="D26:G30"/>
-    <mergeCell ref="D36:G40"/>
-    <mergeCell ref="D134:F134"/>
-    <mergeCell ref="D138:E138"/>
-    <mergeCell ref="F138:G138"/>
-    <mergeCell ref="D135:G135"/>
-    <mergeCell ref="D136:G136"/>
-    <mergeCell ref="D137:G137"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K10" r:id="rId1" xr:uid="{4CDEDA9D-6A17-4E55-8BF2-30A318687126}"/>
+    <hyperlink ref="K21" r:id="rId1" xr:uid="{4CDEDA9D-6A17-4E55-8BF2-30A318687126}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
@@ -3152,15 +2861,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100428D6099D6E2B6448E8A88B2B567960C" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="d06e3c45a3f093fe91a85c3d3a514f99">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="602d6013-12bf-42a7-bc7f-2fade0e82371" xmlns:ns4="98306238-8ebe-44ab-acf1-12aa768c5e84" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="892bbdd5d735959505dc654187d2f43d" ns3:_="" ns4:_="">
     <xsd:import namespace="602d6013-12bf-42a7-bc7f-2fade0e82371"/>
@@ -3355,6 +3055,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3364,14 +3073,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AF9C2AB-D531-4B8D-9A76-F0FAB1D11F28}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3386,6 +3087,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Started the process of adding a GUI using Qt
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/wh40k_NTAG215_memoryMapping.xlsx
+++ b/wh40k_NTAG215_memoryMapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fuzzy\wh40k_nfc_project\wh40k_nfc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03717F51-B96D-431E-AA05-9B9B2C78FE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11917E0-1425-4A83-999D-A0238B3370AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
   <si>
     <t>NTAG215</t>
   </si>
@@ -532,6 +532,32 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -568,32 +594,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -986,7 +986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E22B5351-43EC-4BE6-A109-53A8CF40F7FA}">
-  <dimension ref="A1:K155"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="18.90625" customWidth="1"/>
@@ -1002,16 +1002,16 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="22"/>
-      <c r="D2" s="23" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="25"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="39"/>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="2" t="s">
@@ -1041,12 +1041,12 @@
         <f>DEC2HEX(B4)&amp;"h"</f>
         <v>0h</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
       <c r="J4" t="s">
         <v>31</v>
       </c>
@@ -1059,10 +1059,10 @@
         <f t="shared" ref="C5:C68" si="0">DEC2HEX(B5)&amp;"h"</f>
         <v>1h</v>
       </c>
-      <c r="D5" s="27"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
       <c r="I5" s="6" t="s">
         <v>10</v>
       </c>
@@ -1082,10 +1082,10 @@
       <c r="E6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="28" t="s">
+      <c r="F6" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="29"/>
+      <c r="G6" s="43"/>
       <c r="I6" s="11" t="s">
         <v>28</v>
       </c>
@@ -1104,12 +1104,12 @@
         <f t="shared" si="0"/>
         <v>3h</v>
       </c>
-      <c r="D7" s="30" t="s">
+      <c r="D7" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="31"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="32"/>
+      <c r="E7" s="45"/>
+      <c r="F7" s="45"/>
+      <c r="G7" s="46"/>
       <c r="I7" s="18" t="s">
         <v>8</v>
       </c>
@@ -1125,20 +1125,20 @@
         <f t="shared" si="0"/>
         <v>4h</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="44" t="s">
+      <c r="E8" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="45" t="s">
+      <c r="F8" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="G8" s="43"/>
-      <c r="I8" s="39" t="s">
+      <c r="G8" s="31"/>
+      <c r="I8" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="27">
         <v>1</v>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
         <f t="shared" si="0"/>
         <v>5h</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="29" t="s">
         <v>17</v>
       </c>
       <c r="E9" s="13" t="s">
@@ -1159,10 +1159,10 @@
       <c r="F9" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="42" t="s">
+      <c r="G9" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="44" t="s">
+      <c r="I9" s="32" t="s">
         <v>41</v>
       </c>
       <c r="J9">
@@ -1177,13 +1177,13 @@
         <f t="shared" si="0"/>
         <v>6h</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="34" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="46"/>
-      <c r="F10" s="46"/>
-      <c r="G10" s="46"/>
-      <c r="I10" s="45" t="s">
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="I10" s="33" t="s">
         <v>42</v>
       </c>
       <c r="J10">
@@ -1198,16 +1198,16 @@
         <f t="shared" si="0"/>
         <v>7h</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="I11" s="43" t="s">
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="I11" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="31">
         <v>5</v>
       </c>
     </row>
@@ -1219,10 +1219,10 @@
         <f t="shared" si="0"/>
         <v>8h</v>
       </c>
-      <c r="D12" s="34"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B13" s="4">
@@ -1232,10 +1232,10 @@
         <f t="shared" si="0"/>
         <v>9h</v>
       </c>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B14" s="4">
@@ -1245,10 +1245,10 @@
         <f t="shared" si="0"/>
         <v>Ah</v>
       </c>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B15" s="4">
@@ -1258,10 +1258,10 @@
         <f t="shared" si="0"/>
         <v>Bh</v>
       </c>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
       <c r="I15" s="12" t="s">
         <v>9</v>
       </c>
@@ -1280,14 +1280,14 @@
         <f t="shared" si="0"/>
         <v>Ch</v>
       </c>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="I16" s="41" t="s">
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="I16" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="J16" s="41">
+      <c r="J16" s="29">
         <v>1</v>
       </c>
       <c r="K16" t="s">
@@ -1302,10 +1302,10 @@
         <f t="shared" si="0"/>
         <v>Dh</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
       <c r="I17" s="13" t="s">
         <v>18</v>
       </c>
@@ -1324,10 +1324,10 @@
         <f t="shared" si="0"/>
         <v>Eh</v>
       </c>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
       <c r="I18" s="14" t="s">
         <v>15</v>
       </c>
@@ -1346,10 +1346,10 @@
         <f t="shared" si="0"/>
         <v>Fh</v>
       </c>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
       <c r="I19" s="15" t="s">
         <v>16</v>
       </c>
@@ -1368,14 +1368,14 @@
         <f t="shared" si="0"/>
         <v>10h</v>
       </c>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="I20" s="43" t="s">
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="I20" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="J20" s="43">
+      <c r="J20" s="31">
         <v>4</v>
       </c>
     </row>
@@ -1387,10 +1387,10 @@
         <f t="shared" si="0"/>
         <v>11h</v>
       </c>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
       <c r="I21" s="17" t="s">
         <v>20</v>
       </c>
@@ -1409,10 +1409,10 @@
         <f t="shared" si="0"/>
         <v>12h</v>
       </c>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
       <c r="K22" t="s">
         <v>21</v>
       </c>
@@ -1425,10 +1425,10 @@
         <f t="shared" si="0"/>
         <v>13h</v>
       </c>
-      <c r="D23" s="34"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="22"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
       <c r="K23" t="s">
         <v>22</v>
       </c>
@@ -1441,6 +1441,12 @@
         <f t="shared" si="0"/>
         <v>14h</v>
       </c>
+      <c r="D24" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
       <c r="I24" s="19" t="s">
         <v>29</v>
       </c>
@@ -1456,12 +1462,10 @@
         <f t="shared" si="0"/>
         <v>15h</v>
       </c>
-      <c r="D25" s="43" t="s">
-        <v>38</v>
-      </c>
-      <c r="E25" s="43"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="43"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
       <c r="I25" s="20" t="s">
         <v>30</v>
       </c>
@@ -1477,6 +1481,10 @@
         <f t="shared" si="0"/>
         <v>16h</v>
       </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B27" s="4">
@@ -1486,6 +1494,10 @@
         <f t="shared" si="0"/>
         <v>17h</v>
       </c>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
       <c r="I27" t="s">
         <v>32</v>
       </c>
@@ -1502,6 +1514,10 @@
         <f t="shared" si="0"/>
         <v>18h</v>
       </c>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
       <c r="I28" t="s">
         <v>33</v>
       </c>
@@ -1518,6 +1534,12 @@
         <f t="shared" si="0"/>
         <v>19h</v>
       </c>
+      <c r="D29" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B30" s="4">
@@ -1527,6 +1549,10 @@
         <f t="shared" si="0"/>
         <v>1Ah</v>
       </c>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B31" s="4">
@@ -1536,6 +1562,10 @@
         <f t="shared" si="0"/>
         <v>1Bh</v>
       </c>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B32" s="4">
@@ -1545,8 +1575,12 @@
         <f t="shared" si="0"/>
         <v>1Ch</v>
       </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="23"/>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B33" s="4">
         <v>29</v>
       </c>
@@ -1554,8 +1588,12 @@
         <f t="shared" si="0"/>
         <v>1Dh</v>
       </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B34" s="4">
         <v>30</v>
       </c>
@@ -1563,8 +1601,14 @@
         <f t="shared" si="0"/>
         <v>1Eh</v>
       </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D34" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B35" s="4">
         <v>31</v>
       </c>
@@ -1572,8 +1616,12 @@
         <f t="shared" si="0"/>
         <v>1Fh</v>
       </c>
-    </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B36" s="4">
         <v>32</v>
       </c>
@@ -1581,8 +1629,12 @@
         <f t="shared" si="0"/>
         <v>20h</v>
       </c>
-    </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B37" s="4">
         <v>33</v>
       </c>
@@ -1590,8 +1642,12 @@
         <f t="shared" si="0"/>
         <v>21h</v>
       </c>
-    </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B38" s="4">
         <v>34</v>
       </c>
@@ -1599,8 +1655,12 @@
         <f t="shared" si="0"/>
         <v>22h</v>
       </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B39" s="4">
         <v>35</v>
       </c>
@@ -1608,8 +1668,14 @@
         <f t="shared" si="0"/>
         <v>23h</v>
       </c>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D39" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25"/>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B40" s="4">
         <v>36</v>
       </c>
@@ -1617,8 +1683,12 @@
         <f t="shared" si="0"/>
         <v>24h</v>
       </c>
-    </row>
-    <row r="41" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D40" s="25"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="25"/>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B41" s="4">
         <v>37</v>
       </c>
@@ -1626,8 +1696,12 @@
         <f t="shared" si="0"/>
         <v>25h</v>
       </c>
-    </row>
-    <row r="42" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D41" s="25"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="25"/>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B42" s="4">
         <v>38</v>
       </c>
@@ -1635,8 +1709,12 @@
         <f t="shared" si="0"/>
         <v>26h</v>
       </c>
-    </row>
-    <row r="43" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B43" s="4">
         <v>39</v>
       </c>
@@ -1644,8 +1722,12 @@
         <f t="shared" si="0"/>
         <v>27h</v>
       </c>
-    </row>
-    <row r="44" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D43" s="25"/>
+      <c r="E43" s="25"/>
+      <c r="F43" s="25"/>
+      <c r="G43" s="25"/>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B44" s="4">
         <v>40</v>
       </c>
@@ -1653,8 +1735,14 @@
         <f t="shared" si="0"/>
         <v>28h</v>
       </c>
-    </row>
-    <row r="45" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D44" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="E44" s="26"/>
+      <c r="F44" s="26"/>
+      <c r="G44" s="26"/>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B45" s="4">
         <v>41</v>
       </c>
@@ -1662,8 +1750,12 @@
         <f t="shared" si="0"/>
         <v>29h</v>
       </c>
-    </row>
-    <row r="46" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D45" s="26"/>
+      <c r="E45" s="26"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="26"/>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B46" s="4">
         <v>42</v>
       </c>
@@ -1671,8 +1763,12 @@
         <f t="shared" si="0"/>
         <v>2Ah</v>
       </c>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B47" s="4">
         <v>43</v>
       </c>
@@ -1680,8 +1776,12 @@
         <f t="shared" si="0"/>
         <v>2Bh</v>
       </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D47" s="26"/>
+      <c r="E47" s="26"/>
+      <c r="F47" s="26"/>
+      <c r="G47" s="26"/>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B48" s="4">
         <v>44</v>
       </c>
@@ -1689,8 +1789,12 @@
         <f t="shared" si="0"/>
         <v>2Ch</v>
       </c>
-    </row>
-    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="26"/>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B49" s="4">
         <v>45</v>
       </c>
@@ -1698,8 +1802,12 @@
         <f t="shared" si="0"/>
         <v>2Dh</v>
       </c>
-    </row>
-    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D49" s="26"/>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26"/>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B50" s="4">
         <v>46</v>
       </c>
@@ -1707,8 +1815,12 @@
         <f t="shared" si="0"/>
         <v>2Eh</v>
       </c>
-    </row>
-    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D50" s="26"/>
+      <c r="E50" s="26"/>
+      <c r="F50" s="26"/>
+      <c r="G50" s="26"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B51" s="4">
         <v>47</v>
       </c>
@@ -1716,8 +1828,12 @@
         <f t="shared" si="0"/>
         <v>2Fh</v>
       </c>
-    </row>
-    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D51" s="26"/>
+      <c r="E51" s="26"/>
+      <c r="F51" s="26"/>
+      <c r="G51" s="26"/>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B52" s="4">
         <v>48</v>
       </c>
@@ -1725,8 +1841,12 @@
         <f t="shared" si="0"/>
         <v>30h</v>
       </c>
-    </row>
-    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D52" s="26"/>
+      <c r="E52" s="26"/>
+      <c r="F52" s="26"/>
+      <c r="G52" s="26"/>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B53" s="4">
         <v>49</v>
       </c>
@@ -1734,8 +1854,12 @@
         <f t="shared" si="0"/>
         <v>31h</v>
       </c>
-    </row>
-    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D53" s="26"/>
+      <c r="E53" s="26"/>
+      <c r="F53" s="26"/>
+      <c r="G53" s="26"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B54" s="4">
         <v>50</v>
       </c>
@@ -1743,8 +1867,12 @@
         <f t="shared" si="0"/>
         <v>32h</v>
       </c>
-    </row>
-    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D54" s="26"/>
+      <c r="E54" s="26"/>
+      <c r="F54" s="26"/>
+      <c r="G54" s="26"/>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B55" s="4">
         <v>51</v>
       </c>
@@ -1752,8 +1880,12 @@
         <f t="shared" si="0"/>
         <v>33h</v>
       </c>
-    </row>
-    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D55" s="26"/>
+      <c r="E55" s="26"/>
+      <c r="F55" s="26"/>
+      <c r="G55" s="26"/>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B56" s="4">
         <v>52</v>
       </c>
@@ -1761,8 +1893,12 @@
         <f t="shared" si="0"/>
         <v>34h</v>
       </c>
-    </row>
-    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D56" s="26"/>
+      <c r="E56" s="26"/>
+      <c r="F56" s="26"/>
+      <c r="G56" s="26"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B57" s="4">
         <v>53</v>
       </c>
@@ -1770,8 +1906,12 @@
         <f t="shared" si="0"/>
         <v>35h</v>
       </c>
-    </row>
-    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D57" s="26"/>
+      <c r="E57" s="26"/>
+      <c r="F57" s="26"/>
+      <c r="G57" s="26"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B58" s="4">
         <v>54</v>
       </c>
@@ -1779,8 +1919,12 @@
         <f t="shared" si="0"/>
         <v>36h</v>
       </c>
-    </row>
-    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D58" s="26"/>
+      <c r="E58" s="26"/>
+      <c r="F58" s="26"/>
+      <c r="G58" s="26"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B59" s="4">
         <v>55</v>
       </c>
@@ -1788,8 +1932,12 @@
         <f t="shared" si="0"/>
         <v>37h</v>
       </c>
-    </row>
-    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D59" s="26"/>
+      <c r="E59" s="26"/>
+      <c r="F59" s="26"/>
+      <c r="G59" s="26"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B60" s="4">
         <v>56</v>
       </c>
@@ -1797,8 +1945,12 @@
         <f t="shared" si="0"/>
         <v>38h</v>
       </c>
-    </row>
-    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D60" s="26"/>
+      <c r="E60" s="26"/>
+      <c r="F60" s="26"/>
+      <c r="G60" s="26"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B61" s="4">
         <v>57</v>
       </c>
@@ -1806,8 +1958,12 @@
         <f t="shared" si="0"/>
         <v>39h</v>
       </c>
-    </row>
-    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D61" s="26"/>
+      <c r="E61" s="26"/>
+      <c r="F61" s="26"/>
+      <c r="G61" s="26"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B62" s="4">
         <v>58</v>
       </c>
@@ -1815,8 +1971,12 @@
         <f t="shared" si="0"/>
         <v>3Ah</v>
       </c>
-    </row>
-    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D62" s="26"/>
+      <c r="E62" s="26"/>
+      <c r="F62" s="26"/>
+      <c r="G62" s="26"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B63" s="4">
         <v>59</v>
       </c>
@@ -1824,8 +1984,12 @@
         <f t="shared" si="0"/>
         <v>3Bh</v>
       </c>
-    </row>
-    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D63" s="26"/>
+      <c r="E63" s="26"/>
+      <c r="F63" s="26"/>
+      <c r="G63" s="26"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B64" s="4">
         <v>60</v>
       </c>
@@ -1833,8 +1997,12 @@
         <f t="shared" si="0"/>
         <v>3Ch</v>
       </c>
-    </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D64" s="26"/>
+      <c r="E64" s="26"/>
+      <c r="F64" s="26"/>
+      <c r="G64" s="26"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B65" s="4">
         <v>61</v>
       </c>
@@ -1842,8 +2010,12 @@
         <f t="shared" si="0"/>
         <v>3Dh</v>
       </c>
-    </row>
-    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D65" s="26"/>
+      <c r="E65" s="26"/>
+      <c r="F65" s="26"/>
+      <c r="G65" s="26"/>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B66" s="4">
         <v>62</v>
       </c>
@@ -1851,8 +2023,12 @@
         <f t="shared" si="0"/>
         <v>3Eh</v>
       </c>
-    </row>
-    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D66" s="26"/>
+      <c r="E66" s="26"/>
+      <c r="F66" s="26"/>
+      <c r="G66" s="26"/>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B67" s="4">
         <v>63</v>
       </c>
@@ -1860,8 +2036,12 @@
         <f t="shared" si="0"/>
         <v>3Fh</v>
       </c>
-    </row>
-    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D67" s="26"/>
+      <c r="E67" s="26"/>
+      <c r="F67" s="26"/>
+      <c r="G67" s="26"/>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B68" s="4">
         <v>64</v>
       </c>
@@ -1869,8 +2049,12 @@
         <f t="shared" si="0"/>
         <v>40h</v>
       </c>
-    </row>
-    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D68" s="26"/>
+      <c r="E68" s="26"/>
+      <c r="F68" s="26"/>
+      <c r="G68" s="26"/>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B69" s="4">
         <v>65</v>
       </c>
@@ -1878,8 +2062,12 @@
         <f t="shared" ref="C69:C132" si="1">DEC2HEX(B69)&amp;"h"</f>
         <v>41h</v>
       </c>
-    </row>
-    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D69" s="26"/>
+      <c r="E69" s="26"/>
+      <c r="F69" s="26"/>
+      <c r="G69" s="26"/>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B70" s="4">
         <v>66</v>
       </c>
@@ -1887,8 +2075,12 @@
         <f t="shared" si="1"/>
         <v>42h</v>
       </c>
-    </row>
-    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D70" s="26"/>
+      <c r="E70" s="26"/>
+      <c r="F70" s="26"/>
+      <c r="G70" s="26"/>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B71" s="4">
         <v>67</v>
       </c>
@@ -1896,8 +2088,12 @@
         <f t="shared" si="1"/>
         <v>43h</v>
       </c>
-    </row>
-    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D71" s="26"/>
+      <c r="E71" s="26"/>
+      <c r="F71" s="26"/>
+      <c r="G71" s="26"/>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B72" s="4">
         <v>68</v>
       </c>
@@ -1905,8 +2101,12 @@
         <f t="shared" si="1"/>
         <v>44h</v>
       </c>
-    </row>
-    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D72" s="26"/>
+      <c r="E72" s="26"/>
+      <c r="F72" s="26"/>
+      <c r="G72" s="26"/>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B73" s="4">
         <v>69</v>
       </c>
@@ -1914,8 +2114,12 @@
         <f t="shared" si="1"/>
         <v>45h</v>
       </c>
-    </row>
-    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D73" s="26"/>
+      <c r="E73" s="26"/>
+      <c r="F73" s="26"/>
+      <c r="G73" s="26"/>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B74" s="4">
         <v>70</v>
       </c>
@@ -1923,8 +2127,12 @@
         <f t="shared" si="1"/>
         <v>46h</v>
       </c>
-    </row>
-    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D74" s="26"/>
+      <c r="E74" s="26"/>
+      <c r="F74" s="26"/>
+      <c r="G74" s="26"/>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B75" s="4">
         <v>71</v>
       </c>
@@ -1932,8 +2140,12 @@
         <f t="shared" si="1"/>
         <v>47h</v>
       </c>
-    </row>
-    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D75" s="26"/>
+      <c r="E75" s="26"/>
+      <c r="F75" s="26"/>
+      <c r="G75" s="26"/>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B76" s="4">
         <v>72</v>
       </c>
@@ -1941,8 +2153,12 @@
         <f t="shared" si="1"/>
         <v>48h</v>
       </c>
-    </row>
-    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D76" s="26"/>
+      <c r="E76" s="26"/>
+      <c r="F76" s="26"/>
+      <c r="G76" s="26"/>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B77" s="4">
         <v>73</v>
       </c>
@@ -1950,8 +2166,12 @@
         <f t="shared" si="1"/>
         <v>49h</v>
       </c>
-    </row>
-    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D77" s="26"/>
+      <c r="E77" s="26"/>
+      <c r="F77" s="26"/>
+      <c r="G77" s="26"/>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B78" s="4">
         <v>74</v>
       </c>
@@ -1959,8 +2179,12 @@
         <f t="shared" si="1"/>
         <v>4Ah</v>
       </c>
-    </row>
-    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D78" s="26"/>
+      <c r="E78" s="26"/>
+      <c r="F78" s="26"/>
+      <c r="G78" s="26"/>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B79" s="4">
         <v>75</v>
       </c>
@@ -1968,8 +2192,12 @@
         <f t="shared" si="1"/>
         <v>4Bh</v>
       </c>
-    </row>
-    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="D79" s="26"/>
+      <c r="E79" s="26"/>
+      <c r="F79" s="26"/>
+      <c r="G79" s="26"/>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B80" s="4">
         <v>76</v>
       </c>
@@ -1977,6 +2205,10 @@
         <f t="shared" si="1"/>
         <v>4Ch</v>
       </c>
+      <c r="D80" s="26"/>
+      <c r="E80" s="26"/>
+      <c r="F80" s="26"/>
+      <c r="G80" s="26"/>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B81" s="4">
@@ -1986,10 +2218,10 @@
         <f t="shared" si="1"/>
         <v>4Dh</v>
       </c>
-      <c r="D81" s="1"/>
-      <c r="E81" s="1"/>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
+      <c r="D81" s="26"/>
+      <c r="E81" s="26"/>
+      <c r="F81" s="26"/>
+      <c r="G81" s="26"/>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B82" s="4">
@@ -1999,10 +2231,10 @@
         <f t="shared" si="1"/>
         <v>4Eh</v>
       </c>
-      <c r="D82" s="1"/>
-      <c r="E82" s="1"/>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
+      <c r="D82" s="26"/>
+      <c r="E82" s="26"/>
+      <c r="F82" s="26"/>
+      <c r="G82" s="26"/>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B83" s="4">
@@ -2012,10 +2244,10 @@
         <f t="shared" si="1"/>
         <v>4Fh</v>
       </c>
-      <c r="D83" s="1"/>
-      <c r="E83" s="1"/>
-      <c r="F83" s="1"/>
-      <c r="G83" s="1"/>
+      <c r="D83" s="26"/>
+      <c r="E83" s="26"/>
+      <c r="F83" s="26"/>
+      <c r="G83" s="26"/>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B84" s="4">
@@ -2181,14 +2413,8 @@
         <f t="shared" si="1"/>
         <v>5Ch</v>
       </c>
-      <c r="D96" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="E96" s="33"/>
-      <c r="F96" s="33"/>
-      <c r="G96" s="33"/>
-    </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B97" s="4">
         <v>93</v>
       </c>
@@ -2196,12 +2422,8 @@
         <f t="shared" si="1"/>
         <v>5Dh</v>
       </c>
-      <c r="D97" s="33"/>
-      <c r="E97" s="33"/>
-      <c r="F97" s="33"/>
-      <c r="G97" s="33"/>
-    </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B98" s="4">
         <v>94</v>
       </c>
@@ -2209,12 +2431,8 @@
         <f t="shared" si="1"/>
         <v>5Eh</v>
       </c>
-      <c r="D98" s="33"/>
-      <c r="E98" s="33"/>
-      <c r="F98" s="33"/>
-      <c r="G98" s="33"/>
-    </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B99" s="4">
         <v>95</v>
       </c>
@@ -2222,12 +2440,8 @@
         <f t="shared" si="1"/>
         <v>5Fh</v>
       </c>
-      <c r="D99" s="33"/>
-      <c r="E99" s="33"/>
-      <c r="F99" s="33"/>
-      <c r="G99" s="33"/>
-    </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B100" s="4">
         <v>96</v>
       </c>
@@ -2235,12 +2449,8 @@
         <f t="shared" si="1"/>
         <v>60h</v>
       </c>
-      <c r="D100" s="33"/>
-      <c r="E100" s="33"/>
-      <c r="F100" s="33"/>
-      <c r="G100" s="33"/>
-    </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B101" s="4">
         <v>97</v>
       </c>
@@ -2248,14 +2458,8 @@
         <f t="shared" si="1"/>
         <v>61h</v>
       </c>
-      <c r="D101" s="35" t="s">
-        <v>18</v>
-      </c>
-      <c r="E101" s="35"/>
-      <c r="F101" s="35"/>
-      <c r="G101" s="35"/>
-    </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B102" s="4">
         <v>98</v>
       </c>
@@ -2263,12 +2467,8 @@
         <f t="shared" si="1"/>
         <v>62h</v>
       </c>
-      <c r="D102" s="35"/>
-      <c r="E102" s="35"/>
-      <c r="F102" s="35"/>
-      <c r="G102" s="35"/>
-    </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B103" s="4">
         <v>99</v>
       </c>
@@ -2276,12 +2476,8 @@
         <f t="shared" si="1"/>
         <v>63h</v>
       </c>
-      <c r="D103" s="35"/>
-      <c r="E103" s="35"/>
-      <c r="F103" s="35"/>
-      <c r="G103" s="35"/>
-    </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B104" s="4">
         <v>100</v>
       </c>
@@ -2289,12 +2485,8 @@
         <f t="shared" si="1"/>
         <v>64h</v>
       </c>
-      <c r="D104" s="35"/>
-      <c r="E104" s="35"/>
-      <c r="F104" s="35"/>
-      <c r="G104" s="35"/>
-    </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B105" s="4">
         <v>101</v>
       </c>
@@ -2302,12 +2494,8 @@
         <f t="shared" si="1"/>
         <v>65h</v>
       </c>
-      <c r="D105" s="35"/>
-      <c r="E105" s="35"/>
-      <c r="F105" s="35"/>
-      <c r="G105" s="35"/>
-    </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B106" s="4">
         <v>102</v>
       </c>
@@ -2315,14 +2503,8 @@
         <f t="shared" si="1"/>
         <v>66h</v>
       </c>
-      <c r="D106" s="36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E106" s="36"/>
-      <c r="F106" s="36"/>
-      <c r="G106" s="36"/>
-    </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B107" s="4">
         <v>103</v>
       </c>
@@ -2330,12 +2512,8 @@
         <f t="shared" si="1"/>
         <v>67h</v>
       </c>
-      <c r="D107" s="36"/>
-      <c r="E107" s="36"/>
-      <c r="F107" s="36"/>
-      <c r="G107" s="36"/>
-    </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B108" s="4">
         <v>104</v>
       </c>
@@ -2343,12 +2521,8 @@
         <f t="shared" si="1"/>
         <v>68h</v>
       </c>
-      <c r="D108" s="36"/>
-      <c r="E108" s="36"/>
-      <c r="F108" s="36"/>
-      <c r="G108" s="36"/>
-    </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B109" s="4">
         <v>105</v>
       </c>
@@ -2356,12 +2530,8 @@
         <f t="shared" si="1"/>
         <v>69h</v>
       </c>
-      <c r="D109" s="36"/>
-      <c r="E109" s="36"/>
-      <c r="F109" s="36"/>
-      <c r="G109" s="36"/>
-    </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B110" s="4">
         <v>106</v>
       </c>
@@ -2369,12 +2539,8 @@
         <f t="shared" si="1"/>
         <v>6Ah</v>
       </c>
-      <c r="D110" s="36"/>
-      <c r="E110" s="36"/>
-      <c r="F110" s="36"/>
-      <c r="G110" s="36"/>
-    </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B111" s="4">
         <v>107</v>
       </c>
@@ -2382,14 +2548,8 @@
         <f t="shared" si="1"/>
         <v>6Bh</v>
       </c>
-      <c r="D111" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="E111" s="37"/>
-      <c r="F111" s="37"/>
-      <c r="G111" s="37"/>
-    </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B112" s="4">
         <v>108</v>
       </c>
@@ -2397,12 +2557,8 @@
         <f t="shared" si="1"/>
         <v>6Ch</v>
       </c>
-      <c r="D112" s="37"/>
-      <c r="E112" s="37"/>
-      <c r="F112" s="37"/>
-      <c r="G112" s="37"/>
-    </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B113" s="4">
         <v>109</v>
       </c>
@@ -2410,12 +2566,8 @@
         <f t="shared" si="1"/>
         <v>6Dh</v>
       </c>
-      <c r="D113" s="37"/>
-      <c r="E113" s="37"/>
-      <c r="F113" s="37"/>
-      <c r="G113" s="37"/>
-    </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B114" s="4">
         <v>110</v>
       </c>
@@ -2423,12 +2575,8 @@
         <f t="shared" si="1"/>
         <v>6Eh</v>
       </c>
-      <c r="D114" s="37"/>
-      <c r="E114" s="37"/>
-      <c r="F114" s="37"/>
-      <c r="G114" s="37"/>
-    </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B115" s="4">
         <v>111</v>
       </c>
@@ -2436,12 +2584,8 @@
         <f t="shared" si="1"/>
         <v>6Fh</v>
       </c>
-      <c r="D115" s="37"/>
-      <c r="E115" s="37"/>
-      <c r="F115" s="37"/>
-      <c r="G115" s="37"/>
-    </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B116" s="4">
         <v>112</v>
       </c>
@@ -2449,14 +2593,8 @@
         <f t="shared" si="1"/>
         <v>70h</v>
       </c>
-      <c r="D116" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="E116" s="38"/>
-      <c r="F116" s="38"/>
-      <c r="G116" s="38"/>
-    </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B117" s="4">
         <v>113</v>
       </c>
@@ -2464,12 +2602,8 @@
         <f t="shared" si="1"/>
         <v>71h</v>
       </c>
-      <c r="D117" s="38"/>
-      <c r="E117" s="38"/>
-      <c r="F117" s="38"/>
-      <c r="G117" s="38"/>
-    </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B118" s="4">
         <v>114</v>
       </c>
@@ -2477,12 +2611,8 @@
         <f t="shared" si="1"/>
         <v>72h</v>
       </c>
-      <c r="D118" s="38"/>
-      <c r="E118" s="38"/>
-      <c r="F118" s="38"/>
-      <c r="G118" s="38"/>
-    </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B119" s="4">
         <v>115</v>
       </c>
@@ -2490,12 +2620,8 @@
         <f t="shared" si="1"/>
         <v>73h</v>
       </c>
-      <c r="D119" s="38"/>
-      <c r="E119" s="38"/>
-      <c r="F119" s="38"/>
-      <c r="G119" s="38"/>
-    </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B120" s="4">
         <v>116</v>
       </c>
@@ -2503,12 +2629,8 @@
         <f t="shared" si="1"/>
         <v>74h</v>
       </c>
-      <c r="D120" s="38"/>
-      <c r="E120" s="38"/>
-      <c r="F120" s="38"/>
-      <c r="G120" s="38"/>
-    </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B121" s="4">
         <v>117</v>
       </c>
@@ -2516,12 +2638,8 @@
         <f t="shared" si="1"/>
         <v>75h</v>
       </c>
-      <c r="D121" s="38"/>
-      <c r="E121" s="38"/>
-      <c r="F121" s="38"/>
-      <c r="G121" s="38"/>
-    </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B122" s="4">
         <v>118</v>
       </c>
@@ -2529,12 +2647,8 @@
         <f t="shared" si="1"/>
         <v>76h</v>
       </c>
-      <c r="D122" s="38"/>
-      <c r="E122" s="38"/>
-      <c r="F122" s="38"/>
-      <c r="G122" s="38"/>
-    </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B123" s="4">
         <v>119</v>
       </c>
@@ -2542,12 +2656,8 @@
         <f t="shared" si="1"/>
         <v>77h</v>
       </c>
-      <c r="D123" s="38"/>
-      <c r="E123" s="38"/>
-      <c r="F123" s="38"/>
-      <c r="G123" s="38"/>
-    </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B124" s="4">
         <v>120</v>
       </c>
@@ -2555,12 +2665,8 @@
         <f t="shared" si="1"/>
         <v>78h</v>
       </c>
-      <c r="D124" s="38"/>
-      <c r="E124" s="38"/>
-      <c r="F124" s="38"/>
-      <c r="G124" s="38"/>
-    </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B125" s="4">
         <v>121</v>
       </c>
@@ -2568,12 +2674,8 @@
         <f t="shared" si="1"/>
         <v>79h</v>
       </c>
-      <c r="D125" s="38"/>
-      <c r="E125" s="38"/>
-      <c r="F125" s="38"/>
-      <c r="G125" s="38"/>
-    </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="126" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B126" s="4">
         <v>122</v>
       </c>
@@ -2581,12 +2683,8 @@
         <f t="shared" si="1"/>
         <v>7Ah</v>
       </c>
-      <c r="D126" s="38"/>
-      <c r="E126" s="38"/>
-      <c r="F126" s="38"/>
-      <c r="G126" s="38"/>
-    </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="127" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B127" s="4">
         <v>123</v>
       </c>
@@ -2594,12 +2692,8 @@
         <f t="shared" si="1"/>
         <v>7Bh</v>
       </c>
-      <c r="D127" s="38"/>
-      <c r="E127" s="38"/>
-      <c r="F127" s="38"/>
-      <c r="G127" s="38"/>
-    </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="128" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B128" s="4">
         <v>124</v>
       </c>
@@ -2607,12 +2701,8 @@
         <f t="shared" si="1"/>
         <v>7Ch</v>
       </c>
-      <c r="D128" s="38"/>
-      <c r="E128" s="38"/>
-      <c r="F128" s="38"/>
-      <c r="G128" s="38"/>
-    </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="129" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B129" s="4">
         <v>125</v>
       </c>
@@ -2620,12 +2710,8 @@
         <f t="shared" si="1"/>
         <v>7Dh</v>
       </c>
-      <c r="D129" s="38"/>
-      <c r="E129" s="38"/>
-      <c r="F129" s="38"/>
-      <c r="G129" s="38"/>
-    </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="130" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B130" s="4">
         <v>126</v>
       </c>
@@ -2633,12 +2719,8 @@
         <f t="shared" si="1"/>
         <v>7Eh</v>
       </c>
-      <c r="D130" s="38"/>
-      <c r="E130" s="38"/>
-      <c r="F130" s="38"/>
-      <c r="G130" s="38"/>
-    </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="131" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B131" s="4">
         <v>127</v>
       </c>
@@ -2646,12 +2728,8 @@
         <f t="shared" si="1"/>
         <v>7Fh</v>
       </c>
-      <c r="D131" s="38"/>
-      <c r="E131" s="38"/>
-      <c r="F131" s="38"/>
-      <c r="G131" s="38"/>
-    </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="132" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B132" s="4">
         <v>128</v>
       </c>
@@ -2659,12 +2737,8 @@
         <f t="shared" si="1"/>
         <v>80h</v>
       </c>
-      <c r="D132" s="38"/>
-      <c r="E132" s="38"/>
-      <c r="F132" s="38"/>
-      <c r="G132" s="38"/>
-    </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="133" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B133" s="4">
         <v>129</v>
       </c>
@@ -2672,12 +2746,8 @@
         <f t="shared" ref="C133:C138" si="2">DEC2HEX(B133)&amp;"h"</f>
         <v>81h</v>
       </c>
-      <c r="D133" s="38"/>
-      <c r="E133" s="38"/>
-      <c r="F133" s="38"/>
-      <c r="G133" s="38"/>
-    </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="134" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B134" s="4">
         <v>130</v>
       </c>
@@ -2685,12 +2755,8 @@
         <f t="shared" si="2"/>
         <v>82h</v>
       </c>
-      <c r="D134" s="38"/>
-      <c r="E134" s="38"/>
-      <c r="F134" s="38"/>
-      <c r="G134" s="38"/>
-    </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="135" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B135" s="4">
         <v>131</v>
       </c>
@@ -2698,12 +2764,8 @@
         <f t="shared" si="2"/>
         <v>83h</v>
       </c>
-      <c r="D135" s="38"/>
-      <c r="E135" s="38"/>
-      <c r="F135" s="38"/>
-      <c r="G135" s="38"/>
-    </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="136" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B136" s="4">
         <v>132</v>
       </c>
@@ -2711,12 +2773,8 @@
         <f t="shared" si="2"/>
         <v>84h</v>
       </c>
-      <c r="D136" s="38"/>
-      <c r="E136" s="38"/>
-      <c r="F136" s="38"/>
-      <c r="G136" s="38"/>
-    </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="137" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B137" s="4">
         <v>133</v>
       </c>
@@ -2724,12 +2782,8 @@
         <f t="shared" si="2"/>
         <v>85h</v>
       </c>
-      <c r="D137" s="38"/>
-      <c r="E137" s="38"/>
-      <c r="F137" s="38"/>
-      <c r="G137" s="38"/>
-    </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="138" spans="2:3" x14ac:dyDescent="0.35">
       <c r="B138" s="4">
         <v>134</v>
       </c>
@@ -2737,112 +2791,6 @@
         <f t="shared" si="2"/>
         <v>86h</v>
       </c>
-      <c r="D138" s="38"/>
-      <c r="E138" s="38"/>
-      <c r="F138" s="38"/>
-      <c r="G138" s="38"/>
-    </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D139" s="38"/>
-      <c r="E139" s="38"/>
-      <c r="F139" s="38"/>
-      <c r="G139" s="38"/>
-    </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D140" s="38"/>
-      <c r="E140" s="38"/>
-      <c r="F140" s="38"/>
-      <c r="G140" s="38"/>
-    </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D141" s="38"/>
-      <c r="E141" s="38"/>
-      <c r="F141" s="38"/>
-      <c r="G141" s="38"/>
-    </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D142" s="38"/>
-      <c r="E142" s="38"/>
-      <c r="F142" s="38"/>
-      <c r="G142" s="38"/>
-    </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D143" s="38"/>
-      <c r="E143" s="38"/>
-      <c r="F143" s="38"/>
-      <c r="G143" s="38"/>
-    </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="D144" s="38"/>
-      <c r="E144" s="38"/>
-      <c r="F144" s="38"/>
-      <c r="G144" s="38"/>
-    </row>
-    <row r="145" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D145" s="38"/>
-      <c r="E145" s="38"/>
-      <c r="F145" s="38"/>
-      <c r="G145" s="38"/>
-    </row>
-    <row r="146" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D146" s="38"/>
-      <c r="E146" s="38"/>
-      <c r="F146" s="38"/>
-      <c r="G146" s="38"/>
-    </row>
-    <row r="147" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D147" s="38"/>
-      <c r="E147" s="38"/>
-      <c r="F147" s="38"/>
-      <c r="G147" s="38"/>
-    </row>
-    <row r="148" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D148" s="38"/>
-      <c r="E148" s="38"/>
-      <c r="F148" s="38"/>
-      <c r="G148" s="38"/>
-    </row>
-    <row r="149" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D149" s="38"/>
-      <c r="E149" s="38"/>
-      <c r="F149" s="38"/>
-      <c r="G149" s="38"/>
-    </row>
-    <row r="150" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D150" s="38"/>
-      <c r="E150" s="38"/>
-      <c r="F150" s="38"/>
-      <c r="G150" s="38"/>
-    </row>
-    <row r="151" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D151" s="38"/>
-      <c r="E151" s="38"/>
-      <c r="F151" s="38"/>
-      <c r="G151" s="38"/>
-    </row>
-    <row r="152" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D152" s="38"/>
-      <c r="E152" s="38"/>
-      <c r="F152" s="38"/>
-      <c r="G152" s="38"/>
-    </row>
-    <row r="153" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D153" s="38"/>
-      <c r="E153" s="38"/>
-      <c r="F153" s="38"/>
-      <c r="G153" s="38"/>
-    </row>
-    <row r="154" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D154" s="38"/>
-      <c r="E154" s="38"/>
-      <c r="F154" s="38"/>
-      <c r="G154" s="38"/>
-    </row>
-    <row r="155" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D155" s="38"/>
-      <c r="E155" s="38"/>
-      <c r="F155" s="38"/>
-      <c r="G155" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3056,20 +3004,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="602d6013-12bf-42a7-bc7f-2fade0e82371" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="602d6013-12bf-42a7-bc7f-2fade0e82371" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3092,14 +3040,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E732BC0F-1505-48BB-B355-5D5ECDA47127}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -3114,4 +3054,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added greatestAchievement and worstAchievement and some placeholder buttons for dataSheet and history
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/wh40k_NTAG215_memoryMapping.xlsx
+++ b/wh40k_NTAG215_memoryMapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fuzzy\wh40k_nfc_project\wh40k_nfc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D11917E0-1425-4A83-999D-A0238B3370AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9DF3FF-5D50-4475-A16B-915CE2613F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
+    <workbookView xWindow="-90" yWindow="110" windowWidth="18860" windowHeight="9970" xr2:uid="{4DA63A72-1372-477F-84F9-421F753CD07C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
   <si>
     <t>NTAG215</t>
   </si>
@@ -77,12 +77,6 @@
     <t>I think 50 should cover almost all names, theres probalbly some stupid long ones but usually they can be shortend pretty easily</t>
   </si>
   <si>
-    <t>Kills</t>
-  </si>
-  <si>
-    <t>Deaths</t>
-  </si>
-  <si>
     <t>Total Kills</t>
   </si>
   <si>
@@ -155,9 +149,6 @@
     <t>OTHER DATA</t>
   </si>
   <si>
-    <t>dgi</t>
-  </si>
-  <si>
     <t>dynamic game id (dgi)</t>
   </si>
   <si>
@@ -168,13 +159,61 @@
   </si>
   <si>
     <t>EXTRA SPACE</t>
+  </si>
+  <si>
+    <t>primary</t>
+  </si>
+  <si>
+    <t>secondary</t>
+  </si>
+  <si>
+    <t>epic hero</t>
+  </si>
+  <si>
+    <t>character</t>
+  </si>
+  <si>
+    <t>vehical</t>
+  </si>
+  <si>
+    <t>monster</t>
+  </si>
+  <si>
+    <t>battleline</t>
+  </si>
+  <si>
+    <t>transport</t>
+  </si>
+  <si>
+    <t>mounted</t>
+  </si>
+  <si>
+    <t>other</t>
+  </si>
+  <si>
+    <t>point cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">points/heath deficit/surplus </t>
+  </si>
+  <si>
+    <t>history</t>
+  </si>
+  <si>
+    <t>greatest achivment</t>
+  </si>
+  <si>
+    <t>worst achivment</t>
+  </si>
+  <si>
+    <t>25 games</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,8 +229,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="25">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -294,6 +340,48 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="15">
     <border>
@@ -496,9 +584,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -532,32 +619,18 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -594,6 +667,18 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -986,7 +1071,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E22B5351-43EC-4BE6-A109-53A8CF40F7FA}">
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="18.90625" customWidth="1"/>
@@ -1002,94 +1087,94 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="35" t="s">
+      <c r="B2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="37" t="s">
+      <c r="C2" s="29"/>
+      <c r="D2" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="39"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="32"/>
     </row>
     <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>0</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="6">
         <v>1</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="6">
         <v>2</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="6">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>0</v>
       </c>
-      <c r="C4" s="8" t="str">
+      <c r="C4" s="7" t="str">
         <f>DEC2HEX(B4)&amp;"h"</f>
         <v>0h</v>
       </c>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
       <c r="J4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>1</v>
       </c>
-      <c r="C5" s="4" t="str">
+      <c r="C5" s="3" t="str">
         <f t="shared" ref="C5:C68" si="0">DEC2HEX(B5)&amp;"h"</f>
         <v>1h</v>
       </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="I5" s="6" t="s">
+      <c r="D5" s="34"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="33"/>
+      <c r="I5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="5">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>2</v>
       </c>
-      <c r="C6" s="4" t="str">
+      <c r="C6" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2h</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="10" t="s">
+      <c r="D6" s="8"/>
+      <c r="E6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="42" t="s">
+      <c r="F6" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="43"/>
-      <c r="I6" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="J6" s="11">
+      <c r="G6" s="36"/>
+      <c r="I6" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="10">
         <v>3</v>
       </c>
       <c r="K6" t="s">
@@ -1097,175 +1182,207 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>3</v>
       </c>
-      <c r="C7" s="4" t="str">
+      <c r="C7" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3h</v>
       </c>
-      <c r="D7" s="44" t="s">
+      <c r="D7" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="46"/>
-      <c r="I7" s="18" t="s">
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="39"/>
+      <c r="I7" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="18">
+      <c r="J7" s="17">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>4</v>
       </c>
-      <c r="C8" s="4" t="str">
+      <c r="C8" s="3" t="str">
         <f t="shared" si="0"/>
         <v>4h</v>
       </c>
-      <c r="D8" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="32" t="s">
+      <c r="D8" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B9" s="3">
+        <v>5</v>
+      </c>
+      <c r="C9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>5h</v>
+      </c>
+      <c r="D9" s="42" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="E9" s="42" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="G8" s="31"/>
-      <c r="I8" s="27" t="s">
-        <v>40</v>
-      </c>
-      <c r="J8" s="27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B9" s="4">
-        <v>5</v>
-      </c>
-      <c r="C9" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>5h</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="G9" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9" s="32" t="s">
-        <v>41</v>
+      <c r="G9" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="I9" s="26" t="s">
+        <v>38</v>
       </c>
       <c r="J9">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>6</v>
       </c>
-      <c r="C10" s="4" t="str">
+      <c r="C10" s="3" t="str">
         <f t="shared" si="0"/>
         <v>6h</v>
       </c>
-      <c r="D10" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="I10" s="33" t="s">
-        <v>42</v>
+      <c r="D10" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="27" t="s">
+        <v>39</v>
       </c>
       <c r="J10">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>7</v>
       </c>
-      <c r="C11" s="4" t="str">
+      <c r="C11" s="3" t="str">
         <f t="shared" si="0"/>
         <v>7h</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="43" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="43" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" s="43" t="s">
+        <v>45</v>
+      </c>
+      <c r="G11" s="43" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" s="25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B12" s="3">
+        <v>8</v>
+      </c>
+      <c r="C12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>8h</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="44" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B13" s="3">
         <v>9</v>
       </c>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="I11" s="31" t="s">
-        <v>43</v>
-      </c>
-      <c r="J11" s="31">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B12" s="4">
-        <v>8</v>
-      </c>
-      <c r="C12" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>8h</v>
-      </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B13" s="4">
+      <c r="C13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>9h</v>
+      </c>
+      <c r="D13" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="46" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="B14" s="3">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>Ah</v>
+      </c>
+      <c r="D14" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>9h</v>
-      </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B14" s="4">
-        <v>10</v>
-      </c>
-      <c r="C14" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Ah</v>
-      </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <v>11</v>
       </c>
-      <c r="C15" s="4" t="str">
+      <c r="C15" s="3" t="str">
         <f t="shared" si="0"/>
         <v>Bh</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="I15" s="12" t="s">
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="I15" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="11">
         <v>52</v>
       </c>
       <c r="K15" t="s">
@@ -1273,233 +1390,233 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>12</v>
       </c>
-      <c r="C16" s="4" t="str">
+      <c r="C16" s="3" t="str">
         <f t="shared" si="0"/>
         <v>Ch</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="I16" s="29" t="s">
-        <v>37</v>
-      </c>
-      <c r="J16" s="29">
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="I16" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="J16" s="23">
         <v>1</v>
       </c>
       <c r="K16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B17" s="3">
+        <v>13</v>
+      </c>
+      <c r="C17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>Dh</v>
+      </c>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="I17" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="J17" s="12">
+        <v>1</v>
+      </c>
+      <c r="K17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B18" s="3">
+        <v>14</v>
+      </c>
+      <c r="C18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>Eh</v>
+      </c>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="I18" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" s="13">
+        <v>1</v>
+      </c>
+      <c r="K18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B19" s="3">
+        <v>15</v>
+      </c>
+      <c r="C19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>Fh</v>
+      </c>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="I19" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" s="14">
+        <v>1</v>
+      </c>
+      <c r="K19" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B17" s="4">
-        <v>13</v>
-      </c>
-      <c r="C17" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Dh</v>
-      </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="I17" s="13" t="s">
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B20" s="3">
+        <v>16</v>
+      </c>
+      <c r="C20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>10h</v>
+      </c>
+      <c r="D20" s="20"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="20"/>
+      <c r="I20" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="J20" s="25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B21" s="3">
+        <v>17</v>
+      </c>
+      <c r="C21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>11h</v>
+      </c>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="I21" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="13">
-        <v>1</v>
-      </c>
-      <c r="K17" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B18" s="4">
-        <v>14</v>
-      </c>
-      <c r="C18" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Eh</v>
-      </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="I18" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="J18" s="14">
-        <v>1</v>
-      </c>
-      <c r="K18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B19" s="4">
-        <v>15</v>
-      </c>
-      <c r="C19" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>Fh</v>
-      </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="I19" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="15">
-        <v>1</v>
-      </c>
-      <c r="K19" t="s">
+      <c r="J21" s="16">
+        <v>200</v>
+      </c>
+      <c r="K21" s="15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B22" s="3">
+        <v>18</v>
+      </c>
+      <c r="C22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>12h</v>
+      </c>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="K22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B23" s="3">
+        <v>19</v>
+      </c>
+      <c r="C23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>13h</v>
+      </c>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="K23" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B24" s="3">
+        <v>20</v>
+      </c>
+      <c r="C24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>14h</v>
+      </c>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="I24" s="18" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B20" s="4">
-        <v>16</v>
-      </c>
-      <c r="C20" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>10h</v>
-      </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="I20" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="J20" s="31">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B21" s="4">
+      <c r="J24" s="18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B25" s="3">
+        <v>21</v>
+      </c>
+      <c r="C25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>15h</v>
+      </c>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="I25" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="J25" s="19">
         <v>17</v>
       </c>
-      <c r="C21" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>11h</v>
-      </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="I21" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" s="17">
-        <v>200</v>
-      </c>
-      <c r="K21" s="16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B22" s="4">
-        <v>18</v>
-      </c>
-      <c r="C22" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>12h</v>
-      </c>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="K22" t="s">
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B26" s="3">
+        <v>22</v>
+      </c>
+      <c r="C26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>16h</v>
+      </c>
+      <c r="D26" s="20"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B27" s="3">
+        <v>23</v>
+      </c>
+      <c r="C27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>17h</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B23" s="4">
-        <v>19</v>
-      </c>
-      <c r="C23" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>13h</v>
-      </c>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="K23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B24" s="4">
-        <v>20</v>
-      </c>
-      <c r="C24" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>14h</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="I24" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="J24" s="19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B25" s="4">
-        <v>21</v>
-      </c>
-      <c r="C25" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>15h</v>
-      </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="I25" s="20" t="s">
-        <v>30</v>
-      </c>
-      <c r="J25" s="20">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B26" s="4">
-        <v>22</v>
-      </c>
-      <c r="C26" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>16h</v>
-      </c>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B27" s="4">
-        <v>23</v>
-      </c>
-      <c r="C27" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>17h</v>
-      </c>
-      <c r="D27" s="21"/>
       <c r="E27" s="21"/>
       <c r="F27" s="21"/>
       <c r="G27" s="21"/>
       <c r="I27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J27">
         <f>SUM(J5:J25)</f>
@@ -1507,10 +1624,10 @@
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B28" s="4">
+      <c r="B28" s="3">
         <v>24</v>
       </c>
-      <c r="C28" s="4" t="str">
+      <c r="C28" s="3" t="str">
         <f t="shared" si="0"/>
         <v>18h</v>
       </c>
@@ -1519,7 +1636,7 @@
       <c r="F28" s="21"/>
       <c r="G28" s="21"/>
       <c r="I28" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J28">
         <f>540-J27</f>
@@ -1527,1270 +1644,1570 @@
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B29" s="4">
+      <c r="B29" s="3">
         <v>25</v>
       </c>
-      <c r="C29" s="4" t="str">
+      <c r="C29" s="3" t="str">
         <f t="shared" si="0"/>
         <v>19h</v>
       </c>
-      <c r="D29" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B30" s="4">
+      <c r="B30" s="3">
         <v>26</v>
       </c>
-      <c r="C30" s="4" t="str">
+      <c r="C30" s="3" t="str">
         <f t="shared" si="0"/>
         <v>1Ah</v>
       </c>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B31" s="4">
+      <c r="B31" s="3">
         <v>27</v>
       </c>
-      <c r="C31" s="4" t="str">
+      <c r="C31" s="3" t="str">
         <f t="shared" si="0"/>
         <v>1Bh</v>
       </c>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B32" s="4">
+      <c r="B32" s="3">
         <v>28</v>
       </c>
-      <c r="C32" s="4" t="str">
+      <c r="C32" s="3" t="str">
         <f t="shared" si="0"/>
         <v>1Ch</v>
       </c>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B33" s="4">
+      <c r="B33" s="3">
         <v>29</v>
       </c>
-      <c r="C33" s="4" t="str">
+      <c r="C33" s="3" t="str">
         <f t="shared" si="0"/>
         <v>1Dh</v>
       </c>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B34" s="4">
+      <c r="B34" s="3">
         <v>30</v>
       </c>
-      <c r="C34" s="4" t="str">
+      <c r="C34" s="3" t="str">
         <f t="shared" si="0"/>
         <v>1Eh</v>
       </c>
-      <c r="D34" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="E34" s="24"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B35" s="4">
+      <c r="B35" s="3">
         <v>31</v>
       </c>
-      <c r="C35" s="4" t="str">
+      <c r="C35" s="3" t="str">
         <f t="shared" si="0"/>
         <v>1Fh</v>
       </c>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="24"/>
-      <c r="G35" s="24"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B36" s="4">
+      <c r="B36" s="3">
         <v>32</v>
       </c>
-      <c r="C36" s="4" t="str">
+      <c r="C36" s="3" t="str">
         <f t="shared" si="0"/>
         <v>20h</v>
       </c>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="24"/>
-      <c r="G36" s="24"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="21"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B37" s="4">
+      <c r="B37" s="3">
         <v>33</v>
       </c>
-      <c r="C37" s="4" t="str">
+      <c r="C37" s="3" t="str">
         <f t="shared" si="0"/>
         <v>21h</v>
       </c>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="24"/>
-      <c r="G37" s="24"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="21"/>
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B38" s="4">
+      <c r="B38" s="3">
         <v>34</v>
       </c>
-      <c r="C38" s="4" t="str">
+      <c r="C38" s="3" t="str">
         <f t="shared" si="0"/>
         <v>22h</v>
       </c>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="24"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="21"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B39" s="4">
+      <c r="B39" s="3">
         <v>35</v>
       </c>
-      <c r="C39" s="4" t="str">
+      <c r="C39" s="3" t="str">
         <f t="shared" si="0"/>
         <v>23h</v>
       </c>
-      <c r="D39" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B40" s="4">
+      <c r="B40" s="3">
         <v>36</v>
       </c>
-      <c r="C40" s="4" t="str">
+      <c r="C40" s="3" t="str">
         <f t="shared" si="0"/>
         <v>24h</v>
       </c>
-      <c r="D40" s="25"/>
-      <c r="E40" s="25"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="25"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="21"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B41" s="4">
+      <c r="B41" s="3">
         <v>37</v>
       </c>
-      <c r="C41" s="4" t="str">
+      <c r="C41" s="3" t="str">
         <f t="shared" si="0"/>
         <v>25h</v>
       </c>
-      <c r="D41" s="25"/>
-      <c r="E41" s="25"/>
-      <c r="F41" s="25"/>
-      <c r="G41" s="25"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B42" s="4">
+      <c r="B42" s="3">
         <v>38</v>
       </c>
-      <c r="C42" s="4" t="str">
+      <c r="C42" s="3" t="str">
         <f t="shared" si="0"/>
         <v>26h</v>
       </c>
-      <c r="D42" s="25"/>
-      <c r="E42" s="25"/>
-      <c r="F42" s="25"/>
-      <c r="G42" s="25"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="21"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B43" s="4">
+      <c r="B43" s="3">
         <v>39</v>
       </c>
-      <c r="C43" s="4" t="str">
+      <c r="C43" s="3" t="str">
         <f t="shared" si="0"/>
         <v>27h</v>
       </c>
-      <c r="D43" s="25"/>
-      <c r="E43" s="25"/>
-      <c r="F43" s="25"/>
-      <c r="G43" s="25"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="21"/>
     </row>
     <row r="44" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B44" s="4">
+      <c r="B44" s="3">
         <v>40</v>
       </c>
-      <c r="C44" s="4" t="str">
+      <c r="C44" s="3" t="str">
         <f t="shared" si="0"/>
         <v>28h</v>
       </c>
-      <c r="D44" s="26" t="s">
-        <v>23</v>
-      </c>
-      <c r="E44" s="26"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="26"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="21"/>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B45" s="4">
+      <c r="B45" s="3">
         <v>41</v>
       </c>
-      <c r="C45" s="4" t="str">
+      <c r="C45" s="3" t="str">
         <f t="shared" si="0"/>
         <v>29h</v>
       </c>
-      <c r="D45" s="26"/>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="26"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B46" s="4">
+      <c r="B46" s="3">
         <v>42</v>
       </c>
-      <c r="C46" s="4" t="str">
+      <c r="C46" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2Ah</v>
       </c>
-      <c r="D46" s="26"/>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="26"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B47" s="4">
+      <c r="B47" s="3">
         <v>43</v>
       </c>
-      <c r="C47" s="4" t="str">
+      <c r="C47" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2Bh</v>
       </c>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="26"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B48" s="4">
+      <c r="B48" s="3">
         <v>44</v>
       </c>
-      <c r="C48" s="4" t="str">
+      <c r="C48" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2Ch</v>
       </c>
-      <c r="D48" s="26"/>
-      <c r="E48" s="26"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="26"/>
+      <c r="D48" s="21"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="21"/>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B49" s="4">
+      <c r="B49" s="3">
         <v>45</v>
       </c>
-      <c r="C49" s="4" t="str">
+      <c r="C49" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2Dh</v>
       </c>
-      <c r="D49" s="26"/>
-      <c r="E49" s="26"/>
-      <c r="F49" s="26"/>
-      <c r="G49" s="26"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="21"/>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B50" s="4">
+      <c r="B50" s="3">
         <v>46</v>
       </c>
-      <c r="C50" s="4" t="str">
+      <c r="C50" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2Eh</v>
       </c>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="26"/>
+      <c r="D50" s="21"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="21"/>
+      <c r="G50" s="21"/>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B51" s="4">
+      <c r="B51" s="3">
         <v>47</v>
       </c>
-      <c r="C51" s="4" t="str">
+      <c r="C51" s="3" t="str">
         <f t="shared" si="0"/>
         <v>2Fh</v>
       </c>
-      <c r="D51" s="26"/>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
-      <c r="G51" s="26"/>
+      <c r="D51" s="21"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="21"/>
+      <c r="G51" s="21"/>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B52" s="4">
+      <c r="B52" s="3">
         <v>48</v>
       </c>
-      <c r="C52" s="4" t="str">
+      <c r="C52" s="3" t="str">
         <f t="shared" si="0"/>
         <v>30h</v>
       </c>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="21"/>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B53" s="4">
+      <c r="B53" s="3">
         <v>49</v>
       </c>
-      <c r="C53" s="4" t="str">
+      <c r="C53" s="3" t="str">
         <f t="shared" si="0"/>
         <v>31h</v>
       </c>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="26"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="21"/>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B54" s="4">
+      <c r="B54" s="3">
         <v>50</v>
       </c>
-      <c r="C54" s="4" t="str">
+      <c r="C54" s="3" t="str">
         <f t="shared" si="0"/>
         <v>32h</v>
       </c>
-      <c r="D54" s="26"/>
-      <c r="E54" s="26"/>
-      <c r="F54" s="26"/>
-      <c r="G54" s="26"/>
+      <c r="D54" s="21"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="21"/>
+      <c r="G54" s="21"/>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B55" s="4">
+      <c r="B55" s="3">
         <v>51</v>
       </c>
-      <c r="C55" s="4" t="str">
+      <c r="C55" s="3" t="str">
         <f t="shared" si="0"/>
         <v>33h</v>
       </c>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="21"/>
+      <c r="G55" s="21"/>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B56" s="4">
+      <c r="B56" s="3">
         <v>52</v>
       </c>
-      <c r="C56" s="4" t="str">
+      <c r="C56" s="3" t="str">
         <f t="shared" si="0"/>
         <v>34h</v>
       </c>
-      <c r="D56" s="26"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
-      <c r="G56" s="26"/>
+      <c r="D56" s="21"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="21"/>
+      <c r="G56" s="21"/>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B57" s="4">
+      <c r="B57" s="3">
         <v>53</v>
       </c>
-      <c r="C57" s="4" t="str">
+      <c r="C57" s="3" t="str">
         <f t="shared" si="0"/>
         <v>35h</v>
       </c>
-      <c r="D57" s="26"/>
-      <c r="E57" s="26"/>
-      <c r="F57" s="26"/>
-      <c r="G57" s="26"/>
+      <c r="D57" s="21"/>
+      <c r="E57" s="21"/>
+      <c r="F57" s="21"/>
+      <c r="G57" s="21"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B58" s="4">
+      <c r="B58" s="3">
         <v>54</v>
       </c>
-      <c r="C58" s="4" t="str">
+      <c r="C58" s="3" t="str">
         <f t="shared" si="0"/>
         <v>36h</v>
       </c>
-      <c r="D58" s="26"/>
-      <c r="E58" s="26"/>
-      <c r="F58" s="26"/>
-      <c r="G58" s="26"/>
+      <c r="D58" s="21"/>
+      <c r="E58" s="21"/>
+      <c r="F58" s="21"/>
+      <c r="G58" s="21"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B59" s="4">
+      <c r="B59" s="3">
         <v>55</v>
       </c>
-      <c r="C59" s="4" t="str">
+      <c r="C59" s="3" t="str">
         <f t="shared" si="0"/>
         <v>37h</v>
       </c>
-      <c r="D59" s="26"/>
-      <c r="E59" s="26"/>
-      <c r="F59" s="26"/>
-      <c r="G59" s="26"/>
+      <c r="D59" s="21"/>
+      <c r="E59" s="21"/>
+      <c r="F59" s="21"/>
+      <c r="G59" s="21"/>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B60" s="4">
+      <c r="B60" s="3">
         <v>56</v>
       </c>
-      <c r="C60" s="4" t="str">
+      <c r="C60" s="3" t="str">
         <f t="shared" si="0"/>
         <v>38h</v>
       </c>
-      <c r="D60" s="26"/>
-      <c r="E60" s="26"/>
-      <c r="F60" s="26"/>
-      <c r="G60" s="26"/>
+      <c r="D60" s="21"/>
+      <c r="E60" s="21"/>
+      <c r="F60" s="21"/>
+      <c r="G60" s="21"/>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B61" s="4">
+      <c r="B61" s="3">
         <v>57</v>
       </c>
-      <c r="C61" s="4" t="str">
+      <c r="C61" s="3" t="str">
         <f t="shared" si="0"/>
         <v>39h</v>
       </c>
-      <c r="D61" s="26"/>
-      <c r="E61" s="26"/>
-      <c r="F61" s="26"/>
-      <c r="G61" s="26"/>
+      <c r="D61" s="21"/>
+      <c r="E61" s="21"/>
+      <c r="F61" s="21"/>
+      <c r="G61" s="21"/>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B62" s="4">
+      <c r="B62" s="3">
         <v>58</v>
       </c>
-      <c r="C62" s="4" t="str">
+      <c r="C62" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3Ah</v>
       </c>
-      <c r="D62" s="26"/>
-      <c r="E62" s="26"/>
-      <c r="F62" s="26"/>
-      <c r="G62" s="26"/>
+      <c r="D62" s="21"/>
+      <c r="E62" s="21"/>
+      <c r="F62" s="21"/>
+      <c r="G62" s="21"/>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B63" s="4">
+      <c r="B63" s="3">
         <v>59</v>
       </c>
-      <c r="C63" s="4" t="str">
+      <c r="C63" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3Bh</v>
       </c>
-      <c r="D63" s="26"/>
-      <c r="E63" s="26"/>
-      <c r="F63" s="26"/>
-      <c r="G63" s="26"/>
+      <c r="D63" s="21"/>
+      <c r="E63" s="21"/>
+      <c r="F63" s="21"/>
+      <c r="G63" s="21"/>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B64" s="4">
+      <c r="B64" s="3">
         <v>60</v>
       </c>
-      <c r="C64" s="4" t="str">
+      <c r="C64" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3Ch</v>
       </c>
-      <c r="D64" s="26"/>
-      <c r="E64" s="26"/>
-      <c r="F64" s="26"/>
-      <c r="G64" s="26"/>
+      <c r="D64" s="21"/>
+      <c r="E64" s="21"/>
+      <c r="F64" s="21"/>
+      <c r="G64" s="21"/>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B65" s="4">
+      <c r="B65" s="3">
         <v>61</v>
       </c>
-      <c r="C65" s="4" t="str">
+      <c r="C65" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3Dh</v>
       </c>
-      <c r="D65" s="26"/>
-      <c r="E65" s="26"/>
-      <c r="F65" s="26"/>
-      <c r="G65" s="26"/>
+      <c r="D65" s="21"/>
+      <c r="E65" s="21"/>
+      <c r="F65" s="21"/>
+      <c r="G65" s="21"/>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B66" s="4">
+      <c r="B66" s="3">
         <v>62</v>
       </c>
-      <c r="C66" s="4" t="str">
+      <c r="C66" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3Eh</v>
       </c>
-      <c r="D66" s="26"/>
-      <c r="E66" s="26"/>
-      <c r="F66" s="26"/>
-      <c r="G66" s="26"/>
+      <c r="D66" s="21"/>
+      <c r="E66" s="21"/>
+      <c r="F66" s="21"/>
+      <c r="G66" s="21"/>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B67" s="4">
+      <c r="B67" s="3">
         <v>63</v>
       </c>
-      <c r="C67" s="4" t="str">
+      <c r="C67" s="3" t="str">
         <f t="shared" si="0"/>
         <v>3Fh</v>
       </c>
-      <c r="D67" s="26"/>
-      <c r="E67" s="26"/>
-      <c r="F67" s="26"/>
-      <c r="G67" s="26"/>
+      <c r="D67" s="47" t="s">
+        <v>54</v>
+      </c>
+      <c r="E67" s="47"/>
+      <c r="F67" s="47"/>
+      <c r="G67" s="47"/>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B68" s="4">
+      <c r="B68" s="3">
         <v>64</v>
       </c>
-      <c r="C68" s="4" t="str">
+      <c r="C68" s="3" t="str">
         <f t="shared" si="0"/>
         <v>40h</v>
       </c>
-      <c r="D68" s="26"/>
-      <c r="E68" s="26"/>
-      <c r="F68" s="26"/>
-      <c r="G68" s="26"/>
+      <c r="D68" s="47"/>
+      <c r="E68" s="47"/>
+      <c r="F68" s="47"/>
+      <c r="G68" s="47"/>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B69" s="4">
+      <c r="B69" s="3">
         <v>65</v>
       </c>
-      <c r="C69" s="4" t="str">
+      <c r="C69" s="3" t="str">
         <f t="shared" ref="C69:C132" si="1">DEC2HEX(B69)&amp;"h"</f>
         <v>41h</v>
       </c>
-      <c r="D69" s="26"/>
-      <c r="E69" s="26"/>
-      <c r="F69" s="26"/>
-      <c r="G69" s="26"/>
+      <c r="D69" s="47"/>
+      <c r="E69" s="47"/>
+      <c r="F69" s="47"/>
+      <c r="G69" s="47"/>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B70" s="4">
+      <c r="B70" s="3">
         <v>66</v>
       </c>
-      <c r="C70" s="4" t="str">
+      <c r="C70" s="3" t="str">
         <f t="shared" si="1"/>
         <v>42h</v>
       </c>
-      <c r="D70" s="26"/>
-      <c r="E70" s="26"/>
-      <c r="F70" s="26"/>
-      <c r="G70" s="26"/>
+      <c r="D70" s="47"/>
+      <c r="E70" s="47"/>
+      <c r="F70" s="47"/>
+      <c r="G70" s="47"/>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B71" s="4">
+      <c r="B71" s="3">
         <v>67</v>
       </c>
-      <c r="C71" s="4" t="str">
+      <c r="C71" s="3" t="str">
         <f t="shared" si="1"/>
         <v>43h</v>
       </c>
-      <c r="D71" s="26"/>
-      <c r="E71" s="26"/>
-      <c r="F71" s="26"/>
-      <c r="G71" s="26"/>
+      <c r="D71" s="47"/>
+      <c r="E71" s="47"/>
+      <c r="F71" s="47"/>
+      <c r="G71" s="47"/>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B72" s="4">
+      <c r="B72" s="3">
         <v>68</v>
       </c>
-      <c r="C72" s="4" t="str">
+      <c r="C72" s="3" t="str">
         <f t="shared" si="1"/>
         <v>44h</v>
       </c>
-      <c r="D72" s="26"/>
-      <c r="E72" s="26"/>
-      <c r="F72" s="26"/>
-      <c r="G72" s="26"/>
+      <c r="D72" s="47"/>
+      <c r="E72" s="47"/>
+      <c r="F72" s="47"/>
+      <c r="G72" s="47"/>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B73" s="4">
+      <c r="B73" s="3">
         <v>69</v>
       </c>
-      <c r="C73" s="4" t="str">
+      <c r="C73" s="3" t="str">
         <f t="shared" si="1"/>
         <v>45h</v>
       </c>
-      <c r="D73" s="26"/>
-      <c r="E73" s="26"/>
-      <c r="F73" s="26"/>
-      <c r="G73" s="26"/>
+      <c r="D73" s="47"/>
+      <c r="E73" s="47"/>
+      <c r="F73" s="47"/>
+      <c r="G73" s="47"/>
     </row>
     <row r="74" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B74" s="4">
+      <c r="B74" s="3">
         <v>70</v>
       </c>
-      <c r="C74" s="4" t="str">
+      <c r="C74" s="3" t="str">
         <f t="shared" si="1"/>
         <v>46h</v>
       </c>
-      <c r="D74" s="26"/>
-      <c r="E74" s="26"/>
-      <c r="F74" s="26"/>
-      <c r="G74" s="26"/>
+      <c r="D74" s="47"/>
+      <c r="E74" s="47"/>
+      <c r="F74" s="47"/>
+      <c r="G74" s="47"/>
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B75" s="4">
+      <c r="B75" s="3">
         <v>71</v>
       </c>
-      <c r="C75" s="4" t="str">
+      <c r="C75" s="3" t="str">
         <f t="shared" si="1"/>
         <v>47h</v>
       </c>
-      <c r="D75" s="26"/>
-      <c r="E75" s="26"/>
-      <c r="F75" s="26"/>
-      <c r="G75" s="26"/>
+      <c r="D75" s="47"/>
+      <c r="E75" s="47"/>
+      <c r="F75" s="47"/>
+      <c r="G75" s="47"/>
     </row>
     <row r="76" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B76" s="4">
+      <c r="B76" s="3">
         <v>72</v>
       </c>
-      <c r="C76" s="4" t="str">
+      <c r="C76" s="3" t="str">
         <f t="shared" si="1"/>
         <v>48h</v>
       </c>
-      <c r="D76" s="26"/>
-      <c r="E76" s="26"/>
-      <c r="F76" s="26"/>
-      <c r="G76" s="26"/>
+      <c r="D76" s="47"/>
+      <c r="E76" s="47"/>
+      <c r="F76" s="47"/>
+      <c r="G76" s="47"/>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B77" s="4">
+      <c r="B77" s="3">
         <v>73</v>
       </c>
-      <c r="C77" s="4" t="str">
+      <c r="C77" s="3" t="str">
         <f t="shared" si="1"/>
         <v>49h</v>
       </c>
-      <c r="D77" s="26"/>
-      <c r="E77" s="26"/>
-      <c r="F77" s="26"/>
-      <c r="G77" s="26"/>
+      <c r="D77" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="E77" s="48"/>
+      <c r="F77" s="48"/>
+      <c r="G77" s="48"/>
     </row>
     <row r="78" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B78" s="4">
+      <c r="B78" s="3">
         <v>74</v>
       </c>
-      <c r="C78" s="4" t="str">
+      <c r="C78" s="3" t="str">
         <f t="shared" si="1"/>
         <v>4Ah</v>
       </c>
-      <c r="D78" s="26"/>
-      <c r="E78" s="26"/>
-      <c r="F78" s="26"/>
-      <c r="G78" s="26"/>
+      <c r="D78" s="48"/>
+      <c r="E78" s="48"/>
+      <c r="F78" s="48"/>
+      <c r="G78" s="48"/>
     </row>
     <row r="79" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B79" s="4">
+      <c r="B79" s="3">
         <v>75</v>
       </c>
-      <c r="C79" s="4" t="str">
+      <c r="C79" s="3" t="str">
         <f t="shared" si="1"/>
         <v>4Bh</v>
       </c>
-      <c r="D79" s="26"/>
-      <c r="E79" s="26"/>
-      <c r="F79" s="26"/>
-      <c r="G79" s="26"/>
+      <c r="D79" s="48"/>
+      <c r="E79" s="48"/>
+      <c r="F79" s="48"/>
+      <c r="G79" s="48"/>
     </row>
     <row r="80" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B80" s="4">
+      <c r="B80" s="3">
         <v>76</v>
       </c>
-      <c r="C80" s="4" t="str">
+      <c r="C80" s="3" t="str">
         <f t="shared" si="1"/>
         <v>4Ch</v>
       </c>
-      <c r="D80" s="26"/>
-      <c r="E80" s="26"/>
-      <c r="F80" s="26"/>
-      <c r="G80" s="26"/>
+      <c r="D80" s="48"/>
+      <c r="E80" s="48"/>
+      <c r="F80" s="48"/>
+      <c r="G80" s="48"/>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B81" s="4">
+      <c r="B81" s="3">
         <v>77</v>
       </c>
-      <c r="C81" s="4" t="str">
+      <c r="C81" s="3" t="str">
         <f t="shared" si="1"/>
         <v>4Dh</v>
       </c>
-      <c r="D81" s="26"/>
-      <c r="E81" s="26"/>
-      <c r="F81" s="26"/>
-      <c r="G81" s="26"/>
+      <c r="D81" s="48"/>
+      <c r="E81" s="48"/>
+      <c r="F81" s="48"/>
+      <c r="G81" s="48"/>
     </row>
     <row r="82" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B82" s="4">
+      <c r="B82" s="3">
         <v>78</v>
       </c>
-      <c r="C82" s="4" t="str">
+      <c r="C82" s="3" t="str">
         <f t="shared" si="1"/>
         <v>4Eh</v>
       </c>
-      <c r="D82" s="26"/>
-      <c r="E82" s="26"/>
-      <c r="F82" s="26"/>
-      <c r="G82" s="26"/>
+      <c r="D82" s="48"/>
+      <c r="E82" s="48"/>
+      <c r="F82" s="48"/>
+      <c r="G82" s="48"/>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B83" s="4">
+      <c r="B83" s="3">
         <v>79</v>
       </c>
-      <c r="C83" s="4" t="str">
+      <c r="C83" s="3" t="str">
         <f t="shared" si="1"/>
         <v>4Fh</v>
       </c>
-      <c r="D83" s="26"/>
-      <c r="E83" s="26"/>
-      <c r="F83" s="26"/>
-      <c r="G83" s="26"/>
+      <c r="D83" s="48"/>
+      <c r="E83" s="48"/>
+      <c r="F83" s="48"/>
+      <c r="G83" s="48"/>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B84" s="4">
+      <c r="B84" s="3">
         <v>80</v>
       </c>
-      <c r="C84" s="4" t="str">
+      <c r="C84" s="3" t="str">
         <f t="shared" si="1"/>
         <v>50h</v>
       </c>
-      <c r="D84" s="1"/>
-      <c r="E84" s="1"/>
-      <c r="F84" s="1"/>
-      <c r="G84" s="1"/>
+      <c r="D84" s="48"/>
+      <c r="E84" s="48"/>
+      <c r="F84" s="48"/>
+      <c r="G84" s="48"/>
     </row>
     <row r="85" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B85" s="4">
+      <c r="B85" s="3">
         <v>81</v>
       </c>
-      <c r="C85" s="4" t="str">
+      <c r="C85" s="3" t="str">
         <f t="shared" si="1"/>
         <v>51h</v>
       </c>
-      <c r="D85" s="1"/>
-      <c r="E85" s="1"/>
-      <c r="F85" s="1"/>
-      <c r="G85" s="1"/>
+      <c r="D85" s="48"/>
+      <c r="E85" s="48"/>
+      <c r="F85" s="48"/>
+      <c r="G85" s="48"/>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B86" s="4">
+      <c r="B86" s="3">
         <v>82</v>
       </c>
-      <c r="C86" s="4" t="str">
+      <c r="C86" s="3" t="str">
         <f t="shared" si="1"/>
         <v>52h</v>
       </c>
-      <c r="D86" s="1"/>
-      <c r="E86" s="1"/>
-      <c r="F86" s="1"/>
-      <c r="G86" s="1"/>
+      <c r="D86" s="48"/>
+      <c r="E86" s="48"/>
+      <c r="F86" s="48"/>
+      <c r="G86" s="48"/>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B87" s="4">
+      <c r="B87" s="3">
         <v>83</v>
       </c>
-      <c r="C87" s="4" t="str">
+      <c r="C87" s="3" t="str">
         <f t="shared" si="1"/>
         <v>53h</v>
       </c>
-      <c r="D87" s="1"/>
-      <c r="E87" s="1"/>
-      <c r="F87" s="1"/>
-      <c r="G87" s="1"/>
+      <c r="D87" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="E87" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F87" s="40"/>
+      <c r="G87" s="40"/>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B88" s="4">
+      <c r="B88" s="3">
         <v>84</v>
       </c>
-      <c r="C88" s="4" t="str">
+      <c r="C88" s="3" t="str">
         <f t="shared" si="1"/>
         <v>54h</v>
       </c>
-      <c r="D88" s="1"/>
-      <c r="E88" s="1"/>
-      <c r="F88" s="1"/>
-      <c r="G88" s="1"/>
+      <c r="D88" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="E88" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="F88" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="G88" s="41" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B89" s="4">
+      <c r="B89" s="3">
         <v>85</v>
       </c>
-      <c r="C89" s="4" t="str">
+      <c r="C89" s="3" t="str">
         <f t="shared" si="1"/>
         <v>55h</v>
       </c>
-      <c r="D89" s="1"/>
-      <c r="E89" s="1"/>
-      <c r="F89" s="1"/>
-      <c r="G89" s="1"/>
+      <c r="D89" s="40"/>
+      <c r="E89" s="40"/>
+      <c r="F89" s="40"/>
+      <c r="G89" s="40"/>
     </row>
     <row r="90" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B90" s="4">
+      <c r="B90" s="3">
         <v>86</v>
       </c>
-      <c r="C90" s="4" t="str">
+      <c r="C90" s="3" t="str">
         <f t="shared" si="1"/>
         <v>56h</v>
       </c>
-      <c r="D90" s="1"/>
-      <c r="E90" s="1"/>
-      <c r="F90" s="1"/>
-      <c r="G90" s="1"/>
+      <c r="D90" s="40"/>
+      <c r="E90" s="40"/>
+      <c r="F90" s="40"/>
+      <c r="G90" s="40"/>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B91" s="4">
+      <c r="B91" s="3">
         <v>87</v>
       </c>
-      <c r="C91" s="4" t="str">
+      <c r="C91" s="3" t="str">
         <f t="shared" si="1"/>
         <v>57h</v>
       </c>
-      <c r="D91" s="1"/>
-      <c r="E91" s="1"/>
-      <c r="F91" s="1"/>
-      <c r="G91" s="1"/>
+      <c r="D91" s="40"/>
+      <c r="E91" s="40"/>
+      <c r="F91" s="40"/>
+      <c r="G91" s="40"/>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B92" s="4">
+      <c r="B92" s="3">
         <v>88</v>
       </c>
-      <c r="C92" s="4" t="str">
+      <c r="C92" s="3" t="str">
         <f t="shared" si="1"/>
         <v>58h</v>
       </c>
-      <c r="D92" s="1"/>
-      <c r="E92" s="1"/>
-      <c r="F92" s="1"/>
-      <c r="G92" s="1"/>
+      <c r="D92" s="40"/>
+      <c r="E92" s="40"/>
+      <c r="F92" s="40"/>
+      <c r="G92" s="40"/>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B93" s="4">
+      <c r="B93" s="3">
         <v>89</v>
       </c>
-      <c r="C93" s="4" t="str">
+      <c r="C93" s="3" t="str">
         <f t="shared" si="1"/>
         <v>59h</v>
       </c>
-      <c r="D93" s="1"/>
-      <c r="E93" s="1"/>
-      <c r="F93" s="1"/>
-      <c r="G93" s="1"/>
+      <c r="D93" s="40"/>
+      <c r="E93" s="40"/>
+      <c r="F93" s="40"/>
+      <c r="G93" s="40"/>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B94" s="4">
+      <c r="B94" s="3">
         <v>90</v>
       </c>
-      <c r="C94" s="4" t="str">
+      <c r="C94" s="3" t="str">
         <f t="shared" si="1"/>
         <v>5Ah</v>
       </c>
-      <c r="D94" s="1"/>
-      <c r="E94" s="1"/>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
+      <c r="D94" s="40"/>
+      <c r="E94" s="40"/>
+      <c r="F94" s="40"/>
+      <c r="G94" s="40"/>
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B95" s="4">
+      <c r="B95" s="3">
         <v>91</v>
       </c>
-      <c r="C95" s="4" t="str">
+      <c r="C95" s="3" t="str">
         <f t="shared" si="1"/>
         <v>5Bh</v>
       </c>
-      <c r="D95" s="1"/>
-      <c r="E95" s="1"/>
-      <c r="F95" s="1"/>
-      <c r="G95" s="1"/>
+      <c r="D95" s="40"/>
+      <c r="E95" s="40"/>
+      <c r="F95" s="40"/>
+      <c r="G95" s="40"/>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B96" s="4">
+      <c r="B96" s="3">
         <v>92</v>
       </c>
-      <c r="C96" s="4" t="str">
+      <c r="C96" s="3" t="str">
         <f t="shared" si="1"/>
         <v>5Ch</v>
       </c>
-    </row>
-    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B97" s="4">
+      <c r="D96" s="40"/>
+      <c r="E96" s="40"/>
+      <c r="F96" s="40"/>
+      <c r="G96" s="40"/>
+    </row>
+    <row r="97" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B97" s="3">
         <v>93</v>
       </c>
-      <c r="C97" s="4" t="str">
+      <c r="C97" s="3" t="str">
         <f t="shared" si="1"/>
         <v>5Dh</v>
       </c>
-    </row>
-    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B98" s="4">
+      <c r="D97" s="40"/>
+      <c r="E97" s="40"/>
+      <c r="F97" s="40"/>
+      <c r="G97" s="40"/>
+    </row>
+    <row r="98" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B98" s="3">
         <v>94</v>
       </c>
-      <c r="C98" s="4" t="str">
+      <c r="C98" s="3" t="str">
         <f t="shared" si="1"/>
         <v>5Eh</v>
       </c>
-    </row>
-    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B99" s="4">
+      <c r="D98" s="40"/>
+      <c r="E98" s="40"/>
+      <c r="F98" s="40"/>
+      <c r="G98" s="40"/>
+    </row>
+    <row r="99" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B99" s="3">
         <v>95</v>
       </c>
-      <c r="C99" s="4" t="str">
+      <c r="C99" s="3" t="str">
         <f t="shared" si="1"/>
         <v>5Fh</v>
       </c>
-    </row>
-    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B100" s="4">
+      <c r="D99" s="40"/>
+      <c r="E99" s="40"/>
+      <c r="F99" s="40"/>
+      <c r="G99" s="40"/>
+    </row>
+    <row r="100" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B100" s="3">
         <v>96</v>
       </c>
-      <c r="C100" s="4" t="str">
+      <c r="C100" s="3" t="str">
         <f t="shared" si="1"/>
         <v>60h</v>
       </c>
-    </row>
-    <row r="101" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B101" s="4">
+      <c r="D100" s="40"/>
+      <c r="E100" s="40"/>
+      <c r="F100" s="40"/>
+      <c r="G100" s="40"/>
+    </row>
+    <row r="101" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B101" s="3">
         <v>97</v>
       </c>
-      <c r="C101" s="4" t="str">
+      <c r="C101" s="3" t="str">
         <f t="shared" si="1"/>
         <v>61h</v>
       </c>
-    </row>
-    <row r="102" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B102" s="4">
+      <c r="D101" s="40"/>
+      <c r="E101" s="40"/>
+      <c r="F101" s="40"/>
+      <c r="G101" s="40"/>
+    </row>
+    <row r="102" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B102" s="3">
         <v>98</v>
       </c>
-      <c r="C102" s="4" t="str">
+      <c r="C102" s="3" t="str">
         <f t="shared" si="1"/>
         <v>62h</v>
       </c>
-    </row>
-    <row r="103" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B103" s="4">
+      <c r="D102" s="40"/>
+      <c r="E102" s="40"/>
+      <c r="F102" s="40"/>
+      <c r="G102" s="40"/>
+    </row>
+    <row r="103" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B103" s="3">
         <v>99</v>
       </c>
-      <c r="C103" s="4" t="str">
+      <c r="C103" s="3" t="str">
         <f t="shared" si="1"/>
         <v>63h</v>
       </c>
-    </row>
-    <row r="104" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B104" s="4">
+      <c r="D103" s="40"/>
+      <c r="E103" s="40"/>
+      <c r="F103" s="40"/>
+      <c r="G103" s="40"/>
+    </row>
+    <row r="104" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B104" s="3">
         <v>100</v>
       </c>
-      <c r="C104" s="4" t="str">
+      <c r="C104" s="3" t="str">
         <f t="shared" si="1"/>
         <v>64h</v>
       </c>
-    </row>
-    <row r="105" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B105" s="4">
+      <c r="D104" s="40"/>
+      <c r="E104" s="40"/>
+      <c r="F104" s="40"/>
+      <c r="G104" s="40"/>
+    </row>
+    <row r="105" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B105" s="3">
         <v>101</v>
       </c>
-      <c r="C105" s="4" t="str">
+      <c r="C105" s="3" t="str">
         <f t="shared" si="1"/>
         <v>65h</v>
       </c>
-    </row>
-    <row r="106" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B106" s="4">
+      <c r="D105" s="40"/>
+      <c r="E105" s="40"/>
+      <c r="F105" s="40"/>
+      <c r="G105" s="40"/>
+    </row>
+    <row r="106" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B106" s="3">
         <v>102</v>
       </c>
-      <c r="C106" s="4" t="str">
+      <c r="C106" s="3" t="str">
         <f t="shared" si="1"/>
         <v>66h</v>
       </c>
-    </row>
-    <row r="107" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B107" s="4">
+      <c r="D106" s="40"/>
+      <c r="E106" s="40"/>
+      <c r="F106" s="40"/>
+      <c r="G106" s="40"/>
+    </row>
+    <row r="107" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B107" s="3">
         <v>103</v>
       </c>
-      <c r="C107" s="4" t="str">
+      <c r="C107" s="3" t="str">
         <f t="shared" si="1"/>
         <v>67h</v>
       </c>
-    </row>
-    <row r="108" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B108" s="4">
+      <c r="D107" s="40"/>
+      <c r="E107" s="40"/>
+      <c r="F107" s="40"/>
+      <c r="G107" s="40"/>
+    </row>
+    <row r="108" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B108" s="3">
         <v>104</v>
       </c>
-      <c r="C108" s="4" t="str">
+      <c r="C108" s="3" t="str">
         <f t="shared" si="1"/>
         <v>68h</v>
       </c>
-    </row>
-    <row r="109" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B109" s="4">
+      <c r="D108" s="40"/>
+      <c r="E108" s="40"/>
+      <c r="F108" s="40"/>
+      <c r="G108" s="40"/>
+    </row>
+    <row r="109" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B109" s="3">
         <v>105</v>
       </c>
-      <c r="C109" s="4" t="str">
+      <c r="C109" s="3" t="str">
         <f t="shared" si="1"/>
         <v>69h</v>
       </c>
-    </row>
-    <row r="110" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B110" s="4">
+      <c r="D109" s="40"/>
+      <c r="E109" s="40"/>
+      <c r="F109" s="40"/>
+      <c r="G109" s="40"/>
+    </row>
+    <row r="110" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B110" s="3">
         <v>106</v>
       </c>
-      <c r="C110" s="4" t="str">
+      <c r="C110" s="3" t="str">
         <f t="shared" si="1"/>
         <v>6Ah</v>
       </c>
-    </row>
-    <row r="111" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B111" s="4">
+      <c r="D110" s="40"/>
+      <c r="E110" s="40"/>
+      <c r="F110" s="40"/>
+      <c r="G110" s="40"/>
+    </row>
+    <row r="111" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B111" s="3">
         <v>107</v>
       </c>
-      <c r="C111" s="4" t="str">
+      <c r="C111" s="3" t="str">
         <f t="shared" si="1"/>
         <v>6Bh</v>
       </c>
-    </row>
-    <row r="112" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B112" s="4">
+      <c r="D111" s="40"/>
+      <c r="E111" s="40"/>
+      <c r="F111" s="40"/>
+      <c r="G111" s="40"/>
+    </row>
+    <row r="112" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B112" s="3">
         <v>108</v>
       </c>
-      <c r="C112" s="4" t="str">
+      <c r="C112" s="3" t="str">
         <f t="shared" si="1"/>
         <v>6Ch</v>
       </c>
-    </row>
-    <row r="113" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B113" s="4">
+      <c r="D112" s="40"/>
+      <c r="E112" s="40"/>
+      <c r="F112" s="40"/>
+      <c r="G112" s="40"/>
+    </row>
+    <row r="113" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B113" s="3">
         <v>109</v>
       </c>
-      <c r="C113" s="4" t="str">
+      <c r="C113" s="3" t="str">
         <f t="shared" si="1"/>
         <v>6Dh</v>
       </c>
-    </row>
-    <row r="114" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B114" s="4">
+      <c r="D113" s="40"/>
+      <c r="E113" s="40"/>
+      <c r="F113" s="40"/>
+      <c r="G113" s="40"/>
+    </row>
+    <row r="114" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B114" s="3">
         <v>110</v>
       </c>
-      <c r="C114" s="4" t="str">
+      <c r="C114" s="3" t="str">
         <f t="shared" si="1"/>
         <v>6Eh</v>
       </c>
-    </row>
-    <row r="115" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B115" s="4">
+      <c r="D114" s="40"/>
+      <c r="E114" s="40"/>
+      <c r="F114" s="40"/>
+      <c r="G114" s="40"/>
+    </row>
+    <row r="115" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B115" s="3">
         <v>111</v>
       </c>
-      <c r="C115" s="4" t="str">
+      <c r="C115" s="3" t="str">
         <f t="shared" si="1"/>
         <v>6Fh</v>
       </c>
-    </row>
-    <row r="116" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B116" s="4">
+      <c r="D115" s="40"/>
+      <c r="E115" s="40"/>
+      <c r="F115" s="40"/>
+      <c r="G115" s="40"/>
+    </row>
+    <row r="116" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B116" s="3">
         <v>112</v>
       </c>
-      <c r="C116" s="4" t="str">
+      <c r="C116" s="3" t="str">
         <f t="shared" si="1"/>
         <v>70h</v>
       </c>
-    </row>
-    <row r="117" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B117" s="4">
+      <c r="D116" s="40"/>
+      <c r="E116" s="40"/>
+      <c r="F116" s="40"/>
+      <c r="G116" s="40"/>
+    </row>
+    <row r="117" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B117" s="3">
         <v>113</v>
       </c>
-      <c r="C117" s="4" t="str">
+      <c r="C117" s="3" t="str">
         <f t="shared" si="1"/>
         <v>71h</v>
       </c>
-    </row>
-    <row r="118" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B118" s="4">
+      <c r="D117" s="40"/>
+      <c r="E117" s="40"/>
+      <c r="F117" s="40"/>
+      <c r="G117" s="40"/>
+    </row>
+    <row r="118" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B118" s="3">
         <v>114</v>
       </c>
-      <c r="C118" s="4" t="str">
+      <c r="C118" s="3" t="str">
         <f t="shared" si="1"/>
         <v>72h</v>
       </c>
-    </row>
-    <row r="119" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B119" s="4">
+      <c r="D118" s="40"/>
+      <c r="E118" s="40"/>
+      <c r="F118" s="40"/>
+      <c r="G118" s="40"/>
+    </row>
+    <row r="119" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B119" s="3">
         <v>115</v>
       </c>
-      <c r="C119" s="4" t="str">
+      <c r="C119" s="3" t="str">
         <f t="shared" si="1"/>
         <v>73h</v>
       </c>
-    </row>
-    <row r="120" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B120" s="4">
+      <c r="D119" s="40"/>
+      <c r="E119" s="40"/>
+      <c r="F119" s="40"/>
+      <c r="G119" s="40"/>
+    </row>
+    <row r="120" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B120" s="3">
         <v>116</v>
       </c>
-      <c r="C120" s="4" t="str">
+      <c r="C120" s="3" t="str">
         <f t="shared" si="1"/>
         <v>74h</v>
       </c>
-    </row>
-    <row r="121" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B121" s="4">
+      <c r="D120" s="40"/>
+      <c r="E120" s="40"/>
+      <c r="F120" s="40"/>
+      <c r="G120" s="40"/>
+    </row>
+    <row r="121" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B121" s="3">
         <v>117</v>
       </c>
-      <c r="C121" s="4" t="str">
+      <c r="C121" s="3" t="str">
         <f t="shared" si="1"/>
         <v>75h</v>
       </c>
-    </row>
-    <row r="122" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B122" s="4">
+      <c r="D121" s="40"/>
+      <c r="E121" s="40"/>
+      <c r="F121" s="40"/>
+      <c r="G121" s="40"/>
+    </row>
+    <row r="122" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B122" s="3">
         <v>118</v>
       </c>
-      <c r="C122" s="4" t="str">
+      <c r="C122" s="3" t="str">
         <f t="shared" si="1"/>
         <v>76h</v>
       </c>
-    </row>
-    <row r="123" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B123" s="4">
+      <c r="D122" s="40"/>
+      <c r="E122" s="40"/>
+      <c r="F122" s="40"/>
+      <c r="G122" s="40"/>
+    </row>
+    <row r="123" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B123" s="3">
         <v>119</v>
       </c>
-      <c r="C123" s="4" t="str">
+      <c r="C123" s="3" t="str">
         <f t="shared" si="1"/>
         <v>77h</v>
       </c>
-    </row>
-    <row r="124" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B124" s="4">
+      <c r="D123" s="40"/>
+      <c r="E123" s="40"/>
+      <c r="F123" s="40"/>
+      <c r="G123" s="40"/>
+    </row>
+    <row r="124" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B124" s="3">
         <v>120</v>
       </c>
-      <c r="C124" s="4" t="str">
+      <c r="C124" s="3" t="str">
         <f t="shared" si="1"/>
         <v>78h</v>
       </c>
-    </row>
-    <row r="125" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B125" s="4">
+      <c r="D124" s="40"/>
+      <c r="E124" s="40"/>
+      <c r="F124" s="40"/>
+      <c r="G124" s="40"/>
+    </row>
+    <row r="125" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B125" s="3">
         <v>121</v>
       </c>
-      <c r="C125" s="4" t="str">
+      <c r="C125" s="3" t="str">
         <f t="shared" si="1"/>
         <v>79h</v>
       </c>
-    </row>
-    <row r="126" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B126" s="4">
+      <c r="D125" s="40"/>
+      <c r="E125" s="40"/>
+      <c r="F125" s="40"/>
+      <c r="G125" s="40"/>
+    </row>
+    <row r="126" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B126" s="3">
         <v>122</v>
       </c>
-      <c r="C126" s="4" t="str">
+      <c r="C126" s="3" t="str">
         <f t="shared" si="1"/>
         <v>7Ah</v>
       </c>
-    </row>
-    <row r="127" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B127" s="4">
+      <c r="D126" s="40"/>
+      <c r="E126" s="40"/>
+      <c r="F126" s="40"/>
+      <c r="G126" s="40"/>
+    </row>
+    <row r="127" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B127" s="3">
         <v>123</v>
       </c>
-      <c r="C127" s="4" t="str">
+      <c r="C127" s="3" t="str">
         <f t="shared" si="1"/>
         <v>7Bh</v>
       </c>
-    </row>
-    <row r="128" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B128" s="4">
+      <c r="D127" s="40"/>
+      <c r="E127" s="40"/>
+      <c r="F127" s="40"/>
+      <c r="G127" s="40"/>
+    </row>
+    <row r="128" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B128" s="3">
         <v>124</v>
       </c>
-      <c r="C128" s="4" t="str">
+      <c r="C128" s="3" t="str">
         <f t="shared" si="1"/>
         <v>7Ch</v>
       </c>
-    </row>
-    <row r="129" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B129" s="4">
+      <c r="D128" s="40"/>
+      <c r="E128" s="40"/>
+      <c r="F128" s="40"/>
+      <c r="G128" s="40"/>
+    </row>
+    <row r="129" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B129" s="3">
         <v>125</v>
       </c>
-      <c r="C129" s="4" t="str">
+      <c r="C129" s="3" t="str">
         <f t="shared" si="1"/>
         <v>7Dh</v>
       </c>
-    </row>
-    <row r="130" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B130" s="4">
+      <c r="D129" s="40"/>
+      <c r="E129" s="40"/>
+      <c r="F129" s="40"/>
+      <c r="G129" s="40"/>
+    </row>
+    <row r="130" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B130" s="3">
         <v>126</v>
       </c>
-      <c r="C130" s="4" t="str">
+      <c r="C130" s="3" t="str">
         <f t="shared" si="1"/>
         <v>7Eh</v>
       </c>
-    </row>
-    <row r="131" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B131" s="4">
+      <c r="D130" s="40"/>
+      <c r="E130" s="40"/>
+      <c r="F130" s="40"/>
+      <c r="G130" s="40"/>
+    </row>
+    <row r="131" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B131" s="3">
         <v>127</v>
       </c>
-      <c r="C131" s="4" t="str">
+      <c r="C131" s="3" t="str">
         <f t="shared" si="1"/>
         <v>7Fh</v>
       </c>
-    </row>
-    <row r="132" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B132" s="4">
+      <c r="D131" s="40"/>
+      <c r="E131" s="40"/>
+      <c r="F131" s="40"/>
+      <c r="G131" s="40"/>
+    </row>
+    <row r="132" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B132" s="3">
         <v>128</v>
       </c>
-      <c r="C132" s="4" t="str">
+      <c r="C132" s="3" t="str">
         <f t="shared" si="1"/>
         <v>80h</v>
       </c>
-    </row>
-    <row r="133" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B133" s="4">
+      <c r="D132" s="40"/>
+      <c r="E132" s="40"/>
+      <c r="F132" s="40"/>
+      <c r="G132" s="40"/>
+    </row>
+    <row r="133" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B133" s="3">
         <v>129</v>
       </c>
-      <c r="C133" s="4" t="str">
+      <c r="C133" s="3" t="str">
         <f t="shared" ref="C133:C138" si="2">DEC2HEX(B133)&amp;"h"</f>
         <v>81h</v>
       </c>
-    </row>
-    <row r="134" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B134" s="4">
+      <c r="D133" s="40"/>
+      <c r="E133" s="40"/>
+      <c r="F133" s="40"/>
+      <c r="G133" s="40"/>
+    </row>
+    <row r="134" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B134" s="3">
         <v>130</v>
       </c>
-      <c r="C134" s="4" t="str">
+      <c r="C134" s="3" t="str">
         <f t="shared" si="2"/>
         <v>82h</v>
       </c>
-    </row>
-    <row r="135" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B135" s="4">
+      <c r="D134" s="40"/>
+      <c r="E134" s="40"/>
+      <c r="F134" s="40"/>
+      <c r="G134" s="40"/>
+    </row>
+    <row r="135" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B135" s="3">
         <v>131</v>
       </c>
-      <c r="C135" s="4" t="str">
+      <c r="C135" s="3" t="str">
         <f t="shared" si="2"/>
         <v>83h</v>
       </c>
-    </row>
-    <row r="136" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B136" s="4">
+      <c r="D135" s="40"/>
+      <c r="E135" s="40"/>
+      <c r="F135" s="40"/>
+      <c r="G135" s="40"/>
+    </row>
+    <row r="136" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B136" s="3">
         <v>132</v>
       </c>
-      <c r="C136" s="4" t="str">
+      <c r="C136" s="3" t="str">
         <f t="shared" si="2"/>
         <v>84h</v>
       </c>
-    </row>
-    <row r="137" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B137" s="4">
+      <c r="D136" s="40"/>
+      <c r="E136" s="40"/>
+      <c r="F136" s="40"/>
+      <c r="G136" s="40"/>
+    </row>
+    <row r="137" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B137" s="3">
         <v>133</v>
       </c>
-      <c r="C137" s="4" t="str">
+      <c r="C137" s="3" t="str">
         <f t="shared" si="2"/>
         <v>85h</v>
       </c>
-    </row>
-    <row r="138" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B138" s="4">
+      <c r="D137" s="50"/>
+      <c r="E137" s="50"/>
+      <c r="F137" s="50"/>
+      <c r="G137" s="50"/>
+    </row>
+    <row r="138" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B138" s="3">
         <v>134</v>
       </c>
-      <c r="C138" s="4" t="str">
+      <c r="C138" s="3" t="str">
         <f t="shared" si="2"/>
         <v>86h</v>
       </c>
+      <c r="D138" s="51"/>
+      <c r="E138" s="51"/>
+      <c r="F138" s="51"/>
+      <c r="G138" s="51"/>
+    </row>
+    <row r="139" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D139" s="49"/>
+      <c r="E139" s="49"/>
+      <c r="F139" s="49"/>
+      <c r="G139" s="49"/>
+    </row>
+    <row r="140" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D140" s="49"/>
+      <c r="E140" s="49"/>
+      <c r="F140" s="49"/>
+      <c r="G140" s="49"/>
+    </row>
+    <row r="141" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D141" s="49"/>
+      <c r="E141" s="49"/>
+      <c r="F141" s="49"/>
+      <c r="G141" s="49"/>
+    </row>
+    <row r="142" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D142" s="49"/>
+      <c r="E142" s="49"/>
+      <c r="F142" s="49"/>
+      <c r="G142" s="49"/>
+    </row>
+    <row r="143" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D143" s="49"/>
+      <c r="E143" s="49"/>
+      <c r="F143" s="49"/>
+      <c r="G143" s="49"/>
+    </row>
+    <row r="144" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="D144" s="49"/>
+      <c r="E144" s="49"/>
+      <c r="F144" s="49"/>
+      <c r="G144" s="49"/>
+    </row>
+    <row r="145" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D145" s="49"/>
+      <c r="E145" s="49"/>
+      <c r="F145" s="49"/>
+      <c r="G145" s="49"/>
+    </row>
+    <row r="146" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D146" s="49"/>
+      <c r="E146" s="49"/>
+      <c r="F146" s="49"/>
+      <c r="G146" s="49"/>
+    </row>
+    <row r="147" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D147" s="49"/>
+      <c r="E147" s="49"/>
+      <c r="F147" s="49"/>
+      <c r="G147" s="49"/>
+    </row>
+    <row r="148" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D148" s="49"/>
+      <c r="E148" s="49"/>
+      <c r="F148" s="49"/>
+      <c r="G148" s="49"/>
+    </row>
+    <row r="149" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D149" s="49"/>
+      <c r="E149" s="49"/>
+      <c r="F149" s="49"/>
+      <c r="G149" s="49"/>
+    </row>
+    <row r="150" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D150" s="49"/>
+      <c r="E150" s="49"/>
+      <c r="F150" s="49"/>
+      <c r="G150" s="49"/>
+    </row>
+    <row r="151" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D151" s="49"/>
+      <c r="E151" s="49"/>
+      <c r="F151" s="49"/>
+      <c r="G151" s="49"/>
+    </row>
+    <row r="152" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D152" s="49"/>
+      <c r="E152" s="49"/>
+      <c r="F152" s="49"/>
+      <c r="G152" s="49"/>
+    </row>
+    <row r="153" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D153" s="49"/>
+      <c r="E153" s="49"/>
+      <c r="F153" s="49"/>
+      <c r="G153" s="49"/>
+    </row>
+    <row r="154" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D154" s="49"/>
+      <c r="E154" s="49"/>
+      <c r="F154" s="49"/>
+      <c r="G154" s="49"/>
+    </row>
+    <row r="155" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D155" s="49"/>
+      <c r="E155" s="49"/>
+      <c r="F155" s="49"/>
+      <c r="G155" s="49"/>
+    </row>
+    <row r="156" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D156" s="49"/>
+      <c r="E156" s="49"/>
+      <c r="F156" s="49"/>
+      <c r="G156" s="49"/>
+    </row>
+    <row r="157" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D157" s="49"/>
+      <c r="E157" s="49"/>
+      <c r="F157" s="49"/>
+      <c r="G157" s="49"/>
+    </row>
+    <row r="158" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D158" s="49"/>
+      <c r="E158" s="49"/>
+      <c r="F158" s="49"/>
+      <c r="G158" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -3004,20 +3421,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="602d6013-12bf-42a7-bc7f-2fade0e82371" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="602d6013-12bf-42a7-bc7f-2fade0e82371" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3040,6 +3457,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E732BC0F-1505-48BB-B355-5D5ECDA47127}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -3054,12 +3479,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3CCCF266-1755-4F5F-AFB7-075C74CE2D71}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>